<commit_message>
Mark list-type posts with ⚠️ FOLLOW-UP CLICK LINK marker (Nitter blocks crawler · manual click needed)
</commit_message>
<xml_diff>
--- a/Transfer_Tracker.xlsx
+++ b/Transfer_Tracker.xlsx
@@ -490,7 +490,7 @@
       <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-11 02:14</t>
+          <t>2026-06-11 02:31</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -520,7 +520,7 @@
       <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-06-11 02:14</t>
+          <t>2026-06-11 02:31</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -550,7 +550,7 @@
       <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-06-11 02:14</t>
+          <t>2026-06-11 02:31</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -579,7 +579,7 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-06-11 02:14</t>
+          <t>2026-06-11 02:31</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -608,7 +608,7 @@
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-06-11 02:14</t>
+          <t>2026-06-11 02:31</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -638,7 +638,7 @@
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-06-11 02:14</t>
+          <t>2026-06-11 02:31</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -667,7 +667,7 @@
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-06-11 02:14</t>
+          <t>2026-06-11 02:31</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -695,7 +695,7 @@
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-06-11 02:14</t>
+          <t>2026-06-11 02:31</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -723,7 +723,7 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-06-11 02:14</t>
+          <t>2026-06-11 02:31</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -751,7 +751,7 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-06-11 02:14</t>
+          <t>2026-06-11 02:31</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -781,7 +781,7 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-06-11 02:14</t>
+          <t>2026-06-11 02:31</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -809,7 +809,7 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-06-11 02:14</t>
+          <t>2026-06-11 02:31</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -824,7 +824,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>confirmed, release, released</t>
+          <t>⚠️ FOLLOW-UP CLICK LINK, confirmed, release, released</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -837,7 +837,7 @@
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-06-11 02:14</t>
+          <t>2026-06-11 02:31</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -852,7 +852,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>confirmed, release, released</t>
+          <t>⚠️ FOLLOW-UP CLICK LINK, confirmed, release, released</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -865,7 +865,7 @@
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-06-11 02:14</t>
+          <t>2026-06-11 02:31</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -893,7 +893,7 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-06-11 02:14</t>
+          <t>2026-06-11 02:31</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -908,7 +908,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>confirmed, release, released</t>
+          <t>⚠️ FOLLOW-UP CLICK LINK, confirmed, release, released</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -975,7 +975,7 @@
       <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-11 02:14</t>
+          <t>2026-06-11 02:31</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1029,7 +1029,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Created: 2026-06-10 22:14</t>
+          <t>Created: 2026-06-10 22:31</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add maisfutebol cronologia direct HTML scrape (h2>a entries) · captures OFICIAL Portuguese transfers
</commit_message>
<xml_diff>
--- a/Transfer_Tracker.xlsx
+++ b/Transfer_Tracker.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -490,29 +490,27 @@
       <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-11 02:31</t>
+          <t>2026-06-11 02:41</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>X:@FabrizioRomano</t>
+          <t>X:@David_Ornstein</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>🚨🐺 EXCL: Wolves agree deal in principle to appoint Cesar Peixoto as new head coach.
-Interest reported by O Jogo, now verbal agremeent in place with Peixoto to take over at #WWFC.
-Excellent job at Gil Vicente with record results and seen among top talented young managers.</t>
+          <t>🚨 Jose Mourinho has signed contract to become Real Madrid head coach. 63yo leaving Benfica for 2nd spell in charge of #RMFC after putting pen to paper last week on 3yr deal. Set to be announced post presidential election. W/ @MarioCortegana @TheAthleticFC https://www.nytimes.com/athletic/7284488/202</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>deal, new head coach</t>
+          <t>deal, signed, leaving</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://nitter.net/FabrizioRomano/status/2064838763570733105#m</t>
+          <t>https://nitter.net/David_Ornstein/status/2060361927084167282#m</t>
         </is>
       </c>
     </row>
@@ -520,29 +518,27 @@
       <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-06-11 02:31</t>
+          <t>2026-06-11 02:41</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>X:@FabrizioRomano</t>
+          <t>X:@premierleague</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>🚨🟣🔵 Excl: Zion Suzuki among 3 GKs in list at Aston Villa for summer window if Emiliano Martínez ends up leaving.
-Aston Villa aware of Juve being in talks with the Argentine GK but nothing agreed club to club yet.
-Suzuki been scouted for months at Parma.</t>
+          <t>Premier League clubs have confirmed which players are set to be released once their contract expires on June 30 ⬇️</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>agreed, leaving, talks, talks with</t>
+          <t>confirmed, release, released, contract expires</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://nitter.net/FabrizioRomano/status/2064768287464894700#m</t>
+          <t>https://nitter.net/premierleague/status/2064664119354015875#m</t>
         </is>
       </c>
     </row>
@@ -550,28 +546,27 @@
       <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-06-11 02:31</t>
+          <t>2026-06-11 02:41</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>X:@FabrizioRomano</t>
+          <t>X:@ManCity</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>🚨👋🏼 OFFICIAL: Kieran McKenna takes a break from football and leaves his job at Ipswich Town.
-After promotion to Premier League, McKenna leaves #ITFC job. 🚜</t>
+          <t>We are delighted to announce that Divine Mukasa has signed a new long-term deal with the Club 🩵</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>OFFICIAL:, leaves</t>
+          <t>we are delighted to announce, are delighted to announce, deal, signed</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://nitter.net/FabrizioRomano/status/2064756037807190093#m</t>
+          <t>https://nitter.net/ManCity/status/2064347029867057428#m</t>
         </is>
       </c>
     </row>
@@ -579,28 +574,29 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-06-11 02:31</t>
+          <t>2026-06-11 02:41</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>X:@FabrizioRomano</t>
+          <t>X:@SpursOfficial</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>🚨 OFFICIAL: Marcos Senesi, confirmed as new Tottenham signing and set to wear shirt number 5.
-Deal confirmed. 🇦🇷</t>
+          <t>We are delighted to announce that Ben Davies has signed a new contract with the club ✍️
+Congratulations, Ben! 🙌
+🔗 https://thfc.pro/4urnFuA</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>OFFICIAL:, confirmed, deal, 🚨 OFFICIAL</t>
+          <t>we are delighted to announce, are delighted to announce, signed</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://nitter.net/FabrizioRomano/status/2064742959061328030#m</t>
+          <t>https://nitter.net/SpursOfficial/status/2064619165260923166#m</t>
         </is>
       </c>
     </row>
@@ -608,29 +604,27 @@
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-06-11 02:31</t>
+          <t>2026-06-11 02:41</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>X:@FabrizioRomano</t>
+          <t>X:@ChelseaFC</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">🚨 Kennet Eichorn has just completed his medical as new Bayer Leverkusen player. Deal done for one of the best talents in Germany.
-Several English and German clubs keen but Eichorn picks Leverkusen project. €9m release clause has been activated.
-Contract until June 2031, as @Plettigoal @SkySportDE </t>
+          <t>World Cup winners Chelsea have signed! 🏆</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>deal, release</t>
+          <t>have signed, signed</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://nitter.net/FabrizioRomano/status/2064694320427380771#m</t>
+          <t>https://nitter.net/ChelseaFC/status/2064760557182296531#m</t>
         </is>
       </c>
     </row>
@@ -638,28 +632,27 @@
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-06-11 02:31</t>
+          <t>2026-06-11 02:41</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>X:@FabrizioRomano</t>
+          <t>X:@ChelseaFC</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>🚨🔵 José Bordalás signs new two-year deal at Getafe valid until June 2028. 🫱🏻‍🫲🏼
-After long discussions, the coach decides to stay.</t>
+          <t>The list of Chelsea players who have been retained or released by the club at the end of the 25/26 season have been confirmed.</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>deal, signs, discussions</t>
+          <t>⚠️ FOLLOW-UP CLICK LINK, confirmed, release, released</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://nitter.net/FabrizioRomano/status/2064691681740378468#m</t>
+          <t>https://nitter.net/ChelseaFC/status/2064633680702627993#m</t>
         </is>
       </c>
     </row>
@@ -667,27 +660,27 @@
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-06-11 02:31</t>
+          <t>2026-06-11 02:41</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>X:@David_Ornstein</t>
+          <t>X:@CPFC</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>🚨 Jose Mourinho has signed contract to become Real Madrid head coach. 63yo leaving Benfica for 2nd spell in charge of #RMFC after putting pen to paper last week on 3yr deal. Set to be announced post presidential election. W/ @MarioCortegana @TheAthleticFC https://www.nytimes.com/athletic/7284488/202</t>
+          <t>The list of Crystal Palace players who have been retained or released by the club at the end of the 25/26 season has been confirmed.</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>deal, signed, leaving</t>
+          <t>⚠️ FOLLOW-UP CLICK LINK, confirmed, release, released</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://nitter.net/David_Ornstein/status/2060361927084167282#m</t>
+          <t>https://nitter.net/CPFC/status/2064681986711593211#m</t>
         </is>
       </c>
     </row>
@@ -695,27 +688,27 @@
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-06-11 02:31</t>
+          <t>2026-06-11 02:41</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>X:@premierleague</t>
+          <t>X:@Coventry_City</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Premier League clubs have confirmed which players are set to be released once their contract expires on June 30 ⬇️</t>
+          <t>We are delighted to announce that Victor Torp has signed a new contract with the Club. 🩵</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>confirmed, release, released, contract expires</t>
+          <t>we are delighted to announce, are delighted to announce, signed</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://nitter.net/premierleague/status/2064664119354015875#m</t>
+          <t>https://nitter.net/Coventry_City/status/2060328196826878386#m</t>
         </is>
       </c>
     </row>
@@ -723,27 +716,27 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-06-11 02:31</t>
+          <t>2026-06-11 02:41</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>X:@ManCity</t>
+          <t>X:@BurnleyOfficial</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>We are delighted to announce that Divine Mukasa has signed a new long-term deal with the Club 🩵</t>
+          <t>Our retained and released list has been confirmed following the conclusion of the 2025/26 campaign 📋</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>we are delighted to announce, are delighted to announce, deal, signed</t>
+          <t>⚠️ FOLLOW-UP CLICK LINK, confirmed, release, released</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://nitter.net/ManCity/status/2064347029867057428#m</t>
+          <t>https://nitter.net/BurnleyOfficial/status/2064665490576884001#m</t>
         </is>
       </c>
     </row>
@@ -751,29 +744,27 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-06-11 02:31</t>
+          <t>2026-06-11 02:41</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>X:@SpursOfficial</t>
+          <t>maisfutebol cronologia</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>We are delighted to announce that Ben Davies has signed a new contract with the club ✍️
-Congratulations, Ben! 🙌
-🔗 https://thfc.pro/4urnFuA</t>
+          <t>OFICIAL: Mauro Jerónimo é o novo treinador do Borneo Samarinda</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>we are delighted to announce, are delighted to announce, signed</t>
+          <t>OFICIAL, novo treinador</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://nitter.net/SpursOfficial/status/2064619165260923166#m</t>
+          <t>https://maisfutebol.iol.pt/oficial/indonesia/oficial-mauro-jeronimo-e-o-novo-treinador-do-borneo-samarinda</t>
         </is>
       </c>
     </row>
@@ -781,27 +772,27 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-06-11 02:31</t>
+          <t>2026-06-11 02:41</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>X:@ChelseaFC</t>
+          <t>maisfutebol cronologia</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>World Cup winners Chelsea have signed! 🏆</t>
+          <t>Ipswich anuncia saída do treinador que subiu a equipa duas vezes à Premier League</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>have signed, signed</t>
+          <t>anuncia, saída</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://nitter.net/ChelseaFC/status/2064760557182296531#m</t>
+          <t>https://maisfutebol.iol.pt/transferencias/mercado/ipswich-anuncia-saida-do-treinador-que-subiu-a-equipa-duas-vezes-a-premier-league</t>
         </is>
       </c>
     </row>
@@ -809,27 +800,27 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-06-11 02:31</t>
+          <t>2026-06-11 02:41</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>X:@ChelseaFC</t>
+          <t>maisfutebol cronologia</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>The list of Chelsea players who have been retained or released by the club at the end of the 25/26 season have been confirmed.</t>
+          <t>OFICIAL: Adama Traoré e Fabianski deixam o West Ham</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>⚠️ FOLLOW-UP CLICK LINK, confirmed, release, released</t>
+          <t>OFICIAL, deixa</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://nitter.net/ChelseaFC/status/2064633680702627993#m</t>
+          <t>https://maisfutebol.iol.pt/transferencias/adama-traore/oficial-adama-traore-e-fabianski-deixam-o-west-ham</t>
         </is>
       </c>
     </row>
@@ -837,27 +828,27 @@
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-06-11 02:31</t>
+          <t>2026-06-11 02:41</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>X:@CPFC</t>
+          <t>maisfutebol cronologia</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>The list of Crystal Palace players who have been retained or released by the club at the end of the 25/26 season has been confirmed.</t>
+          <t>OFICIAL: irmão de Michael Olise deixa o Chelsea</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>⚠️ FOLLOW-UP CLICK LINK, confirmed, release, released</t>
+          <t>OFICIAL, deixa</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://nitter.net/CPFC/status/2064681986711593211#m</t>
+          <t>https://maisfutebol.iol.pt/transferencias/richard-olise/oficial-irmao-de-michael-olise-deixa-o-chelsea</t>
         </is>
       </c>
     </row>
@@ -865,55 +856,27 @@
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-06-11 02:31</t>
+          <t>2026-06-11 02:41</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>X:@Coventry_City</t>
+          <t>maisfutebol cronologia</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>We are delighted to announce that Victor Torp has signed a new contract with the Club. 🩵</t>
+          <t>OFICIAL: Manchester United confirma saídas de Sancho e Malacia</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>we are delighted to announce, are delighted to announce, signed</t>
+          <t>OFICIAL, confirma, saída</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://nitter.net/Coventry_City/status/2060328196826878386#m</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr"/>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>2026-06-11 02:31</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>X:@BurnleyOfficial</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>Our retained and released list has been confirmed following the conclusion of the 2025/26 campaign 📋</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>⚠️ FOLLOW-UP CLICK LINK, confirmed, release, released</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>https://nitter.net/BurnleyOfficial/status/2064665490576884001#m</t>
+          <t>https://maisfutebol.iol.pt/transferencias/manchester-united/oficial-manchester-united-confirma-saidas-de-sancho-e-malacia</t>
         </is>
       </c>
     </row>
@@ -975,7 +938,7 @@
       <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-11 02:31</t>
+          <t>2026-06-11 02:41</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1029,7 +992,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Created: 2026-06-10 22:31</t>
+          <t>Created: 2026-06-10 22:41</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dedup uses link+title-hash · title edits re-emit · cleaner duplicate handling
</commit_message>
<xml_diff>
--- a/Transfer_Tracker.xlsx
+++ b/Transfer_Tracker.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -490,27 +490,28 @@
       <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-11 02:41</t>
+          <t>2026-06-11 12:12</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>X:@David_Ornstein</t>
+          <t>X:@FabrizioRomano</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>🚨 Jose Mourinho has signed contract to become Real Madrid head coach. 63yo leaving Benfica for 2nd spell in charge of #RMFC after putting pen to paper last week on 3yr deal. Set to be announced post presidential election. W/ @MarioCortegana @TheAthleticFC https://www.nytimes.com/athletic/7284488/202</t>
+          <t>🚨🇩🇪 Excl: Bayern talent Maurice Krattenmacher to SV Elversberg, deal done and medical today. 
+The 20-year-old fulfil his dream of playing in the Bundesliga after a season on loan at Hertha BSC, now moving to Elversberg where he will have a central role.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>deal, signed, leaving</t>
+          <t>deal, loan</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://nitter.net/David_Ornstein/status/2060361927084167282#m</t>
+          <t>https://nitter.net/FabrizioRomano/status/2065012506381205642#m</t>
         </is>
       </c>
     </row>
@@ -518,27 +519,27 @@
       <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-06-11 02:41</t>
+          <t>2026-06-11 12:12</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>X:@premierleague</t>
+          <t>X:@FabrizioRomano</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Premier League clubs have confirmed which players are set to be released once their contract expires on June 30 ⬇️</t>
+          <t>⤵️🟠⚫️✅ #WWFC</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>confirmed, release, released, contract expires</t>
+          <t>deal, new head coach</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://nitter.net/premierleague/status/2064664119354015875#m</t>
+          <t>https://nitter.net/FabrizioRomano/status/2065003796149711073#m</t>
         </is>
       </c>
     </row>
@@ -546,27 +547,29 @@
       <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-06-11 02:41</t>
+          <t>2026-06-11 12:12</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>X:@ManCity</t>
+          <t>X:@FabrizioRomano</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>We are delighted to announce that Divine Mukasa has signed a new long-term deal with the Club 🩵</t>
+          <t>RT by @FabrizioRomano: 🚨🐺 EXCL: Wolves agree deal in principle to appoint Cesar Peixoto as new head coach.
+Interest reported by O Jogo, now verbal agremeent in place with Peixoto to take over at #WWFC.
+Excellent job at Gil Vicente with record results and seen among top talented young managers.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>we are delighted to announce, are delighted to announce, deal, signed</t>
+          <t>deal, new head coach</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://nitter.net/ManCity/status/2064347029867057428#m</t>
+          <t>https://nitter.net/FabrizioRomano/status/2064838763570733105#m</t>
         </is>
       </c>
     </row>
@@ -574,141 +577,143 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-06-11 02:41</t>
+          <t>2026-06-11 12:12</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>🚨🟣🔵 Excl: Zion Suzuki among 3 GKs in list at Aston Villa for summer window if Emiliano Martínez ends up leaving.
+Aston Villa aware of Juve being in talks with the Argentine GK but nothing agreed club to club yet.
+Suzuki been scouted for months at Parma.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>agreed, leaving, talks, talks with</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2064768287464894700#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-06-11 12:12</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>X:@David_Ornstein</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>🚨 Jose Mourinho has signed contract to become Real Madrid head coach. 63yo leaving Benfica for 2nd spell in charge of #RMFC after putting pen to paper last week on 3yr deal. Set to be announced post presidential election. W/ @MarioCortegana @TheAthleticFC https://www.nytimes.com/athletic/7284488/202</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>deal, signed, leaving</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>https://nitter.net/David_Ornstein/status/2060361927084167282#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-06-11 12:12</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>X:@premierleague</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Premier League clubs have confirmed which players are set to be released once their contract expires on June 30 ⬇️</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>confirmed, release, released, contract expires</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>https://nitter.net/premierleague/status/2064664119354015875#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-06-11 12:12</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>X:@ManCity</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>We are delighted to announce that Divine Mukasa has signed a new long-term deal with the Club 🩵</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>we are delighted to announce, are delighted to announce, deal, signed</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>https://nitter.net/ManCity/status/2064347029867057428#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-06-11 12:12</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
           <t>X:@SpursOfficial</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>We are delighted to announce that Ben Davies has signed a new contract with the club ✍️
 Congratulations, Ben! 🙌
 🔗 https://thfc.pro/4urnFuA</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>we are delighted to announce, are delighted to announce, signed</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>https://nitter.net/SpursOfficial/status/2064619165260923166#m</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr"/>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2026-06-11 02:41</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>X:@ChelseaFC</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>World Cup winners Chelsea have signed! 🏆</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>have signed, signed</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>https://nitter.net/ChelseaFC/status/2064760557182296531#m</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>2026-06-11 02:41</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>X:@ChelseaFC</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>The list of Chelsea players who have been retained or released by the club at the end of the 25/26 season have been confirmed.</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>⚠️ FOLLOW-UP CLICK LINK, confirmed, release, released</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>https://nitter.net/ChelseaFC/status/2064633680702627993#m</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr"/>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>2026-06-11 02:41</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>X:@CPFC</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>The list of Crystal Palace players who have been retained or released by the club at the end of the 25/26 season has been confirmed.</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>⚠️ FOLLOW-UP CLICK LINK, confirmed, release, released</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>https://nitter.net/CPFC/status/2064681986711593211#m</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>2026-06-11 02:41</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>X:@Coventry_City</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>We are delighted to announce that Victor Torp has signed a new contract with the Club. 🩵</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>we are delighted to announce, are delighted to announce, signed</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>https://nitter.net/Coventry_City/status/2060328196826878386#m</t>
         </is>
       </c>
     </row>
@@ -716,27 +721,27 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-06-11 02:41</t>
+          <t>2026-06-11 12:12</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>X:@BurnleyOfficial</t>
+          <t>X:@ChelseaFC</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Our retained and released list has been confirmed following the conclusion of the 2025/26 campaign 📋</t>
+          <t>World Cup winners Chelsea have signed! 🏆</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>⚠️ FOLLOW-UP CLICK LINK, confirmed, release, released</t>
+          <t>have signed, signed</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://nitter.net/BurnleyOfficial/status/2064665490576884001#m</t>
+          <t>https://nitter.net/ChelseaFC/status/2064760557182296531#m</t>
         </is>
       </c>
     </row>
@@ -744,27 +749,27 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-06-11 02:41</t>
+          <t>2026-06-11 12:12</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>maisfutebol cronologia</t>
+          <t>X:@ChelseaFC</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>OFICIAL: Mauro Jerónimo é o novo treinador do Borneo Samarinda</t>
+          <t>The list of Chelsea players who have been retained or released by the club at the end of the 25/26 season have been confirmed.</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>OFICIAL, novo treinador</t>
+          <t>⚠️ FOLLOW-UP CLICK LINK, confirmed, release, released</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://maisfutebol.iol.pt/oficial/indonesia/oficial-mauro-jeronimo-e-o-novo-treinador-do-borneo-samarinda</t>
+          <t>https://nitter.net/ChelseaFC/status/2064633680702627993#m</t>
         </is>
       </c>
     </row>
@@ -772,27 +777,27 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-06-11 02:41</t>
+          <t>2026-06-11 12:12</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>maisfutebol cronologia</t>
+          <t>X:@CPFC</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Ipswich anuncia saída do treinador que subiu a equipa duas vezes à Premier League</t>
+          <t>The list of Crystal Palace players who have been retained or released by the club at the end of the 25/26 season has been confirmed.</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>anuncia, saída</t>
+          <t>⚠️ FOLLOW-UP CLICK LINK, confirmed, release, released</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://maisfutebol.iol.pt/transferencias/mercado/ipswich-anuncia-saida-do-treinador-que-subiu-a-equipa-duas-vezes-a-premier-league</t>
+          <t>https://nitter.net/CPFC/status/2064681986711593211#m</t>
         </is>
       </c>
     </row>
@@ -800,27 +805,27 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-06-11 02:41</t>
+          <t>2026-06-11 12:12</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>maisfutebol cronologia</t>
+          <t>X:@Coventry_City</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>OFICIAL: Adama Traoré e Fabianski deixam o West Ham</t>
+          <t>We are delighted to announce that Victor Torp has signed a new contract with the Club. 🩵</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>OFICIAL, deixa</t>
+          <t>we are delighted to announce, are delighted to announce, signed</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://maisfutebol.iol.pt/transferencias/adama-traore/oficial-adama-traore-e-fabianski-deixam-o-west-ham</t>
+          <t>https://nitter.net/Coventry_City/status/2060328196826878386#m</t>
         </is>
       </c>
     </row>
@@ -828,27 +833,27 @@
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-06-11 02:41</t>
+          <t>2026-06-11 12:12</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>maisfutebol cronologia</t>
+          <t>X:@BurnleyOfficial</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>OFICIAL: irmão de Michael Olise deixa o Chelsea</t>
+          <t>Our retained and released list has been confirmed following the conclusion of the 2025/26 campaign 📋</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>OFICIAL, deixa</t>
+          <t>⚠️ FOLLOW-UP CLICK LINK, confirmed, release, released</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://maisfutebol.iol.pt/transferencias/richard-olise/oficial-irmao-de-michael-olise-deixa-o-chelsea</t>
+          <t>https://nitter.net/BurnleyOfficial/status/2064665490576884001#m</t>
         </is>
       </c>
     </row>
@@ -856,27 +861,167 @@
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-06-11 02:41</t>
+          <t>2026-06-11 12:12</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Rob Edwards despedido do comando técnico do Wolverhampton</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, deixa</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/transferencias/inglaterra/oficial-rob-edwards-despedido-do-comando-tecnico-do-wolverhampton</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr"/>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-06-11 12:12</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Sampaoli substitui Carlos Tévez como novo treinador do Talleres</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, novo treinador</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/transferencias/jorge-sampaoli/oficial-sampaoli-substitui-carlos-tevez-como-novo-treinador-do-talleres</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-06-11 12:12</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
           <t>maisfutebol cronologia</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>OFICIAL: Manchester United confirma saídas de Sancho e Malacia</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>OFICIAL, confirma, saída</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>https://maisfutebol.iol.pt/transferencias/manchester-united/oficial-manchester-united-confirma-saidas-de-sancho-e-malacia</t>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Sampaoli substitui Carlos Tévez como novo treinador do Talleres</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, novo treinador</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/transferencias/jorge-sampaoli/oficial-sampaoli-substitui-carlos-tevez-como-novo-treinador-do-talleres</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-06-11 12:12</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Mauro Jerónimo é o novo treinador do Borneo Samarinda</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, novo treinador</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/oficial/indonesia/oficial-mauro-jeronimo-e-o-novo-treinador-do-borneo-samarinda</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-06-11 12:12</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Ipswich anuncia saída do treinador que subiu a equipa duas vezes à Premier League</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>anuncia, saída</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/transferencias/mercado/ipswich-anuncia-saida-do-treinador-que-subiu-a-equipa-duas-vezes-a-premier-league</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-06-11 12:12</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Adama Traoré e Fabianski deixam o West Ham</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, deixa</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/transferencias/adama-traore/oficial-adama-traore-e-fabianski-deixam-o-west-ham</t>
         </is>
       </c>
     </row>
@@ -938,7 +1083,7 @@
       <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-11 02:41</t>
+          <t>2026-06-11 12:12</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -992,7 +1137,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Created: 2026-06-10 22:41</t>
+          <t>Created: 2026-06-11 08:12</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cronologia · scrape h2 without inner <a> + add Portuguese rumor keywords (interessado em, procura, alvo, etc)
</commit_message>
<xml_diff>
--- a/Transfer_Tracker.xlsx
+++ b/Transfer_Tracker.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -490,7 +490,7 @@
       <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-11 12:12</t>
+          <t>2026-06-11 17:34</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -519,7 +519,7 @@
       <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-06-11 12:12</t>
+          <t>2026-06-11 17:34</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -547,7 +547,7 @@
       <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-06-11 12:12</t>
+          <t>2026-06-11 17:34</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -577,29 +577,27 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-06-11 12:12</t>
+          <t>2026-06-11 17:34</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>X:@FabrizioRomano</t>
+          <t>X:@David_Ornstein</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>🚨🟣🔵 Excl: Zion Suzuki among 3 GKs in list at Aston Villa for summer window if Emiliano Martínez ends up leaving.
-Aston Villa aware of Juve being in talks with the Argentine GK but nothing agreed club to club yet.
-Suzuki been scouted for months at Parma.</t>
+          <t>🚨 Jose Mourinho has signed contract to become Real Madrid head coach. 63yo leaving Benfica for 2nd spell in charge of #RMFC after putting pen to paper last week on 3yr deal. Set to be announced post presidential election. W/ @MarioCortegana @TheAthleticFC https://www.nytimes.com/athletic/7284488/202</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>agreed, leaving, talks, talks with</t>
+          <t>deal, signed, leaving</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://nitter.net/FabrizioRomano/status/2064768287464894700#m</t>
+          <t>https://nitter.net/David_Ornstein/status/2060361927084167282#m</t>
         </is>
       </c>
     </row>
@@ -607,27 +605,27 @@
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-06-11 12:12</t>
+          <t>2026-06-11 17:34</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>X:@David_Ornstein</t>
+          <t>X:@premierleague</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>🚨 Jose Mourinho has signed contract to become Real Madrid head coach. 63yo leaving Benfica for 2nd spell in charge of #RMFC after putting pen to paper last week on 3yr deal. Set to be announced post presidential election. W/ @MarioCortegana @TheAthleticFC https://www.nytimes.com/athletic/7284488/202</t>
+          <t>Premier League clubs have confirmed which players are set to be released once their contract expires on June 30 ⬇️</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>deal, signed, leaving</t>
+          <t>confirmed, release, released, contract expires</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://nitter.net/David_Ornstein/status/2060361927084167282#m</t>
+          <t>https://nitter.net/premierleague/status/2064664119354015875#m</t>
         </is>
       </c>
     </row>
@@ -635,27 +633,27 @@
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-06-11 12:12</t>
+          <t>2026-06-11 17:34</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>X:@premierleague</t>
+          <t>X:@ManCity</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Premier League clubs have confirmed which players are set to be released once their contract expires on June 30 ⬇️</t>
+          <t>We are delighted to announce that Divine Mukasa has signed a new long-term deal with the Club 🩵</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>confirmed, release, released, contract expires</t>
+          <t>we are delighted to announce, are delighted to announce, deal, signed</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://nitter.net/premierleague/status/2064664119354015875#m</t>
+          <t>https://nitter.net/ManCity/status/2064347029867057428#m</t>
         </is>
       </c>
     </row>
@@ -663,27 +661,29 @@
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-06-11 12:12</t>
+          <t>2026-06-11 17:34</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>X:@ManCity</t>
+          <t>X:@SpursOfficial</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>We are delighted to announce that Divine Mukasa has signed a new long-term deal with the Club 🩵</t>
+          <t>We are delighted to announce that Ben Davies has signed a new contract with the club ✍️
+Congratulations, Ben! 🙌
+🔗 https://thfc.pro/4urnFuA</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>we are delighted to announce, are delighted to announce, deal, signed</t>
+          <t>we are delighted to announce, are delighted to announce, signed</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://nitter.net/ManCity/status/2064347029867057428#m</t>
+          <t>https://nitter.net/SpursOfficial/status/2064619165260923166#m</t>
         </is>
       </c>
     </row>
@@ -691,29 +691,27 @@
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-06-11 12:12</t>
+          <t>2026-06-11 17:34</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>X:@SpursOfficial</t>
+          <t>X:@ChelseaFC</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>We are delighted to announce that Ben Davies has signed a new contract with the club ✍️
-Congratulations, Ben! 🙌
-🔗 https://thfc.pro/4urnFuA</t>
+          <t>World Cup winners Chelsea have signed! 🏆</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>we are delighted to announce, are delighted to announce, signed</t>
+          <t>have signed, signed</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://nitter.net/SpursOfficial/status/2064619165260923166#m</t>
+          <t>https://nitter.net/ChelseaFC/status/2064760557182296531#m</t>
         </is>
       </c>
     </row>
@@ -721,7 +719,7 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-06-11 12:12</t>
+          <t>2026-06-11 17:34</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -731,17 +729,17 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>World Cup winners Chelsea have signed! 🏆</t>
+          <t>The list of Chelsea players who have been retained or released by the club at the end of the 25/26 season have been confirmed.</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>have signed, signed</t>
+          <t>⚠️ FOLLOW-UP CLICK LINK, confirmed, release, released</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://nitter.net/ChelseaFC/status/2064760557182296531#m</t>
+          <t>https://nitter.net/ChelseaFC/status/2064633680702627993#m</t>
         </is>
       </c>
     </row>
@@ -749,17 +747,17 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-06-11 12:12</t>
+          <t>2026-06-11 17:34</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>X:@ChelseaFC</t>
+          <t>X:@CPFC</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>The list of Chelsea players who have been retained or released by the club at the end of the 25/26 season have been confirmed.</t>
+          <t>The list of Crystal Palace players who have been retained or released by the club at the end of the 25/26 season has been confirmed.</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -769,7 +767,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://nitter.net/ChelseaFC/status/2064633680702627993#m</t>
+          <t>https://nitter.net/CPFC/status/2064681986711593211#m</t>
         </is>
       </c>
     </row>
@@ -777,27 +775,27 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-06-11 12:12</t>
+          <t>2026-06-11 17:34</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>X:@CPFC</t>
+          <t>X:@Coventry_City</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>The list of Crystal Palace players who have been retained or released by the club at the end of the 25/26 season has been confirmed.</t>
+          <t>We are delighted to announce that Victor Torp has signed a new contract with the Club. 🩵</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>⚠️ FOLLOW-UP CLICK LINK, confirmed, release, released</t>
+          <t>we are delighted to announce, are delighted to announce, signed</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://nitter.net/CPFC/status/2064681986711593211#m</t>
+          <t>https://nitter.net/Coventry_City/status/2060328196826878386#m</t>
         </is>
       </c>
     </row>
@@ -805,27 +803,27 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-06-11 12:12</t>
+          <t>2026-06-11 17:34</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>X:@Coventry_City</t>
+          <t>X:@BurnleyOfficial</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>We are delighted to announce that Victor Torp has signed a new contract with the Club. 🩵</t>
+          <t>Our retained and released list has been confirmed following the conclusion of the 2025/26 campaign 📋</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>we are delighted to announce, are delighted to announce, signed</t>
+          <t>⚠️ FOLLOW-UP CLICK LINK, confirmed, release, released</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://nitter.net/Coventry_City/status/2060328196826878386#m</t>
+          <t>https://nitter.net/BurnleyOfficial/status/2064665490576884001#m</t>
         </is>
       </c>
     </row>
@@ -833,27 +831,27 @@
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-06-11 12:12</t>
+          <t>2026-06-11 17:34</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>X:@BurnleyOfficial</t>
+          <t>maisfutebol RSS</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Our retained and released list has been confirmed following the conclusion of the 2025/26 campaign 📋</t>
+          <t>OFICIAL: Tomás Cordeiro assina contrato profissional com o Benfica</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>⚠️ FOLLOW-UP CLICK LINK, confirmed, release, released</t>
+          <t>OFICIAL, contrato</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://nitter.net/BurnleyOfficial/status/2064665490576884001#m</t>
+          <t>https://maisfutebol.iol.pt/benfica/contrato-profissional/oficial-tomas-cordeiro-assina-contrato-profissional-com-o-benfica</t>
         </is>
       </c>
     </row>
@@ -861,27 +859,27 @@
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-06-11 12:12</t>
+          <t>2026-06-11 17:34</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>maisfutebol RSS</t>
+          <t>maisfutebol cronologia</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>OFICIAL: Rob Edwards despedido do comando técnico do Wolverhampton</t>
+          <t>Rui Costa: «Mourinho sabia que era o treinador para a próxima época»</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>OFICIAL, deixa</t>
+          <t>anunciou, contrato, saída</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://maisfutebol.iol.pt/transferencias/inglaterra/oficial-rob-edwards-despedido-do-comando-tecnico-do-wolverhampton</t>
+          <t>https://maisfutebol.iol.pt/benfica/mercado-de-transferencias/rui-costa-jose-mourinho-sabia-que-era-o-treinador-para-a-proxima-epoca</t>
         </is>
       </c>
     </row>
@@ -889,27 +887,27 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-06-11 12:12</t>
+          <t>2026-06-11 17:34</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>maisfutebol RSS</t>
+          <t>maisfutebol cronologia</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>OFICIAL: Sampaoli substitui Carlos Tévez como novo treinador do Talleres</t>
+          <t>OFICIAL: Montréal devolve Iván Jaime ao FC Porto</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>OFICIAL, novo treinador</t>
+          <t>OFICIAL, anunciou, contrato, saída</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://maisfutebol.iol.pt/transferencias/jorge-sampaoli/oficial-sampaoli-substitui-carlos-tevez-como-novo-treinador-do-talleres</t>
+          <t>https://maisfutebol.iol.pt/fc-porto/mercado/oficial-montreal-devolve-ivan-jaime-ao-fc-porto</t>
         </is>
       </c>
     </row>
@@ -917,7 +915,7 @@
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-06-11 12:12</t>
+          <t>2026-06-11 17:34</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -927,17 +925,17 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>OFICIAL: Sampaoli substitui Carlos Tévez como novo treinador do Talleres</t>
+          <t>OFICIAL: Tomás Cordeiro assina contrato profissional com o Benfica</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>OFICIAL, novo treinador</t>
+          <t>OFICIAL, anunciou, contrato, saída</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://maisfutebol.iol.pt/transferencias/jorge-sampaoli/oficial-sampaoli-substitui-carlos-tevez-como-novo-treinador-do-talleres</t>
+          <t>https://maisfutebol.iol.pt/benfica/contrato-profissional/oficial-tomas-cordeiro-assina-contrato-profissional-com-o-benfica</t>
         </is>
       </c>
     </row>
@@ -945,7 +943,7 @@
       <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-06-11 12:12</t>
+          <t>2026-06-11 17:34</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -955,17 +953,17 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>OFICIAL: Mauro Jerónimo é o novo treinador do Borneo Samarinda</t>
+          <t>OFICIAL: Miguel Campos de saída do FK Oleksandriya</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>OFICIAL, novo treinador</t>
+          <t>OFICIAL, anunciou, contrato, saída</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://maisfutebol.iol.pt/oficial/indonesia/oficial-mauro-jeronimo-e-o-novo-treinador-do-borneo-samarinda</t>
+          <t>https://maisfutebol.iol.pt/cronologia/6373897a0cf2254fb2824fe4#OFICIAL: Miguel Campos de saída do FK Ol</t>
         </is>
       </c>
     </row>
@@ -973,7 +971,7 @@
       <c r="A19" t="inlineStr"/>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-06-11 12:12</t>
+          <t>2026-06-11 17:34</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -983,17 +981,17 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Ipswich anuncia saída do treinador que subiu a equipa duas vezes à Premier League</t>
+          <t>OFICIAL: Keisuke Goto assina com o Friburgo</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>anuncia, saída</t>
+          <t>OFICIAL, anunciou, contratação</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://maisfutebol.iol.pt/transferencias/mercado/ipswich-anuncia-saida-do-treinador-que-subiu-a-equipa-duas-vezes-a-premier-league</t>
+          <t>https://www.instagram.com/p/DZcJ8TMqro1/?utm_source=ig_embed&amp;utm_campaign=loading</t>
         </is>
       </c>
     </row>
@@ -1001,7 +999,7 @@
       <c r="A20" t="inlineStr"/>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-06-11 12:12</t>
+          <t>2026-06-11 17:34</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1011,17 +1009,157 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>OFICIAL: Adama Traoré e Fabianski deixam o West Ham</t>
+          <t>OFICIAL: Juan Iglesias é reforço do Sevilha</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>OFICIAL, deixa</t>
+          <t>OFICIAL, confirma, deixa</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://maisfutebol.iol.pt/transferencias/adama-traore/oficial-adama-traore-e-fabianski-deixam-o-west-ham</t>
+          <t>https://x.com/juan2iglesias?ref_src=twsrc%5Etfw</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-06-11 17:34</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Julián Calero é o novo treinador do Real Oviedo</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, novo treinador</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>https://t.co/XqshI72lx5</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr"/>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-06-11 17:34</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Sampaoli substitui Carlos Tévez como novo treinador do Talleres</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, chega, novo treinador</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/transferencias/jorge-sampaoli/oficial-sampaoli-substitui-carlos-tevez-como-novo-treinador-do-talleres</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr"/>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-06-11 17:34</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Bayer Leverkusen contrata pérola de 16 anos</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, chega</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>https://t.co/TRYeZsYnut</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr"/>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-06-11 17:34</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Mauro Jerónimo é o novo treinador do Borneo Samarinda</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, novo treinador</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/oficial/indonesia/oficial-mauro-jeronimo-e-o-novo-treinador-do-borneo-samarinda</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr"/>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-06-11 17:34</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Ipswich anuncia saída do treinador que subiu a equipa duas vezes à Premier League</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>anuncia, saída</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/transferencias/mercado/ipswich-anuncia-saida-do-treinador-que-subiu-a-equipa-duas-vezes-a-premier-league</t>
         </is>
       </c>
     </row>
@@ -1036,7 +1174,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1083,27 +1221,253 @@
       <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-11 12:12</t>
+          <t>2026-06-11 17:34</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>🚨🔴⚫️ AC Milan proceed in talks to find new manager and despite reports, nothing close or done with Oliver Glasner yet.
+Matthias Jaissle and Rúben Amorim are in the running as options to become new head coach.
+🎥🇮🇹 https://youtu.be/P5eGbnJi9-s</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>new head coach, new manager, talks</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2065097173805445363#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-06-11 17:34</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>X:@David_Ornstein</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>🚨 EXCL: Fulham have held talks with Alvaro Arbeloa about head coach vacancy following Marco Silva exit. 43yo Spaniard available after leaving Real Madrid &amp; has met #FFC to discuss possibility of taking Craven Cottage role. W/ @GuillermoRai_ @TheAthleticFC https://www.nytimes.com/athletic/7083005/202</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>leaving, talks, talks with</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>https://nitter.net/David_Ornstein/status/2064825056031580597#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-06-11 17:34</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Pepa bem encaminhado para ser o novo treinador do Estrela</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>novo treinador, perto de</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/liga/estrela-amadora/pepa-bem-encaminhado-para-ser-o-novo-treinador-do-estrela</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-06-11 17:34</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Gil Vicente: contactos por Luís Pinto</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>transferência, contratação, saída, interessado em</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/liga/gil-vicente/gil-vicente-contactos-por-luis-pinto</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-06-11 17:34</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Pepa bem encaminhado para ser o novo treinador do Estrela</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>transferência, contratação, saída, novo treinador, interessado em</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/liga/estrela-amadora/pepa-bem-encaminhado-para-ser-o-novo-treinador-do-estrela</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-06-11 17:34</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>II Liga: antigo adjunto de Petit vai treinar o Feirense</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>transferência, contratação, saída, interessado em</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/ii-liga/feirense/ii-liga-antigo-adjunto-de-petit-vai-treinar-o-feirense</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-06-11 17:34</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Newcastle já procura substituto de Gordon</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>transferência, contratação, saída, interessado em, procura</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>https://x.com/alex_crook?ref_src=twsrc%5Etfw</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-06-11 17:34</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>César Peixoto fechado no Wolverhampton</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>transferência, contrato, acordo verbal</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DZbCb9Yx00Y/?utm_source=ig_embed&amp;utm_campaign=loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-06-11 17:34</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Três portugueses e Arbeloa apontados à sucessão de Marco Silva</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>contrato, alvo, alvos, apontado, apontados</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>https://t.co/ucJFfBLPBf</t>
         </is>
       </c>
     </row>
@@ -1137,7 +1501,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Created: 2026-06-11 08:12</t>
+          <t>Created: 2026-06-11 13:34</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker refresh 14:21 EDT · van Hecke (BHA→TOT) Romano LOW tier · Tiago Ferreira FCP-B OFICIAL
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Transfer_Tracker.xlsx
+++ b/Transfer_Tracker.xlsx
@@ -500,7 +500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F198"/>
+  <dimension ref="A1:F287"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -3767,7 +3767,6 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" t="inlineStr"/>
       <c r="B120" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -3795,7 +3794,6 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" t="inlineStr"/>
       <c r="B121" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -3823,7 +3821,6 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" t="inlineStr"/>
       <c r="B122" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -3851,7 +3848,6 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" t="inlineStr"/>
       <c r="B123" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -3879,7 +3875,6 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" t="inlineStr"/>
       <c r="B124" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -3907,7 +3902,6 @@
       </c>
     </row>
     <row r="125">
-      <c r="A125" t="inlineStr"/>
       <c r="B125" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -3935,7 +3929,6 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" t="inlineStr"/>
       <c r="B126" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -3963,7 +3956,6 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" t="inlineStr"/>
       <c r="B127" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -3991,7 +3983,6 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" t="inlineStr"/>
       <c r="B128" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -4019,7 +4010,6 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" t="inlineStr"/>
       <c r="B129" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -4047,7 +4037,6 @@
       </c>
     </row>
     <row r="130">
-      <c r="A130" t="inlineStr"/>
       <c r="B130" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -4075,7 +4064,6 @@
       </c>
     </row>
     <row r="131">
-      <c r="A131" t="inlineStr"/>
       <c r="B131" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -4103,7 +4091,6 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" t="inlineStr"/>
       <c r="B132" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -4131,7 +4118,6 @@
       </c>
     </row>
     <row r="133">
-      <c r="A133" t="inlineStr"/>
       <c r="B133" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -4159,7 +4145,6 @@
       </c>
     </row>
     <row r="134">
-      <c r="A134" t="inlineStr"/>
       <c r="B134" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -4187,7 +4172,6 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" t="inlineStr"/>
       <c r="B135" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -4215,7 +4199,6 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" t="inlineStr"/>
       <c r="B136" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -4243,7 +4226,6 @@
       </c>
     </row>
     <row r="137">
-      <c r="A137" t="inlineStr"/>
       <c r="B137" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -4271,7 +4253,6 @@
       </c>
     </row>
     <row r="138">
-      <c r="A138" t="inlineStr"/>
       <c r="B138" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -4299,7 +4280,6 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" t="inlineStr"/>
       <c r="B139" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -4327,7 +4307,6 @@
       </c>
     </row>
     <row r="140">
-      <c r="A140" t="inlineStr"/>
       <c r="B140" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -4355,7 +4334,6 @@
       </c>
     </row>
     <row r="141">
-      <c r="A141" t="inlineStr"/>
       <c r="B141" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -4383,7 +4361,6 @@
       </c>
     </row>
     <row r="142">
-      <c r="A142" t="inlineStr"/>
       <c r="B142" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -4411,7 +4388,6 @@
       </c>
     </row>
     <row r="143">
-      <c r="A143" t="inlineStr"/>
       <c r="B143" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -4439,7 +4415,6 @@
       </c>
     </row>
     <row r="144">
-      <c r="A144" t="inlineStr"/>
       <c r="B144" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -4467,7 +4442,6 @@
       </c>
     </row>
     <row r="145">
-      <c r="A145" t="inlineStr"/>
       <c r="B145" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -4495,7 +4469,6 @@
       </c>
     </row>
     <row r="146">
-      <c r="A146" t="inlineStr"/>
       <c r="B146" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -4523,7 +4496,6 @@
       </c>
     </row>
     <row r="147">
-      <c r="A147" t="inlineStr"/>
       <c r="B147" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -4551,7 +4523,6 @@
       </c>
     </row>
     <row r="148">
-      <c r="A148" t="inlineStr"/>
       <c r="B148" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -4579,7 +4550,6 @@
       </c>
     </row>
     <row r="149">
-      <c r="A149" t="inlineStr"/>
       <c r="B149" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -4607,7 +4577,6 @@
       </c>
     </row>
     <row r="150">
-      <c r="A150" t="inlineStr"/>
       <c r="B150" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -4635,7 +4604,6 @@
       </c>
     </row>
     <row r="151">
-      <c r="A151" t="inlineStr"/>
       <c r="B151" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -4663,7 +4631,6 @@
       </c>
     </row>
     <row r="152">
-      <c r="A152" t="inlineStr"/>
       <c r="B152" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -4691,7 +4658,6 @@
       </c>
     </row>
     <row r="153">
-      <c r="A153" t="inlineStr"/>
       <c r="B153" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -4719,7 +4685,6 @@
       </c>
     </row>
     <row r="154">
-      <c r="A154" t="inlineStr"/>
       <c r="B154" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -4747,7 +4712,6 @@
       </c>
     </row>
     <row r="155">
-      <c r="A155" t="inlineStr"/>
       <c r="B155" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -4775,7 +4739,6 @@
       </c>
     </row>
     <row r="156">
-      <c r="A156" t="inlineStr"/>
       <c r="B156" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -4803,7 +4766,6 @@
       </c>
     </row>
     <row r="157">
-      <c r="A157" t="inlineStr"/>
       <c r="B157" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -4831,7 +4793,6 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" t="inlineStr"/>
       <c r="B158" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -4859,7 +4820,6 @@
       </c>
     </row>
     <row r="159">
-      <c r="A159" t="inlineStr"/>
       <c r="B159" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -4887,7 +4847,6 @@
       </c>
     </row>
     <row r="160">
-      <c r="A160" t="inlineStr"/>
       <c r="B160" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -4915,7 +4874,6 @@
       </c>
     </row>
     <row r="161">
-      <c r="A161" t="inlineStr"/>
       <c r="B161" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -4943,7 +4901,6 @@
       </c>
     </row>
     <row r="162">
-      <c r="A162" t="inlineStr"/>
       <c r="B162" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -4971,7 +4928,6 @@
       </c>
     </row>
     <row r="163">
-      <c r="A163" t="inlineStr"/>
       <c r="B163" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -4999,7 +4955,6 @@
       </c>
     </row>
     <row r="164">
-      <c r="A164" t="inlineStr"/>
       <c r="B164" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -5027,7 +4982,6 @@
       </c>
     </row>
     <row r="165">
-      <c r="A165" t="inlineStr"/>
       <c r="B165" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -5055,7 +5009,6 @@
       </c>
     </row>
     <row r="166">
-      <c r="A166" t="inlineStr"/>
       <c r="B166" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -5083,7 +5036,6 @@
       </c>
     </row>
     <row r="167">
-      <c r="A167" t="inlineStr"/>
       <c r="B167" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -5111,7 +5063,6 @@
       </c>
     </row>
     <row r="168">
-      <c r="A168" t="inlineStr"/>
       <c r="B168" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -5139,7 +5090,6 @@
       </c>
     </row>
     <row r="169">
-      <c r="A169" t="inlineStr"/>
       <c r="B169" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -5167,7 +5117,6 @@
       </c>
     </row>
     <row r="170">
-      <c r="A170" t="inlineStr"/>
       <c r="B170" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -5195,7 +5144,6 @@
       </c>
     </row>
     <row r="171">
-      <c r="A171" t="inlineStr"/>
       <c r="B171" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -5223,7 +5171,6 @@
       </c>
     </row>
     <row r="172">
-      <c r="A172" t="inlineStr"/>
       <c r="B172" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -5251,7 +5198,6 @@
       </c>
     </row>
     <row r="173">
-      <c r="A173" t="inlineStr"/>
       <c r="B173" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -5279,7 +5225,6 @@
       </c>
     </row>
     <row r="174">
-      <c r="A174" t="inlineStr"/>
       <c r="B174" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -5307,7 +5252,6 @@
       </c>
     </row>
     <row r="175">
-      <c r="A175" t="inlineStr"/>
       <c r="B175" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -5335,7 +5279,6 @@
       </c>
     </row>
     <row r="176">
-      <c r="A176" t="inlineStr"/>
       <c r="B176" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -5363,7 +5306,6 @@
       </c>
     </row>
     <row r="177">
-      <c r="A177" t="inlineStr"/>
       <c r="B177" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -5391,7 +5333,6 @@
       </c>
     </row>
     <row r="178">
-      <c r="A178" t="inlineStr"/>
       <c r="B178" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -5419,7 +5360,6 @@
       </c>
     </row>
     <row r="179">
-      <c r="A179" t="inlineStr"/>
       <c r="B179" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -5447,7 +5387,6 @@
       </c>
     </row>
     <row r="180">
-      <c r="A180" t="inlineStr"/>
       <c r="B180" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -5475,7 +5414,6 @@
       </c>
     </row>
     <row r="181">
-      <c r="A181" t="inlineStr"/>
       <c r="B181" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -5503,7 +5441,6 @@
       </c>
     </row>
     <row r="182">
-      <c r="A182" t="inlineStr"/>
       <c r="B182" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -5531,7 +5468,6 @@
       </c>
     </row>
     <row r="183">
-      <c r="A183" t="inlineStr"/>
       <c r="B183" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -5559,7 +5495,6 @@
       </c>
     </row>
     <row r="184">
-      <c r="A184" t="inlineStr"/>
       <c r="B184" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -5587,7 +5522,6 @@
       </c>
     </row>
     <row r="185">
-      <c r="A185" t="inlineStr"/>
       <c r="B185" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -5615,7 +5549,6 @@
       </c>
     </row>
     <row r="186">
-      <c r="A186" t="inlineStr"/>
       <c r="B186" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -5643,7 +5576,6 @@
       </c>
     </row>
     <row r="187">
-      <c r="A187" t="inlineStr"/>
       <c r="B187" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -5671,7 +5603,6 @@
       </c>
     </row>
     <row r="188">
-      <c r="A188" t="inlineStr"/>
       <c r="B188" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -5699,7 +5630,6 @@
       </c>
     </row>
     <row r="189">
-      <c r="A189" t="inlineStr"/>
       <c r="B189" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -5727,7 +5657,6 @@
       </c>
     </row>
     <row r="190">
-      <c r="A190" t="inlineStr"/>
       <c r="B190" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -5755,7 +5684,6 @@
       </c>
     </row>
     <row r="191">
-      <c r="A191" t="inlineStr"/>
       <c r="B191" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -5783,7 +5711,6 @@
       </c>
     </row>
     <row r="192">
-      <c r="A192" t="inlineStr"/>
       <c r="B192" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -5811,7 +5738,6 @@
       </c>
     </row>
     <row r="193">
-      <c r="A193" t="inlineStr"/>
       <c r="B193" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -5839,7 +5765,6 @@
       </c>
     </row>
     <row r="194">
-      <c r="A194" t="inlineStr"/>
       <c r="B194" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -5867,7 +5792,6 @@
       </c>
     </row>
     <row r="195">
-      <c r="A195" t="inlineStr"/>
       <c r="B195" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -5895,7 +5819,6 @@
       </c>
     </row>
     <row r="196">
-      <c r="A196" t="inlineStr"/>
       <c r="B196" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -5923,7 +5846,6 @@
       </c>
     </row>
     <row r="197">
-      <c r="A197" t="inlineStr"/>
       <c r="B197" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -5951,7 +5873,6 @@
       </c>
     </row>
     <row r="198">
-      <c r="A198" t="inlineStr"/>
       <c r="B198" t="inlineStr">
         <is>
           <t>2026-06-14 20:25</t>
@@ -5975,6 +5896,2433 @@
       <c r="F198" t="inlineStr">
         <is>
           <t>https://www.tottenhamhotspur.com/news/1072863/senesi-switch-sealed?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>2026-06-14 23:01</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D199" s="2" t="inlineStr">
+        <is>
+          <t>✨🇳🇱 OFFICIAL: Virgil van Dijk wins FIFA Man of the Match Award for Netherlands vs Japan.</t>
+        </is>
+      </c>
+      <c r="E199" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2066287786022367698#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>2026-06-15 00:01</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D200" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: João Graça deixa Rio Ave ao fim de cinco temporadas</t>
+        </is>
+      </c>
+      <c r="E200" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, transferência, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/transferencias/oficial/oficial-joao-graca-deixa-rio-ave-ao-fim-de-cinco-temporadas</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>2026-06-15 01:01</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D201" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: João Graça deixa Rio Ave ao fim de cinco temporadas</t>
+        </is>
+      </c>
+      <c r="E201" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, contrato, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/transferencias/oficial/oficial-joao-graca-deixa-rio-ave-ao-fim-de-cinco-temporadas</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>2026-06-15 02:01</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D202" s="2" t="inlineStr">
+        <is>
+          <t>⚡️🇨🇮 OFFICIAL: Yan Diomande, FIFA Man of the Match on his debut at World Cup at 19 years old!
+-Most touches (80)
+-Most chances created (5)
+-Most duels won (11)
+-Most progressive carries (15)
+-Most passes in attacking 3rd (22)</t>
+        </is>
+      </c>
+      <c r="E202" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2066334978611261793#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>2026-06-15 05:17</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D203" s="2" t="inlineStr">
+        <is>
+          <t>🔥🇸🇪 OFFICIAL: Alexander Isak, Man of the Match for Sweden against Tunisia.</t>
+        </is>
+      </c>
+      <c r="E203" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2066376631631896762#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>2026-06-15 09:05</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>X:@realmadrid</t>
+        </is>
+      </c>
+      <c r="D204" s="2" t="inlineStr">
+        <is>
+          <t>Comunicado Oficial: Cucurella.
+https://www.realmadrid.com/es-ES/noticias/club/comunicados/comunicado-oficial-cucurella-15-06-2026</t>
+        </is>
+      </c>
+      <c r="E204" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>https://nitter.net/realmadrid/status/2066446508392611973#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>2026-06-15 10:02</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D205" s="2" t="inlineStr">
+        <is>
+          <t>🚨 OFFICIAL: Marc Cucurella joins Real Madrid on €55m plus €5m add-ons deal from Chelsea.
+Contract until June 2032. Exclusive news, confirmed.</t>
+        </is>
+      </c>
+      <c r="E205" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, confirmed, deal, joins, 🚨 OFFICIAL, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2066446489006584029#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>2026-06-15 10:02</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D206" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Moreirense garante jovem espanhol do Bournemouth</t>
+        </is>
+      </c>
+      <c r="E206" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, transferência, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/liga/moreirense/oficial-moreirense-garante-jovem-espanhol-do-bournemouth</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>2026-06-15 10:02</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D207" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Cucurella é o primeiro reforço de Mourinho no Real Madrid</t>
+        </is>
+      </c>
+      <c r="E207" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/espanha/mercado/oficial-cucurella-e-o-primeiro-reforco-de-mourinho-no-real-madrid</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>2026-06-15 10:02</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D208" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Moreirense garante jovem espanhol do Bournemouth</t>
+        </is>
+      </c>
+      <c r="E208" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, transferência, contratação, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/liga/moreirense/oficial-moreirense-garante-jovem-espanhol-do-bournemouth</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>2026-06-15 10:02</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D209" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Cucurella é o primeiro reforço de Mourinho no Real Madrid</t>
+        </is>
+      </c>
+      <c r="E209" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, transferência, contratação, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/espanha/mercado/oficial-cucurella-e-o-primeiro-reforco-de-mourinho-no-real-madrid</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>2026-06-15 10:02</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D210" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Chelsea · Marc Cucurella — Transfer Out · - Real Madrid</t>
+        </is>
+      </c>
+      <c r="E210" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>https://www.chelseafc.com/en/news/article/marc-cucurella-departs-chelsea?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>2026-06-15 11:03</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D211" s="2" t="inlineStr">
+        <is>
+          <t>⚫️🔵 Atalanta have signed Croatian CB Ljubo Puljic from FC Bayern II. Four year contract confirmed.
+Croatian U19 centre back joined today, here with his agents from Bola Group. Done and sealed.</t>
+        </is>
+      </c>
+      <c r="E211" s="2" t="inlineStr">
+        <is>
+          <t>confirmed, have signed, signed, joined</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2066467709311668254#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>2026-06-15 11:03</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D212" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: AFC Bournemouth · Michael Dacosta Gonzalez — Transfer Out · - Moreirense</t>
+        </is>
+      </c>
+      <c r="E212" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>https://www.afcb.co.uk/news/2026/june/15/dacosta-gonzalez-completes-moreirense-switch/?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>2026-06-15 11:03</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D213" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Tottenham Hotspur · Yves Bissouma — Released</t>
+        </is>
+      </c>
+      <c r="E213" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>https://www.tottenhamhotspur.com/news/1072684/mens-player-update?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>2026-06-15 11:11</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D214" s="2" t="inlineStr">
+        <is>
+          <t>Iker Muniain é o novo treinador do Salamanca</t>
+        </is>
+      </c>
+      <c r="E214" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, contratação, novo treinador</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/cronologia/6373897a0cf2254fb2824fe4#Iker Muniain é o novo treinador do Salam</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>2026-06-15 12:01</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D215" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Mitchel van der Gaag está de regresso ao Marítimo</t>
+        </is>
+      </c>
+      <c r="E215" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, contratação, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/liga/maritimo/oficial-mitchel-van-der-gaag-esta-de-regresso-ao-maritimo</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>2026-06-15 13:00</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D216" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Mitchel van der Gaag está de regresso ao Marítimo</t>
+        </is>
+      </c>
+      <c r="E216" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/liga/maritimo/oficial-mitchel-van-der-gaag-esta-de-regresso-ao-maritimo</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>2026-06-15 13:00</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D217" s="2" t="inlineStr">
+        <is>
+          <t>Futebol feminino: Sporting anuncia cinco saídas</t>
+        </is>
+      </c>
+      <c r="E217" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anuncia, contratação, saída</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/sporting/futebol-feminino/futebol-feminino-sporting-anuncia-cinco-saidas</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>2026-06-15 13:00</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D218" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: António Folha ruma à Roménia e assume o Cluj</t>
+        </is>
+      </c>
+      <c r="E218" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, contratação, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/made-in/mercado-de-transferencias/oficial-antonio-folha-ruma-a-romenia-e-assume-o-cluj</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>2026-06-15 13:00</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D219" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Mitchell van der Gaag está de regresso ao Marítimo</t>
+        </is>
+      </c>
+      <c r="E219" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, contratação, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/liga/maritimo/oficial-mitchel-van-der-gaag-esta-de-regresso-ao-maritimo</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>2026-06-15 14:01</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D220" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: António Folha ruma à Roménia e assume o Cluj</t>
+        </is>
+      </c>
+      <c r="E220" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/made-in/mercado-de-transferencias/oficial-antonio-folha-ruma-a-romenia-e-assume-o-cluj</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>2026-06-15 14:01</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D221" s="2" t="inlineStr">
+        <is>
+          <t>Futebol feminino: Sporting anuncia cinco saídas</t>
+        </is>
+      </c>
+      <c r="E221" s="2" t="inlineStr">
+        <is>
+          <t>anuncia, saída</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/sporting/futebol-feminino/futebol-feminino-sporting-anuncia-cinco-saidas</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>2026-06-15 14:01</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D222" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Mitchell van der Gaag está de regresso ao Marítimo</t>
+        </is>
+      </c>
+      <c r="E222" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/liga/maritimo/oficial-mitchel-van-der-gaag-esta-de-regresso-ao-maritimo</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>2026-06-15 15:01</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>X:@IpswichTown</t>
+        </is>
+      </c>
+      <c r="D223" s="2" t="inlineStr">
+        <is>
+          <t>RT by @IpswichTown: 🤝 Ipswich Town Women is pleased to announce that Leah Mitchell has signed a new two-year deal with the club.</t>
+        </is>
+      </c>
+      <c r="E223" s="2" t="inlineStr">
+        <is>
+          <t>deal, signed</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>https://nitter.net/ITFCWomen/status/2066521109642846651#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>2026-06-15 15:01</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>X:@SEFutbol</t>
+        </is>
+      </c>
+      <c r="D224" s="2" t="inlineStr">
+        <is>
+          <t>Pinned: 🚨 OFICIAL | El 𝗢𝗡𝗖𝗘 del debut mundialista.
+¡Nosotros también firmamos nuestro compromiso con vosotros, equipo!
+#VamosEspaña | #CopaMundialFIFA</t>
+        </is>
+      </c>
+      <c r="E224" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, 🚨 OFICIAL</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>https://nitter.net/SEFutbol/status/2066522209632325632#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>2026-06-15 15:01</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D225" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Kiki Silva deixa o Casa Pia</t>
+        </is>
+      </c>
+      <c r="E225" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/casa-pia/kiki-silva/oficial-kiki-silva-deixa-o-casa-pia</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>2026-06-15 15:01</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D226" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Kiki Silva deixa o Casa Pia</t>
+        </is>
+      </c>
+      <c r="E226" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/casa-pia/kiki-silva/oficial-kiki-silva-deixa-o-casa-pia</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:01</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D227" s="2" t="inlineStr">
+        <is>
+          <t>🚨⚪️⚫️ Juventus activate €5m buy option clause for Jeremie Boga, joining on permanent deal from OGC Nice.
+Never in doubt after his impact over second part of the season. ✅</t>
+        </is>
+      </c>
+      <c r="E227" s="2" t="inlineStr">
+        <is>
+          <t>deal, joining</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2066546026752684264#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:01</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D228" s="2" t="inlineStr">
+        <is>
+          <t>🚨🔵 BREAKING: Joško Gvardiol deal, done and confirmed as he signs new contract at Manchester City.
+Agreement until June 2031 and move to Spain off for this summer.
+Seen as key player by director Viana and new coach Enzo Maresca.</t>
+        </is>
+      </c>
+      <c r="E228" s="2" t="inlineStr">
+        <is>
+          <t>confirmed, deal, signs</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2066539151877390486#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:01</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>X:@SEFutbol</t>
+        </is>
+      </c>
+      <c r="D229" s="2" t="inlineStr">
+        <is>
+          <t>🚨 OFICIAL | El 𝗢𝗡𝗖𝗘 del debut mundialista.
+¡Nosotros también firmamos nuestro compromiso con vosotros, equipo!
+#VamosEspaña | #CopaMundialFIFA</t>
+        </is>
+      </c>
+      <c r="E229" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, 🚨 OFICIAL</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>https://nitter.net/SEFutbol/status/2066522209632325632#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:01</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D230" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Anthony Lopes é reforço do Angers</t>
+        </is>
+      </c>
+      <c r="E230" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/franca/internacional/oficial-anthony-lopes-reforca-o-angers</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:01</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D231" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Maurizio Sarri é o novo treinador da Atalanta</t>
+        </is>
+      </c>
+      <c r="E231" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, novo treinador, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/transferencias/italia/oficial-maurizio-sarri-e-o-novo-treinador-da-atalanta</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>2026-06-15 16:01</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D232" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: César Peixoto é o novo treinador do Wolverhampton</t>
+        </is>
+      </c>
+      <c r="E232" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, novo treinador, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mercado/transferencias/oficial-cesar-peixoto-e-o-novo-treinador-do-wolverhampton</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>2026-06-15 17:01</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D233" s="2" t="inlineStr">
+        <is>
+          <t>🚨🇹🇳 OFFICIAL: Tunisia head coach Sabri Lamouchi has been sacked after defeat on World Cup opening game against Sweden.
+Plans are under way ‌to appoint ‌Mondher Kebaier as the new national team ‌coach on an interim basis, Federation confirm.</t>
+        </is>
+      </c>
+      <c r="E233" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2066563523266699422#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>2026-06-15 17:01</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D234" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Anthony Lopes é reforço do Angers</t>
+        </is>
+      </c>
+      <c r="E234" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/franca/internacional/oficial-anthony-lopes-reforca-o-angers</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>2026-06-15 17:01</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D235" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Maurizio Sarri é o novo treinador da Atalanta</t>
+        </is>
+      </c>
+      <c r="E235" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, saída, novo treinador, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/transferencias/italia/oficial-maurizio-sarri-e-o-novo-treinador-da-atalanta</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>2026-06-15 17:01</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D236" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: César Peixoto é o novo treinador do Wolverhampton</t>
+        </is>
+      </c>
+      <c r="E236" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, novo treinador, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mercado/transferencias/oficial-cesar-peixoto-e-o-novo-treinador-do-wolverhampton</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>2026-06-15 17:01</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D237" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Lucas João rescinde com o Nacional</t>
+        </is>
+      </c>
+      <c r="E237" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mercado/liga/oficial-lucas-joao-rescinde-com-o-nacional</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>2026-06-15 18:01</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>X:@premierleague</t>
+        </is>
+      </c>
+      <c r="D238" s="2" t="inlineStr">
+        <is>
+          <t>🦅 @CPFC have confirmed the appointment of Pierre Sage as their new manager on a three-year contract</t>
+        </is>
+      </c>
+      <c r="E238" s="2" t="inlineStr">
+        <is>
+          <t>confirmed, new manager</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>https://nitter.net/premierleague/status/2066568964851785905#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>2026-06-15 18:01</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D239" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Jérémie Boga em definitivo na Juventus</t>
+        </is>
+      </c>
+      <c r="E239" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mercado/italia/oficial-jeremie-boga-em-definitivo-na-juventus</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>2026-06-15 18:01</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D240" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Lucas João rescinde com o Nacional</t>
+        </is>
+      </c>
+      <c r="E240" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, contrato, saída, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mercado/liga/oficial-lucas-joao-rescinde-com-o-nacional</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>2026-06-15 18:01</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D241" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Sage prefere a Liga Europa à Champions e vai treinar o Crystal Palace</t>
+        </is>
+      </c>
+      <c r="E241" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mercado/inglaterra/oficial-sage-prefere-a-liga-europa-a-champions-e-vai-treinar-o-crystal-palace</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>2026-06-15 18:01</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D242" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Jérémie Boga em definitivo na Juventus</t>
+        </is>
+      </c>
+      <c r="E242" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mercado/italia/oficial-jeremie-boga-em-definitivo-na-juventus</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>2026-06-15 18:01</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D243" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Brighton &amp; Hove Albion · Costinha — Transfer In · - Olympiacos</t>
+        </is>
+      </c>
+      <c r="E243" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>https://www.brightonandhovealbion.com/media-article/mft-transfer-news-costinha-olympiacos-june-2026?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>2026-06-15 18:06</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D244" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Costinha vai disputar a Premier League pelo Brighton</t>
+        </is>
+      </c>
+      <c r="E244" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mercado/made-in/oficial-costinha-vai-disputar-a-premier-league-pelo-brighton</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>2026-06-15 19:04</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D245" s="2" t="inlineStr">
+        <is>
+          <t>🌎🇨🇻 OFFICIAL: Vozinha wins FIFA Man of the Match Award for Spain-Cape Verde. 👏🏼</t>
+        </is>
+      </c>
+      <c r="E245" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2066589849226772736#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>2026-06-15 19:04</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D246" s="2" t="inlineStr">
+        <is>
+          <t>🌎🇨🇻 OFFICIAL: Vozinha is the oldest goalkeeper to keep a clean sheet on a World Cup debut, @OptaJoe reports. 🏅</t>
+        </is>
+      </c>
+      <c r="E246" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2066586201172082808#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>2026-06-15 19:04</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D247" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Costinha vai disputar a Premier League pelo Brighton</t>
+        </is>
+      </c>
+      <c r="E247" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mercado/made-in/oficial-costinha-vai-disputar-a-premier-league-pelo-brighton</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>2026-06-15 19:04</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D248" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Sage prefere a Liga Europa à Champions e vai treinar o Crystal Palace</t>
+        </is>
+      </c>
+      <c r="E248" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mercado/inglaterra/oficial-sage-prefere-a-liga-europa-a-champions-e-vai-treinar-o-crystal-palace</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>2026-06-15 19:04</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D249" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Agostinho Bento sucede a Tarantini no banco do Paredes</t>
+        </is>
+      </c>
+      <c r="E249" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, novo treinador, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/cronologia/6373897a0cf2254fb2824fe4#OFICIAL: Agostinho Bento sucede a Tarant</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>2026-06-15 19:04</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D250" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Everton · Isaac Heath — Transfer Out · - Cambridge United</t>
+        </is>
+      </c>
+      <c r="E250" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>https://www.evertonfc.com/news/2026/june/15/heath-departs-for-cambridge?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch?utm_source=premier-league&amp;utm_med</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>2026-06-15 20:01</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D251" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Udinese garante Zaniolo até 2029</t>
+        </is>
+      </c>
+      <c r="E251" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, novo treinador, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mercado/italia/oficial-udinese-garante-zaniolo-ate-2029</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>2026-06-15 21:01</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D252" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Udinese garante Zaniolo até 2029</t>
+        </is>
+      </c>
+      <c r="E252" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, empréstimo, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mercado/italia/oficial-udinese-garante-zaniolo-ate-2029</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>2026-06-15 23:01</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D253" s="2" t="inlineStr">
+        <is>
+          <t>🚨⚪️ Antonio Rüdiger has officially signed his new Real Madrid contract valid until June 2027.
+Announcement coming very soon, likely in next 24 hours. ✅🇩🇪</t>
+        </is>
+      </c>
+      <c r="E253" s="2" t="inlineStr">
+        <is>
+          <t>officially, signed</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2066642303582716133#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>2026-06-16 02:01</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D254" s="2" t="inlineStr">
+        <is>
+          <t>🚨 OFFICIAL: Fede Valverde wins FIFA Man of the Match Award for Uruguay-Saudi. 🇺🇾</t>
+        </is>
+      </c>
+      <c r="E254" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, 🚨 OFFICIAL, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2066694767677669467#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>2026-06-16 08:28</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D255" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Lamouchi deixa a Tunísia, Hervé Renard assume o comando</t>
+        </is>
+      </c>
+      <c r="E255" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mundial-2026/mundial2026/oficial-lamouchi-deixa-a-tunisia-herve-renard-assume-o-comando</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>2026-06-16 08:28</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D256" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Lamouchi deixa a Tunísia, Hervé Renard assume o comando</t>
+        </is>
+      </c>
+      <c r="E256" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, deixa, novo treinador, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mundial-2026/mundial2026/oficial-lamouchi-deixa-a-tunisia-herve-renard-assume-o-comando</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>2026-06-16 09:43</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>X:@David_Ornstein</t>
+        </is>
+      </c>
+      <c r="D257" s="2" t="inlineStr">
+        <is>
+          <t>🚨 Marcus Rashford deal at Man Utd includes £40m clause for all clubs bar #MCFC &amp; #LFC. €30m buy option in Barcelona loan expired yesterday. If returns to #MUFC 28yo’s preference is to honour contract (2028) rather than join another PL side @TheAthleticFC https://www.nytimes.com/athletic/7361885/2026</t>
+        </is>
+      </c>
+      <c r="E257" s="2" t="inlineStr">
+        <is>
+          <t>deal, loan</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>https://nitter.net/David_Ornstein/status/2066800458220359737#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>2026-06-16 09:43</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>X:@realmadrid</t>
+        </is>
+      </c>
+      <c r="D258" s="2" t="inlineStr">
+        <is>
+          <t>Comunicado Oficial: Rüdiger.
+https://www.realmadrid.com/es-ES/noticias/club/comunicados/rudiger-16-06-2026</t>
+        </is>
+      </c>
+      <c r="E258" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>https://nitter.net/realmadrid/status/2066808864947806550#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>2026-06-16 09:43</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D259" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Rüdiger renova pelo Real Madrid por mais uma época</t>
+        </is>
+      </c>
+      <c r="E259" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/internacional/real-madrid/oficial-rudiger-renova-pelo-real-madrid-por-mais-uma-epoca</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>2026-06-16 09:43</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D260" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Léo Teixeira é reforço do Petrolul</t>
+        </is>
+      </c>
+      <c r="E260" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DZnlGljqhJK/?utm_source=ig_embed&amp;utm_campaign=loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>2026-06-16 12:10</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D261" s="2" t="inlineStr">
+        <is>
+          <t>🚨🇩🇪 OFFICIAL: Real Madrid confirm new deal for Toni Rüdiger, as revealed. ✅🔐
+Agreement signed until June 2027, here wirh Sahr Senesie, Hasan Cetinkaya and Alexander Bergweiler from HCM Sports Management after the official signature.
+Deal approved by José Mourinho.</t>
+        </is>
+      </c>
+      <c r="E261" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, deal, signed, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2066809890115293237#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>2026-06-16 12:10</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>X:@SpursOfficial</t>
+        </is>
+      </c>
+      <c r="D262" s="2" t="inlineStr">
+        <is>
+          <t>RT by @SpursOfficial: “I called my Mum &amp; Dad on FaceTime, they were both crying! It was a really nice moment for us to have together.”
+A wholesome family link-up ahead of Father's Day as Tinka and dad Joachim reminisce over her journey to Spurs 🤍
+📺 http://thfc.pro/4uGMDGu</t>
+        </is>
+      </c>
+      <c r="E262" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>https://nitter.net/SpursWomen/status/2066810020155560384#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>2026-06-16 12:10</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D263" s="2" t="inlineStr">
+        <is>
+          <t>César Peixoto e a saída do Gil Vicente: «É um adeus com o coração apertado»</t>
+        </is>
+      </c>
+      <c r="E263" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, saída, deixa</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/liga/gil-vicente/cesar-peixoto-e-a-saida-do-gil-vicente-e-um-adeus-com-o-coracao-apertado</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>2026-06-16 12:10</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D264" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Rüdiger renova pelo Real Madrid por mais uma época</t>
+        </is>
+      </c>
+      <c r="E264" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/internacional/real-madrid/oficial-rudiger-renova-pelo-real-madrid-por-mais-uma-epoca</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>2026-06-16 12:10</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D265" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Dino Toppmöller é o novo treinador do Lens</t>
+        </is>
+      </c>
+      <c r="E265" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, novo treinador, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/internacional/franca/oficial-dino-toppmoller-e-o-novo-treinador-do-lens</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>2026-06-16 12:10</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D266" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Gil Vicente assegura contratação de promessa ex-Sporting</t>
+        </is>
+      </c>
+      <c r="E266" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, transferência, contratação, contrato, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/liga/gil-vicente/oficial-gil-vicente-assegura-contratacao-de-promessa-ex-sporting</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>2026-06-16 12:10</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D267" s="2" t="inlineStr">
+        <is>
+          <t>Gil Vicente: Luís Pinto na linha da frente para suceder a César Peixoto</t>
+        </is>
+      </c>
+      <c r="E267" s="2" t="inlineStr">
+        <is>
+          <t>anunciou, contratação</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/liga/gil-vicente/gil-vicente-luis-pinto-na-linha-da-frente-para-suceder-a-cesar-peixoto</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>2026-06-16 12:10</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D268" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Arouna Sangante é reforço do Sevilha até 2031</t>
+        </is>
+      </c>
+      <c r="E268" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contratação, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>https://x.com/hashtag/WeareSevilla?src=hash&amp;ref_src=twsrc%5Etfw</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>2026-06-16 12:10</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D269" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Edson Farias renova com a Académica de Coimbra</t>
+        </is>
+      </c>
+      <c r="E269" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contrato, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DZpPfgkCnqj/?utm_source=ig_embed&amp;utm_campaign=loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>2026-06-16 12:10</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D270" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Ricardinho e António Montez assinam pelo Lusitânia de Lourosa</t>
+        </is>
+      </c>
+      <c r="E270" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DZmtz81jN13/?utm_source=ig_embed&amp;utm_campaign=loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>2026-06-16 12:10</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D271" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Miguel Mota deixa o P. Ferreira e ruma à Moldávia</t>
+        </is>
+      </c>
+      <c r="E271" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, transferência, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/cronologia/6373897a0cf2254fb2824fe4#OFICIAL: Miguel Mota deixa o P. Ferreira</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>2026-06-16 13:01</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D272" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Gil Vicente assegura contratação de promessa ex-Sporting</t>
+        </is>
+      </c>
+      <c r="E272" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, contratação, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/liga/gil-vicente/oficial-gil-vicente-assegura-contratacao-de-promessa-ex-sporting</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>2026-06-16 14:01</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D273" s="2" t="inlineStr">
+        <is>
+          <t>Antiga promessa neerlandesa anuncia fim de carreira aos 26 anos</t>
+        </is>
+      </c>
+      <c r="E273" s="2" t="inlineStr">
+        <is>
+          <t>anuncia, transferência, contrato</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/internacional/paises-baixos/antiga-promessa-neerlandesa-anuncia-fim-de-carreira-aos-26-anos</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>2026-06-16 15:01</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D274" s="2" t="inlineStr">
+        <is>
+          <t>🚨 Official: Trevoh Chalobah replaces Tino Livramento into the England squad. ✅🏴󠁧󠁢󠁥󠁮󠁧󠁿</t>
+        </is>
+      </c>
+      <c r="E274" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, 🚨 OFFICIAL, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2066883925457133621#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>2026-06-16 15:01</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D275" s="2" t="inlineStr">
+        <is>
+          <t>Antiga promessa neerlandesa anuncia fim de carreira aos 26 anos</t>
+        </is>
+      </c>
+      <c r="E275" s="2" t="inlineStr">
+        <is>
+          <t>anuncia, contrato</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/internacional/paises-baixos/antiga-promessa-neerlandesa-anuncia-fim-de-carreira-aos-26-anos</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>2026-06-16 17:02</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D276" s="2" t="inlineStr">
+        <is>
+          <t>🚨🔴⚫️ OFFICIAL: AC Milan appoint Rúben Amorim as new head coach.
+“We’ve been following him for years and his style of play at Sporting is exactly what we are looking for”, says Gerry Cardinale.</t>
+        </is>
+      </c>
+      <c r="E276" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, new head coach, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2066915221906559359#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>2026-06-16 17:02</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D277" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Famalicão reforça meio-campo com internacional húngaro</t>
+        </is>
+      </c>
+      <c r="E277" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contratação, contrato, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/famalicao/liga/oficial-famalicao-reforca-meio-campo-com-internacional-hungaro</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>2026-06-16 17:02</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D278" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Ruben Amorim é o novo treinador do Milan</t>
+        </is>
+      </c>
+      <c r="E278" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contratação, contrato, novo treinador, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/milan/internacional/oficial-ruben-amorim-e-o-novo-treinador-do-milan</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>2026-06-16 17:02</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D279" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: médio da seleção sub-20 alemã a caminho do Heidenheim</t>
+        </is>
+      </c>
+      <c r="E279" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contratação, contrato, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>https://t.co/fzylTNCe4X</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>2026-06-16 17:02</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D280" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Daisuke Yokota vai ficar no Hannover 96</t>
+        </is>
+      </c>
+      <c r="E280" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contrato, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>https://x.com/hashtag/Yokota?src=hash&amp;ref_src=twsrc%5Etfw</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>2026-06-16 18:15</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D281" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Arouca prolonga contrato de Pablo Gozálbez até 2029</t>
+        </is>
+      </c>
+      <c r="E281" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, contrato, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/arouca/liga/oficial-arouca-prolonga-contrato-de-pablo-gozalbez-ate-2029</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>2026-06-16 18:15</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D282" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: fundo norte-americano não entra no capital social do Benfica</t>
+        </is>
+      </c>
+      <c r="E282" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/liga/benfica/benfica-rejeita-entrada-de-capital-norte-americano-na-sad</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>2026-06-16 18:15</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D283" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Famalicão reforça meio-campo com internacional húngaro</t>
+        </is>
+      </c>
+      <c r="E283" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, chega, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/famalicao/liga/oficial-famalicao-reforca-meio-campo-com-internacional-hungaro</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>2026-06-16 18:15</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D284" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Ruben Amorim é o novo treinador do Milan</t>
+        </is>
+      </c>
+      <c r="E284" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, regressa, novo treinador, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/milan/internacional/oficial-ruben-amorim-e-o-novo-treinador-do-milan</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>2026-06-16 18:15</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D285" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Dailon Livramento deixa o Casa Pia</t>
+        </is>
+      </c>
+      <c r="E285" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, contrato, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/transferencias/casa-pia/oficial-dailon-livramento-deixa-o-casa-pia</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>2026-06-16 18:15</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D286" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Arouca prolonga contrato de Pablo Gozálbez até 2029</t>
+        </is>
+      </c>
+      <c r="E286" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, contrato, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/arouca/liga/oficial-arouca-prolonga-contrato-de-pablo-gozalbez-ate-2029</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr"/>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>2026-06-16 18:21</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D287" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Tiago Ferreira regressa ao FC Porto para a equipa B</t>
+        </is>
+      </c>
+      <c r="E287" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, contrato, regressa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mercado/fc-porto/tiago-ferreira-regressa-ao-fc-porto-para-a-equipa-b</t>
         </is>
       </c>
     </row>
@@ -5984,6 +8332,1042 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="80" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>When (UTC)</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Title / Headline</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Keywords matched</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-06-11 17:34</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>🚨🔴⚫️ AC Milan proceed in talks to find new manager and despite reports, nothing close or done with Oliver Glasner yet.
+Matthias Jaissle and Rúben Amorim are in the running as options to become new head coach.
+🎥🇮🇹 https://youtu.be/P5eGbnJi9-s</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>new head coach, new manager, talks</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2065097173805445363#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-06-11 17:34</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>X:@David_Ornstein</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>🚨 EXCL: Fulham have held talks with Alvaro Arbeloa about head coach vacancy following Marco Silva exit. 43yo Spaniard available after leaving Real Madrid &amp; has met #FFC to discuss possibility of taking Craven Cottage role. W/ @GuillermoRai_ @TheAthleticFC https://www.nytimes.com/athletic/7083005/202</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>leaving, talks, talks with</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>https://nitter.net/David_Ornstein/status/2064825056031580597#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-06-11 17:34</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Pepa bem encaminhado para ser o novo treinador do Estrela</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>novo treinador, perto de</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/liga/estrela-amadora/pepa-bem-encaminhado-para-ser-o-novo-treinador-do-estrela</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-06-11 17:34</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Gil Vicente: contactos por Luís Pinto</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>transferência, contratação, saída, interessado em</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/liga/gil-vicente/gil-vicente-contactos-por-luis-pinto</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-06-11 17:34</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Pepa bem encaminhado para ser o novo treinador do Estrela</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>transferência, contratação, saída, novo treinador, interessado em</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/liga/estrela-amadora/pepa-bem-encaminhado-para-ser-o-novo-treinador-do-estrela</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-06-11 17:34</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>II Liga: antigo adjunto de Petit vai treinar o Feirense</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>transferência, contratação, saída, interessado em</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/ii-liga/feirense/ii-liga-antigo-adjunto-de-petit-vai-treinar-o-feirense</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-06-11 17:34</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Newcastle já procura substituto de Gordon</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>transferência, contratação, saída, interessado em, procura</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>https://x.com/alex_crook?ref_src=twsrc%5Etfw</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-06-11 17:34</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>César Peixoto fechado no Wolverhampton</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>transferência, contrato, acordo verbal</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DZbCb9Yx00Y/?utm_source=ig_embed&amp;utm_campaign=loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-06-11 17:34</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Três portugueses e Arbeloa apontados à sucessão de Marco Silva</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>contrato, alvo, alvos, apontado, apontados</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>https://t.co/ucJFfBLPBf</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-06-11 21:00</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Jornal espanhol dá Bernardo Silva praticamente fechado no Real Madrid</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>contrato, apontado</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/made-in/espanha/jornal-espanhol-da-bernardo-silva-praticamente-fechado-no-real-madrid</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-06-12 23:00</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>RT by @FabrizioRomano: 🚨🔴⚫️ AC Milan proceed in talks to find new manager and despite reports, nothing close or done with Oliver Glasner yet.
+Matthias Jaissle and Rúben Amorim are in the running as options to become new head coach.
+🎥🇮🇹 https://youtu.be/P5eGbnJi9-s</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>new head coach, new manager, talks</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2065097173805445363#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-06-13 16:00</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Big one for football fans.
+@X’s brand new Soccer Custom Timeline powered for the beautiful game.
+48 nations, one platform — this is how you follow football in 2026.
+Here we go! ⚽🔥</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>HERE WE GO, Here we go!, Here We Go, here we go</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2065817683434578034#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-06-14 17:00</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Marc Cucurella joins Real Madrid for €60m package from Chelsea. Here we go. ✅💣</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>joins, HERE WE GO, Here We Go, here we go</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2066197566421692491#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-06-14 17:00</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Pinned: 🚨💣 EXCLUSIVE: Real Madrid reach verbal agreement to sign Marc Cucurella from Chelsea, HERE WE GO!
+Verbal agreement in place between all parties, player too — he’s the left back wanted by Mourinho. Details to follow.
+Cucurella leaves #CFC and joins Madrid after World Cup. ⚪️🇪🇸</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>joins, leaves, verbal agreement, HERE WE GO, Here we go!, Here We Go</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2066186850688029165#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-06-14 18:09</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>RT by @FabrizioRomano: 🚨💣 EXCLUSIVE: Real Madrid reach verbal agreement to sign Marc Cucurella from Chelsea, HERE WE GO!
+Verbal agreement in place between all parties, player too — he’s the left back wanted by Mourinho. Details to follow.
+Cucurella leaves #CFC and joins Madrid after World Cup. ⚪️🇪</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>joins, leaves, verbal agreement, HERE WE GO, Here we go!, Here We Go</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2066186850688029165#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-06-14 20:25</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>🚨💣 BREAKING: Marc Cucurella deal is signed and sealed after surprising exclusive story earlier today.
+Real Madrid to pay €55m fixed fee plus €5m add-ons as Chelsea allowed medical tests.
+Cucurella, new Real Madrid player. 🇪🇸
+Here we go, confirmed. ✅🇪🇸</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>confirmed, deal, signed, HERE WE GO, Here We Go, here we go</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2066253922054947063#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-06-14 23:01</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Marc Cucurella will become a Real Madrid player today, Monday. 💣🆕</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>joins, leaves, verbal agreement, HERE WE GO, Here we go!, Here We Go</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2066281246271942767#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-06-15 09:05</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>🚨✅⚪️ #RealMadrid</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>joins, leaves, verbal agreement, HERE WE GO, Here we go!, Here We Go</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2066446083471933822#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-06-15 09:05</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>🚨🔴⚪️ The exclusive story from two weeks ago, set to become a done deal: Bayern are set to negotiate final details of Ismael Saibari deal.
+Here we go, following next — Saibari already plans for medical in the US.</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>deal, HERE WE GO, Here We Go, here we go</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2066433528070369636#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-06-15 10:02</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>🚨 BREAKING: Ismael Saibari to FC Bayern, HERE WE GO! Deal sealed 🔴⚪️🇲🇦
+Exactly two weeks after exclusive story on Bayern in talks for surprise move, Saibari joins the German champions.
+€55m fee to PSV Eindhoven, medical in USA and then official. All done. ✅</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>deal, joins, talks, HERE WE GO, Here we go!, Here We Go</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2066448878837121047#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-06-15 11:03</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>🔴🔵 Pierre Sage, new #CPFC head coach since Tuesday with all documents in place. 🦅</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>deal, new head coach, HERE WE GO, Here we go!, Here We Go, here we go</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2066470224359051543#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-06-15 11:03</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>RT by @FabrizioRomano: 🚨🔴⚫️ BREAKING: Rúben Amorim to AC Milan as new head coach, HERE WE GO! 🇵🇹
+Verbal agreement done on deal valid until June 2028 plus option until June 2029.
+Amorim has accepted all conditions and will sign this week as new Milan manager. 🫱🏻‍🫲🏼</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>deal, new head coach, verbal agreement, HERE WE GO, Here we go!, Here We Go</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2066457880438448483#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-06-15 11:03</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Acordo verbal entre Ruben Amorim e o Milan</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>transferência, contratação, acordo verbal</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/made-in/internacional/acordo-verbal-entre-ruben-amorim-e-o-milan</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-06-15 11:11</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>🚨🔴⚪️ Giovanni van Bronckhorst will be the new head coach at Feyenoord, deal done and here we go!
+Former Liverpool assistant coach returns to Netherlands and signs as Feyenoord coach.
+Sipke Hulshoff will be the assistant coach.</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>deal, signs, new head coach, HERE WE GO, Here we go!, Here We Go</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2066475655898746948#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-06-15 23:01</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Famalicão negocia contratação de médio internacional húngaro</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>contratação, novo treinador, negocia</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mercado/15-06-2026/famalicao-negocia-contratacao-de-medio-internacional-hungaro</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-06-16 00:01</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Famalicão negocia contratação de médio internacional húngaro</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>contratação, negocia</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mercado/15-06-2026/famalicao-negocia-contratacao-de-medio-internacional-hungaro</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-06-16 07:18</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>🚨🔴🔵 Senny Mayulu signs new deal at Paris Saint-Germain until June 2031, done and here we go!
+All set for PSG gem to stay as @FabriceHawkins reported.
+Two English top clubs were keen but Mayulu wanted to stay.</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>deal, signs, HERE WE GO, Here we go!, Here We Go, here we go</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2066768988366082150#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-06-16 08:28</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>🚨🔵 Manchester City have agreed deal to sign Hermann Malonga as new centre back from PSG, here we go!
+2008 born talent has accepted all terms offered by #MCFC and joins from Paris Saint-Germain to City project.</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>agreed, deal, joins, HERE WE GO, Here we go!, Here We Go</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2066778048368709806#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-06-16 09:43</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>🚨 More on Sandro Tonali and Spurs exclusive story.
+#THFC believe Tonali’s open to joining and keen on the move, while talks with Newcastle will follow on price/package.
+Tottenham want to go ahead strong and get it done as it’s a priority target wanted by De Zerbi.
+🎥 https://youtu.be/aECk3qGyuA8?s</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>joining, talks, talks with</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2066794909491990925#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026-06-16 12:10</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>🚨 BREAKING: Bernardo Silva has now officially signed his Real Madrid contract.
+Here we go from one week ago now confirmed as Portuguese midfielder joins on initial two year deal plus option to extend.
+Wanted by José Mourinho. ⚪️🇵🇹</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>officially, confirmed, deal, signed, joins, HERE WE GO</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2066849770849612238#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026-06-16 12:10</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>🚨🔴⚫️ Understand Rúben Amorim has signed his contract as new AC Milan head coach until June 2028.
+The agreement is valid for two years with one more season as option, as always reported.
+Here we go, formally confirmed. ✅🇵🇹</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>confirmed, signed, HERE WE GO, Here We Go, here we go</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2066817501472665971#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026-06-16 12:10</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>César Peixoto e a saída do Gil Vicente: «É um adeus com o coração apertado»</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>transferência, saída, em conversações</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/liga/gil-vicente/cesar-peixoto-e-a-saida-do-gil-vicente-e-um-adeus-com-o-coracao-apertado</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-06-16 12:10</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Inglaterra: Tottenham avança para a contratação de Tonali</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>transferência, contratação, em conversações</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/cronologia/6373897a0cf2254fb2824fe4#Inglaterra: Tottenham avança para a cont</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026-06-16 15:01</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Football gaming has a new dimension!
+Copa City game has launched with a purpose: Giving you the power to organize football matches, adapt real cities and manage massive fan crowds on PS5, Xbox X|S, and PC.
+Get @copacitygame now on a platform of your choice!
+HERE WE GO!
+#copacity #ad</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>HERE WE GO, Here we go!, Here We Go, here we go</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2066883837112528918#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2026-06-16 18:15</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>🚨 Tottenham agree deal to sign Jan Paul van Hecke from Brighton, here we go! 💣
+New defender wanted by De Zerbi joining on £52m deal, agreement club to club done after player accepted #THFC conditions last week.
+All done and Vuskovic separate case, as @David_Ornstein reports.</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>deal, joining, HERE WE GO, Here we go!, Here We Go, here we go</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2066932361866969202#m</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6001,32 +9385,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>When (UTC)</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>Title / Headline</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>Keywords matched</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
@@ -6035,252 +9419,254 @@
     <row r="2">
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-11 17:34</t>
+          <t>2026-06-12 23:00</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>X:@FabrizioRomano</t>
+          <t>maisfutebol RSS</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>🚨🔴⚫️ AC Milan proceed in talks to find new manager and despite reports, nothing close or done with Oliver Glasner yet.
-Matthias Jaissle and Rúben Amorim are in the running as options to become new head coach.
-🎥🇮🇹 https://youtu.be/P5eGbnJi9-s</t>
+          <t>Lukebakio e a época de estreia no Benfica: «Mal consegui mostrar o meu valor»</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>new head coach, new manager, talks</t>
+          <t>lesão, lesão</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://nitter.net/FabrizioRomano/status/2065097173805445363#m</t>
+          <t>https://maisfutebol.iol.pt/benfica/mundial-2026/lukebakio-e-a-epoca-de-estreia-no-benfica-mal-consegui-mostrar-o-meu-valor</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-06-11 17:34</t>
+          <t>2026-06-13 00:25</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>X:@David_Ornstein</t>
+          <t>maisfutebol RSS</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>🚨 EXCL: Fulham have held talks with Alvaro Arbeloa about head coach vacancy following Marco Silva exit. 43yo Spaniard available after leaving Real Madrid &amp; has met #FFC to discuss possibility of taking Craven Cottage role. W/ @GuillermoRai_ @TheAthleticFC https://www.nytimes.com/athletic/7083005/202</t>
+          <t>Mundial 2026: lesão afasta Michael Oliver do Costa do Marfim-Equador</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>leaving, talks, talks with</t>
+          <t>lesão, lesão</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://nitter.net/David_Ornstein/status/2064825056031580597#m</t>
+          <t>https://maisfutebol.iol.pt/mundial-2026/mundial2026/mundial-2026-lesao-afasta-michael-oliver-do-costa-do-marfim-equador</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-06-11 17:34</t>
+          <t>2026-06-13 04:00</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>maisfutebol RSS</t>
+          <t>X:@FabrizioRomano</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Pepa bem encaminhado para ser o novo treinador do Estrela</t>
+          <t>🚨🇺🇸 No injury or any serious issue for Christian Pulisic after excellent World Cup debut then subbed off at half time.
+Pulisic has been subbed off as precaution.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>novo treinador, perto de</t>
+          <t>injury, injury</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://maisfutebol.iol.pt/liga/estrela-amadora/pepa-bem-encaminhado-para-ser-o-novo-treinador-do-estrela</t>
+          <t>https://nitter.net/FabrizioRomano/status/2065634657555677431#m</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-06-11 17:34</t>
+          <t>2026-06-13 18:00</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>maisfutebol cronologia</t>
+          <t>maisfutebol RSS</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Gil Vicente: contactos por Luís Pinto</t>
+          <t>Superbikes: Miguel Oliveira regressa à competição com pontos</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>transferência, contratação, saída, interessado em</t>
+          <t>lesão, regressa, lesão</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://maisfutebol.iol.pt/liga/gil-vicente/gil-vicente-contactos-por-luis-pinto</t>
+          <t>https://maisfutebol.iol.pt/superbikes/mundial/superbikes-miguel-oliveira-regressa-a-competicao-com-pontos</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-06-11 17:34</t>
+          <t>2026-06-13 23:01</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>maisfutebol cronologia</t>
+          <t>X:@England</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Pepa bem encaminhado para ser o novo treinador do Estrela</t>
+          <t>Straight to work 💪
+All 27 of our #ThreeLions are out for our first training session in Kansas City.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>transferência, contratação, saída, novo treinador, interessado em</t>
+          <t>out for</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://maisfutebol.iol.pt/liga/estrela-amadora/pepa-bem-encaminhado-para-ser-o-novo-treinador-do-estrela</t>
+          <t>https://nitter.net/England/status/2065922633275789639#m</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-06-11 17:34</t>
+          <t>2026-06-15 03:41</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>maisfutebol cronologia</t>
+          <t>User report</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>II Liga: antigo adjunto de Petit vai treinar o Feirense</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>transferência, contratação, saída, interessado em</t>
+          <t>🚨 Gabriel Gudmundsson (LEE LB · SWE LB) injured during SWE v TUN MD1 · subbed off · LEE opener-prep concern · banks ~2 MD1 pts only</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>injury · sub off · LEE</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://maisfutebol.iol.pt/ii-liga/feirense/ii-liga-antigo-adjunto-de-petit-vai-treinar-o-feirense</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-06-11 17:34</t>
+          <t>2026-06-15 09:05</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>maisfutebol cronologia</t>
+          <t>X:@LFC</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Newcastle já procura substituto de Gordon</t>
+          <t>Wataru ❤️
+The Japan team show their support for Wataru Endo after his withdrawal from the tournament due to injury 🇯🇵 #FIFAWorldCup</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>transferência, contratação, saída, interessado em, procura</t>
+          <t>injury, injury</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://x.com/alex_crook?ref_src=twsrc%5Etfw</t>
+          <t>https://nitter.net/LFC/status/2066445904760963330#m</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-06-11 17:34</t>
+          <t>2026-06-16 12:10</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>maisfutebol cronologia</t>
+          <t>X:@David_Ornstein</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>César Peixoto fechado no Wolverhampton</t>
+          <t>🚨 Tino Livramento to miss World Cup with calf injury. Not serious but major blow for Newcastle United defender &amp; #England ahead of #2026FIFAWorldCup opener vs #Croatia  - 23yo returning to #NUFC + Trevoh Chalobah called up @TheAthleticFC post @Matt_Law_DT https://www.nytimes.com/athletic/7365471/202</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>transferência, contrato, acordo verbal</t>
+          <t>miss world cup, injury, calf injury, injury, miss world cup</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DZbCb9Yx00Y/?utm_source=ig_embed&amp;utm_campaign=loading</t>
+          <t>https://nitter.net/David_Ornstein/status/2066854654982463927#m</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-06-11 17:34</t>
+          <t>2026-06-16 13:01</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>maisfutebol cronologia</t>
+          <t>X:@David_Ornstein</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Três portugueses e Arbeloa apontados à sucessão de Marco Silva</t>
+          <t>R to @David_Ornstein: 🚨 Trevoh Chalobah called up last night &amp; travelling to join #England squad in USA. 26yo Chelsea defender not expected to be involved against #Croatia but will be available for subsequent group #2026FIFAWorldCup matches vs #Ghana  &amp; #Panama 
+@TheAthleticFC https://www.nytimes.co</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>contrato, alvo, alvos, apontado, apontados</t>
+          <t>injury, injury</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://t.co/ucJFfBLPBf</t>
+          <t>https://nitter.net/David_Ornstein/status/2066860492295950545#m</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-06-11 21:00</t>
+          <t>2026-06-16 13:01</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -6290,24 +9676,24 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Jornal espanhol dá Bernardo Silva praticamente fechado no Real Madrid</t>
+          <t>Mundial 2026: Tino Livramento lesiona-se e desfalca Inglaterra</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>contrato, apontado</t>
+          <t>lesão, lesão</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://maisfutebol.iol.pt/made-in/espanha/jornal-espanhol-da-bernardo-silva-praticamente-fechado-no-real-madrid</t>
+          <t>https://maisfutebol.iol.pt/internacional/inglaterra/mundial-2026-tino-livramento-lesiona-se-e-desfalca-inglaterra</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-06-12 23:00</t>
+          <t>2026-06-16 14:01</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -6317,356 +9703,157 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>RT by @FabrizioRomano: 🚨🔴⚫️ AC Milan proceed in talks to find new manager and despite reports, nothing close or done with Oliver Glasner yet.
-Matthias Jaissle and Rúben Amorim are in the running as options to become new head coach.
-🎥🇮🇹 https://youtu.be/P5eGbnJi9-s</t>
+          <t>🚨🏴󠁧󠁢󠁥󠁮󠁧󠁿 OFFICIAL: England confirm Tino Livramento will be out of the World Cup due to injury.
+Trevoh Chalobah has been called up. ✅</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>new head coach, new manager, talks</t>
+          <t>out of the world cup, out of the world, injury, OFFICIAL:, out of the world cup, injury</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://nitter.net/FabrizioRomano/status/2065097173805445363#m</t>
+          <t>https://nitter.net/FabrizioRomano/status/2066879106155753490#m</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-06-13 16:00</t>
+          <t>2026-06-16 14:01</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>X:@FabrizioRomano</t>
+          <t>X:@NUFC</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Big one for football fans.
-@X’s brand new Soccer Custom Timeline powered for the beautiful game.
-48 nations, one platform — this is how you follow football in 2026.
-Here we go! ⚽🔥</t>
+          <t>Tino Livramento has withdrawn from @England's #FIFAWorldCup 2026 squad. 
+The 23-year-old picked up a minor calf injury in training with the Three Lions on Sunday afternoon. A subsequent scan and medical assessment on Monday unfortunately confirmed he could play no further part in England's tourname</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>HERE WE GO, Here we go!, Here We Go, here we go</t>
+          <t>withdrawn from, injury, calf injury, confirmed, withdrawn from, injury</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://nitter.net/FabrizioRomano/status/2065817683434578034#m</t>
+          <t>https://nitter.net/NUFC/status/2066875900944056421#m</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-06-14 17:00</t>
+          <t>2026-06-16 14:01</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>X:@FabrizioRomano</t>
+          <t>X:@England</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Marc Cucurella joins Real Madrid for €60m package from Chelsea. Here we go. ✅💣</t>
+          <t>Tino Livramento has withdrawn from the #ThreeLions squad due to injury.
+We're gutted for you, Tino, and wishing you a speedy recovery. ❤️</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>joins, HERE WE GO, Here We Go, here we go</t>
+          <t>withdrawn from, injury, withdrawn from, injury</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://nitter.net/FabrizioRomano/status/2066197566421692491#m</t>
+          <t>https://nitter.net/England/status/2066873454838587820#m</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-06-14 17:00</t>
+          <t>2026-06-16 15:01</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>X:@FabrizioRomano</t>
+          <t>maisfutebol RSS</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Pinned: 🚨💣 EXCLUSIVE: Real Madrid reach verbal agreement to sign Marc Cucurella from Chelsea, HERE WE GO!
-Verbal agreement in place between all parties, player too — he’s the left back wanted by Mourinho. Details to follow.
-Cucurella leaves #CFC and joins Madrid after World Cup. ⚪️🇪🇸</t>
+          <t>Mundial 2026: Tino Livramento lesiona-se e é substituído por Chalobah</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>joins, leaves, verbal agreement, HERE WE GO, Here we go!, Here We Go</t>
+          <t>lesão, lesão</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://nitter.net/FabrizioRomano/status/2066186850688029165#m</t>
+          <t>https://maisfutebol.iol.pt/internacional/inglaterra/mundial-2026-tino-livramento-lesiona-se-e-desfalca-inglaterra</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-06-14 18:09</t>
+          <t>2026-06-16 16:01</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>X:@FabrizioRomano</t>
+          <t>X:@premierleague</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>RT by @FabrizioRomano: 🚨💣 EXCLUSIVE: Real Madrid reach verbal agreement to sign Marc Cucurella from Chelsea, HERE WE GO!
-Verbal agreement in place between all parties, player too — he’s the left back wanted by Mourinho. Details to follow.
-Cucurella leaves #CFC and joins Madrid after World Cup. ⚪️🇪</t>
+          <t>A teenage Trevoh Chalobah always believed 🥹
+The @ChelseaFC defender will be joining Thomas Tuchel’s World Cup squad in place of the injured Tino Livramento</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>joins, leaves, verbal agreement, HERE WE GO, Here we go!, Here We Go</t>
+          <t>injured, joining, injured</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://nitter.net/FabrizioRomano/status/2066186850688029165#m</t>
+          <t>https://nitter.net/premierleague/status/2066901740121665956#m</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-06-14 20:25</t>
+          <t>2026-06-16 16:01</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>X:@FabrizioRomano</t>
+          <t>X:@premierleague</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>🚨💣 BREAKING: Marc Cucurella deal is signed and sealed after surprising exclusive story earlier today.
-Real Madrid to pay €55m fixed fee plus €5m add-ons as Chelsea allowed medical tests.
-Cucurella, new Real Madrid player. 🇪🇸
-Here we go, confirmed. ✅🇪🇸</t>
+          <t>A teenage Trevoh Chalobah always believed 🥹
+The @ChelseaFC defender will be joining Thomas Tuchel’s World Cup squad in place of the injured Tino Livramento</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>confirmed, deal, signed, HERE WE GO, Here We Go, here we go</t>
+          <t>injured, joining, injured</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://nitter.net/FabrizioRomano/status/2066253922054947063#m</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="80" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>When (UTC)</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>Title / Headline</t>
-        </is>
-      </c>
-      <c r="E1" s="5" t="inlineStr">
-        <is>
-          <t>Keywords matched</t>
-        </is>
-      </c>
-      <c r="F1" s="5" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-06-12 23:00</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>maisfutebol RSS</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Lukebakio e a época de estreia no Benfica: «Mal consegui mostrar o meu valor»</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>lesão, lesão</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>https://maisfutebol.iol.pt/benfica/mundial-2026/lukebakio-e-a-epoca-de-estreia-no-benfica-mal-consegui-mostrar-o-meu-valor</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-06-13 00:25</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>maisfutebol RSS</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Mundial 2026: lesão afasta Michael Oliver do Costa do Marfim-Equador</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>lesão, lesão</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>https://maisfutebol.iol.pt/mundial-2026/mundial2026/mundial-2026-lesao-afasta-michael-oliver-do-costa-do-marfim-equador</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-06-13 04:00</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>X:@FabrizioRomano</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>🚨🇺🇸 No injury or any serious issue for Christian Pulisic after excellent World Cup debut then subbed off at half time.
-Pulisic has been subbed off as precaution.</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>injury, injury</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>https://nitter.net/FabrizioRomano/status/2065634657555677431#m</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-06-13 18:00</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>maisfutebol RSS</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Superbikes: Miguel Oliveira regressa à competição com pontos</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>lesão, regressa, lesão</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>https://maisfutebol.iol.pt/superbikes/mundial/superbikes-miguel-oliveira-regressa-a-competicao-com-pontos</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2026-06-13 23:01</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>X:@England</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Straight to work 💪
-All 27 of our #ThreeLions are out for our first training session in Kansas City.</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>out for</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>https://nitter.net/England/status/2065922633275789639#m</t>
+          <t>https://nitter.net/premierleague/status/2066901705279549451#m</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bernardo Silva → RMA OFICIAL Jun 17 · MCI/RMA statements · 2-yr deal until 2028
Also: filter cycling false positives (Van Aert · Tour2026) from INJURY tab.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Transfer_Tracker.xlsx
+++ b/Transfer_Tracker.xlsx
@@ -500,7 +500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F287"/>
+  <dimension ref="A1:F307"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -8299,7 +8299,6 @@
       </c>
     </row>
     <row r="287">
-      <c r="A287" t="inlineStr"/>
       <c r="B287" t="inlineStr">
         <is>
           <t>2026-06-16 18:21</t>
@@ -8323,6 +8322,561 @@
       <c r="F287" t="inlineStr">
         <is>
           <t>https://maisfutebol.iol.pt/mercado/fc-porto/tiago-ferreira-regressa-ao-fc-porto-para-a-equipa-b</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>2026-06-16 19:01</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D288" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Dailon Livramento deixa o Casa Pia</t>
+        </is>
+      </c>
+      <c r="E288" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/transferencias/casa-pia/oficial-dailon-livramento-deixa-o-casa-pia</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>2026-06-16 19:01</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D289" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Tiago Ferreira regressa ao FC Porto para a equipa B</t>
+        </is>
+      </c>
+      <c r="E289" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, regressa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mercado/fc-porto/tiago-ferreira-regressa-ao-fc-porto-para-a-equipa-b</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>2026-06-16 20:01</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D290" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Álvaro Pacheco deixa o Casa Pia</t>
+        </is>
+      </c>
+      <c r="E290" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, confirma, saída, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/liga/16-06-2026/oficial-alvaro-pacheco-deixa-o-casa-pia</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>2026-06-16 20:01</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D291" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Álvaro Pacheco deixa o Casa Pia</t>
+        </is>
+      </c>
+      <c r="E291" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, contrato, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/liga/16-06-2026/oficial-alvaro-pacheco-deixa-o-casa-pia</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>2026-06-16 21:01</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D292" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: jogo entre V. Guimarães e Santos cancelado</t>
+        </is>
+      </c>
+      <c r="E292" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/vitoria-guimaraes/santos/oficial-jogo-entre-v-guimaraes-e-santos-cancelado</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>2026-06-16 22:01</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D293" s="2" t="inlineStr">
+        <is>
+          <t>🚨🇫🇷 OFFICIAL: Michael Olise, FIFA Man of the Match on his World Cup debut.
+✨ 1 assist
+👌🏼 100% shot accuracy, 2/2
+🧞‍♂️ 14 passes into final third 
+🛡️ 6/9 ground duels won
+🧠 4 chances created
+💥 2 big chances created
+🍿 2/3 successful dribbles</t>
+        </is>
+      </c>
+      <c r="E293" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2066998694612758869#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>2026-06-16 23:01</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D294" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Shabab Al Ahli confirma saída de Paulo Sousa</t>
+        </is>
+      </c>
+      <c r="E294" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, confirma, transferência, saída, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/emirados-arabes-unidos/paulo-sousa/oficial-paulo-sousa-deixa-o-comando-tecnico-do-al-ahli</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:01</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D295" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Shabab Al Ahli confirma saída de Paulo Sousa</t>
+        </is>
+      </c>
+      <c r="E295" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, confirma, saída, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/emirados-arabes-unidos/paulo-sousa/oficial-paulo-sousa-deixa-o-comando-tecnico-do-al-ahli</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>2026-06-17 01:01</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D296" s="2" t="inlineStr">
+        <is>
+          <t>🚨🧘🏼‍♂️ OFFICIAL: Erling Haaland wins FIFA Man of the Match for Norway-Iraq on his first World Cup game ever.
+2 goals today, and 22 goals (!) in last 11 games in major competitions with Norway.</t>
+        </is>
+      </c>
+      <c r="E296" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067044742882275462#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>2026-06-17 01:01</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D297" s="2" t="inlineStr">
+        <is>
+          <t>🚨🇵🇹 OFFICIAL: Ruben Dias misses Portugal opening game against Congo. ❌⚠️
+“He’s not fully fit and we won’t take any risks”, says Roberto Martínez.</t>
+        </is>
+      </c>
+      <c r="E297" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067039841859014812#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>2026-06-17 04:01</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D298" s="2" t="inlineStr">
+        <is>
+          <t>🚨🏆 OFFICIAL: Lionel Messi wins FIFA Man of the Match against Algeria. 🇦🇷</t>
+        </is>
+      </c>
+      <c r="E298" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067085157601853605#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>2026-06-17 04:01</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D299" s="2" t="inlineStr">
+        <is>
+          <t>🚨 OFFICIAL: Lionel Messi, TOP SCORER EVER in World Cup history joint with Miro Klose. 🎞️⭐️
+16 goals at the World Cup. 💥🇦🇷
+In one night, on 6th World Cup debut game at 38, Messi surpasses Mbappé (14), Müller (14) and Ronaldo Nazario (15).</t>
+        </is>
+      </c>
+      <c r="E299" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, 🚨 OFFICIAL, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067076943770423654#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>2026-06-17 09:16</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>X:@realmadrid</t>
+        </is>
+      </c>
+      <c r="D300" s="2" t="inlineStr">
+        <is>
+          <t>Comunicado Oficial: Bernardo Silva.</t>
+        </is>
+      </c>
+      <c r="E300" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>https://nitter.net/realmadrid/status/2067170635583807614#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>2026-06-17 09:16</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D301" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Bernardo Silva é reforço do Real Madrid</t>
+        </is>
+      </c>
+      <c r="E301" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contratação, contrato, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/transferencias/oficial/oficial-bernardo-silva-e-reforco-do-real-madrid</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>2026-06-17 09:16</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D302" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Habib Sylla troca U. Leiria pelo Otelul Galati</t>
+        </is>
+      </c>
+      <c r="E302" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contratação, contrato, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/cronologia/6373897a0cf2254fb2824fe4#OFICIAL: Habib Sylla troca U. Leiria pel</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:19</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D303" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Bernardo Silva é reforço do Real Madrid</t>
+        </is>
+      </c>
+      <c r="E303" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/transferencias/oficial/oficial-bernardo-silva-e-reforco-do-real-madrid</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>2026-06-17 11:16</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D304" s="2" t="inlineStr">
+        <is>
+          <t>Nice avança com «chicotada» que atinge treinador e presidente</t>
+        </is>
+      </c>
+      <c r="E304" s="2" t="inlineStr">
+        <is>
+          <t>anuncia, saída</t>
+        </is>
+      </c>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/franca/internacional/nice-avanca-com-chicotada-que-atinge-treinador-e-presidente</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>2026-06-17 12:01</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>X:@AVFCOfficial</t>
+        </is>
+      </c>
+      <c r="D305" s="2" t="inlineStr">
+        <is>
+          <t>RT by @AVFCOfficial: Mia McAulay is a Villan ❤️‍🔥</t>
+        </is>
+      </c>
+      <c r="E305" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>https://nitter.net/AVWFCOfficial/status/2067200590547935582#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr"/>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>2026-06-17 12:46</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D306" s="2" t="inlineStr">
+        <is>
+          <t>🚨 OFFICIAL: Real Madrid statement on Negreira case.
+Real Madrid C. F. communicates that, in relation to the so-called 'Negreira Case', he has presented to UEFA a letter addressed to its disciplinary bodies.
+In this letter, the club has informed UEFA of the existence of relevant evidence that concl</t>
+        </is>
+      </c>
+      <c r="E306" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, 🚨 OFFICIAL, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067216547647570076#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr"/>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>2026-06-17 12:46</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D307" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Ruan Tressoldi fica em definitivo no At. Mineiro</t>
+        </is>
+      </c>
+      <c r="E307" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contrato, saída, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>https://x.com/hashtag/ForzaSasol?src=hash&amp;ref_src=twsrc%5Etfw</t>
         </is>
       </c>
     </row>
@@ -8337,7 +8891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -9362,6 +9916,91 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026-06-16 22:01</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>🚨🔴⚫️ Afonso Moreira to Bayer Leverkusen, here we go! Deal done and sealed tonight.
+Olympique Lyon receive €32m transfer fee from Bayer 04.
+Medical scheduled this week.</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>deal, HERE WE GO, Here we go!, Here We Go, here we go</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2066992446542631062#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2026-06-17 10:19</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>X:@ManCity</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Bernardo Silva is set to join Real Madrid after leaving City this summer.
+🔗 http://mancity.co/BernardoRM</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>leaving, set to join</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>https://nitter.net/ManCity/status/2067182089208844337#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr"/>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2026-06-17 12:46</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>✅✍🏼🔴⚫️ #Bayer04</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>deal, HERE WE GO, Here we go!, Here We Go, here we go</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067222832979820632#m</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9373,7 +10012,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -9854,6 +10493,60 @@
       <c r="F17" t="inlineStr">
         <is>
           <t>https://nitter.net/premierleague/status/2066901705279549451#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-06-16 21:01</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Mundial 2026: Neymar treina pela primeira vez após sofrer lesão</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>lesão, lesão</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mundial2026/mundial-2026/mundial-2026-neymar-treina-pela-primeira-vez-apos-sofrer-lesao</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-06-17 11:16</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Ciclismo: Van Aert falha Tour2026 devido a lesão no cotovelo</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>lesão, lesão</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/ciclismo/modalidades/ciclismo-van-aert-falha-tour2026-devido-a-lesao-no-cotovelo</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker refresh 17:34 EDT · Kane WC milestone + Neves MOTM (non-txfr) · Jay-Morgan CHE→WBA LOW tier · Grealish injury return
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Transfer_Tracker.xlsx
+++ b/Transfer_Tracker.xlsx
@@ -500,7 +500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F307"/>
+  <dimension ref="A1:F324"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -8823,7 +8823,6 @@
       </c>
     </row>
     <row r="306">
-      <c r="A306" t="inlineStr"/>
       <c r="B306" t="inlineStr">
         <is>
           <t>2026-06-17 12:46</t>
@@ -8853,7 +8852,6 @@
       </c>
     </row>
     <row r="307">
-      <c r="A307" t="inlineStr"/>
       <c r="B307" t="inlineStr">
         <is>
           <t>2026-06-17 12:46</t>
@@ -8877,6 +8875,470 @@
       <c r="F307" t="inlineStr">
         <is>
           <t>https://x.com/hashtag/ForzaSasol?src=hash&amp;ref_src=twsrc%5Etfw</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:01</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D308" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Van Bronckhorst é o novo treinador do Feyenoord</t>
+        </is>
+      </c>
+      <c r="E308" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, regressa, novo treinador, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/transferencias/giovanni-van-bronckhorst/oficial-van-bronckhorst-e-o-novo-treinador-do-feyenoord</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:01</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D309" s="2" t="inlineStr">
+        <is>
+          <t>Voleibol: Benfica anuncia novo treinador da equipa masculina</t>
+        </is>
+      </c>
+      <c r="E309" s="2" t="inlineStr">
+        <is>
+          <t>anuncia, contrato, novo treinador</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/modalidades/voleibol/voleibol-benfica-anuncia-novo-treinador-da-equipa-masculina</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:01</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D310" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: técnico do Lecce renova por mais um ano</t>
+        </is>
+      </c>
+      <c r="E310" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>https://t.co/ZpyrtjotTJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>2026-06-17 15:01</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D311" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Van Bronckhorst é o novo treinador do Feyenoord</t>
+        </is>
+      </c>
+      <c r="E311" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, novo treinador, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/transferencias/giovanni-van-bronckhorst/oficial-van-bronckhorst-e-o-novo-treinador-do-feyenoord</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>2026-06-17 16:01</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D312" s="2" t="inlineStr">
+        <is>
+          <t>🚨🇵🇹 OFFICIAL: Cristiano Ronaldo starts for Portugal and plays his 6th World Cup. 👋🏼</t>
+        </is>
+      </c>
+      <c r="E312" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067270992410312732#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>2026-06-17 16:01</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D313" s="2" t="inlineStr">
+        <is>
+          <t>🚨 Inter agree deal to sign Ivan Provedel as new goalkeeper from Lazio for €3m ⚫️🔵
+Provedel signs a three year deal and joins as backup for the Spanish goalkeeper Josep Martinez — starting next season. 🧤🇮🇹</t>
+        </is>
+      </c>
+      <c r="E313" s="2" t="inlineStr">
+        <is>
+          <t>deal, signs, joins</t>
+        </is>
+      </c>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067265640763707460#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>2026-06-17 16:01</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D314" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Tokinho Dória ruma ao Amarante</t>
+        </is>
+      </c>
+      <c r="E314" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DZsIFpPjGOh/?utm_source=ig_embed&amp;utm_campaign=loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>2026-06-17 17:01</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D315" s="2" t="inlineStr">
+        <is>
+          <t>🚨 OFFICIAL: Barcelona statement.
+“The president of FC Barcelona, Rafael Yuste y Abel, today sent a formal letter to the presidents of LaLiga, Javier Tebas; of the Royal Spanish Football Federation (RFEF), Rafael Louzán; and the Technical Committee of Referees (CTA), Francisco Soto, in relation to t</t>
+        </is>
+      </c>
+      <c r="E315" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, 🚨 OFFICIAL, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067286551864779216#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>2026-06-17 17:01</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D316" s="2" t="inlineStr">
+        <is>
+          <t>Martin Demichelis, new RB Leipzig head coach already since last week. 🔴⚪️👋🏼
+Release clause activated from Mallorca and deal pre-signed five days ago. ✅🇩🇪</t>
+        </is>
+      </c>
+      <c r="E316" s="2" t="inlineStr">
+        <is>
+          <t>deal, signed, release, new head coach</t>
+        </is>
+      </c>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067279809823084638#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>2026-06-17 17:01</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D317" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Ole Werner de saída do Leipzig</t>
+        </is>
+      </c>
+      <c r="E317" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, saída, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>https://t.co/IWyVpjA4kq</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>2026-06-17 17:01</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D318" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Danny Röhl deixa o Rangers e ruma ao RB Salzburgo</t>
+        </is>
+      </c>
+      <c r="E318" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, saída, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>https://t.co/gGfL9YAOvF</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>2026-06-17 19:01</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D319" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Rui Ferreira deixa comando técnico do Felgueiras</t>
+        </is>
+      </c>
+      <c r="E319" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, deixa, chega, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/ii-liga/felgueiras/oficial-rui-ferreira-deixa-comando-tecnico-do-felgueiras</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>2026-06-17 19:01</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D320" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Rui Ferreira deixa comando técnico do Felgueiras</t>
+        </is>
+      </c>
+      <c r="E320" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, saída, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/ii-liga/felgueiras/oficial-rui-ferreira-deixa-comando-tecnico-do-felgueiras</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>2026-06-17 19:01</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D321" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Rui Ferreira deixa comando técnico do Felgueiras</t>
+        </is>
+      </c>
+      <c r="E321" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, saída, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F321" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DZsNl2wgekh/?utm_source=ig_embed&amp;utm_campaign=loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>2026-06-17 20:01</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D322" s="2" t="inlineStr">
+        <is>
+          <t>🌎🇵🇹 OFFICIAL: João Neves, FIFA Man of the Match for Portugal-DR Congo.</t>
+        </is>
+      </c>
+      <c r="E322" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067328949982474296#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>2026-06-17 21:01</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D323" s="2" t="inlineStr">
+        <is>
+          <t>🚨🏴󠁧󠁢󠁥󠁮󠁧󠁿 OFFICIAL: Harry Kane becomes England BEST SCORER EVER at the World Cup with 10 goals in 12 games! 🤖
+He’s level with English legend Gary Lineker.</t>
+        </is>
+      </c>
+      <c r="E323" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067347949223371078#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr"/>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>2026-06-17 21:35</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D324" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Famalicão empresta médio georgiano ao Wolfsberger</t>
+        </is>
+      </c>
+      <c r="E324" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, saída, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F324" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/liga/famalicao/oficial-famalicao-empresta-medio-georgiano-ao-wolfsberger</t>
         </is>
       </c>
     </row>
@@ -8891,7 +9353,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -9974,7 +10436,6 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr"/>
       <c r="B39" t="inlineStr">
         <is>
           <t>2026-06-17 12:46</t>
@@ -9998,6 +10459,34 @@
       <c r="F39" t="inlineStr">
         <is>
           <t>https://nitter.net/FabrizioRomano/status/2067222832979820632#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2026-06-17 19:01</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>🚨 Jimmy Jay-Morgan from Chelsea to West Brom, here we go! Deal agreed today for £4m total package.
+#CFC also included a sell-on clause as part of the deal.</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>agreed, deal, HERE WE GO, Here we go!, Here We Go, here we go</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067313857266172393#m</t>
         </is>
       </c>
     </row>
@@ -10012,7 +10501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -10547,6 +11036,87 @@
       <c r="F19" t="inlineStr">
         <is>
           <t>https://maisfutebol.iol.pt/ciclismo/modalidades/ciclismo-van-aert-falha-tour2026-devido-a-lesao-no-cotovelo</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-06-17 17:01</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>😁👋🏼 Jack Grealish, back on the pitch after long injury.</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>injury, injury</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067279561906159707#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-06-17 18:01</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>X:@ManUtd</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Matta has shared a positive update as he progresses in his recovery from a back injury 💪</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>injury, injury</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>https://nitter.net/ManUtd/status/2067296715804180871#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-06-17 19:01</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Atenção, Portugal: Uzbequistão troca de avançados após lesão</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>lesão, lesão</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mundial-2026/uzbequistao/atencao-portugal-uzbequistao-troca-de-avancados-apos-lesao</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Konaté → Real Madrid OFICIAL Jun 18 · 3rd Mourinho signing (after Cucurella + Bernardo Silva)
Free transfer from Liverpool · FRA CB · 27yo · maisfutebol confirmed.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Transfer_Tracker.xlsx
+++ b/Transfer_Tracker.xlsx
@@ -500,7 +500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F324"/>
+  <dimension ref="A1:F339"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -9315,7 +9315,6 @@
       </c>
     </row>
     <row r="324">
-      <c r="A324" t="inlineStr"/>
       <c r="B324" t="inlineStr">
         <is>
           <t>2026-06-17 21:35</t>
@@ -9339,6 +9338,427 @@
       <c r="F324" t="inlineStr">
         <is>
           <t>https://maisfutebol.iol.pt/liga/famalicao/oficial-famalicao-empresta-medio-georgiano-ao-wolfsberger</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>2026-06-17 23:01</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D325" s="2" t="inlineStr">
+        <is>
+          <t>👑🏴󠁧󠁢󠁥󠁮󠁧󠁿 OFFICIAL: Harry Kane, FIFA Man of the Match for England vs Croatia.</t>
+        </is>
+      </c>
+      <c r="E325" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067368832168059216#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>2026-06-17 23:01</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D326" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Famalicão empresta médio georgiano ao Wolfsberger</t>
+        </is>
+      </c>
+      <c r="E326" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F326" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/liga/famalicao/oficial-famalicao-empresta-medio-georgiano-ao-wolfsberger</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>2026-06-17 23:01</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D327" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Derek McInnes é o novo treinador do Rangers</t>
+        </is>
+      </c>
+      <c r="E327" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contratação, novo treinador, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/cronologia/6373897a0cf2254fb2824fe4#OFICIAL: Derek McInnes é o novo treinado</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>2026-06-18 00:01</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D328" s="2" t="inlineStr">
+        <is>
+          <t>🚨🇪🇸 Behind Liverpool surprise deal: €40m for Víctor Muñoz, release clause activated, medical already done in the US.
+Official statement to follow already this week. Big surprise after hijack with Real Madrid getting €20m.
+🎥 Full exclusive story: http://youtu.be/1VtB6MBV3KQ?is=u8-P8bdjJKr6rJnj</t>
+        </is>
+      </c>
+      <c r="E328" s="2" t="inlineStr">
+        <is>
+          <t>deal, release</t>
+        </is>
+      </c>
+      <c r="F328" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067390498231185436#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>2026-06-18 02:01</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D329" s="2" t="inlineStr">
+        <is>
+          <t>🌎🇬🇭 OFFICIAL: Antoine Semenyo, FIFA Man of the Match for Ghana against Panama.</t>
+        </is>
+      </c>
+      <c r="E329" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F329" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067423539020394893#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr"/>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>2026-06-18 12:36</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D330" s="2" t="inlineStr">
+        <is>
+          <t>🚨⚪️ OFFICIAL: Real Madrid confirm Ibrahima Konaté to join on four year deal.
+French defender arrives from Liverpool. 🇫🇷</t>
+        </is>
+      </c>
+      <c r="E330" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, deal, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F330" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067539115046748429#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr"/>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>2026-06-18 12:36</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D331" s="2" t="inlineStr">
+        <is>
+          <t>🚨💣 Víctor Muñoz to Liverpool, it’s all formally sealed as Spanish winger has signed his contract with #LFC valid until June 2032.
+Hijack completed for €40m fee.
+The exclusive story from last night, 100% confirmed.</t>
+        </is>
+      </c>
+      <c r="E331" s="2" t="inlineStr">
+        <is>
+          <t>confirmed, signed</t>
+        </is>
+      </c>
+      <c r="F331" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067502824145945082#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr"/>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>2026-06-18 12:36</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D332" s="2" t="inlineStr">
+        <is>
+          <t>🌎🇨🇴 OFFICIAL: Luis Diaz, FIFA Man of the Match for Colombia vs Uzbekistan.</t>
+        </is>
+      </c>
+      <c r="E332" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F332" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067458464637432056#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr"/>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>2026-06-18 12:36</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>X:@IpswichTown</t>
+        </is>
+      </c>
+      <c r="D333" s="2" t="inlineStr">
+        <is>
+          <t>RT by @IpswichTown: 🤝 The club is delighted to announce that captain Maria Boswell has signed a new deal. 
+Maria joined Town in the summer of 2019 and has now extended her stay in Suffolk for at least another year.</t>
+        </is>
+      </c>
+      <c r="E333" s="2" t="inlineStr">
+        <is>
+          <t>deal, signed, joined</t>
+        </is>
+      </c>
+      <c r="F333" t="inlineStr">
+        <is>
+          <t>https://nitter.net/ITFCWomen/status/2067578083247292810#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr"/>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>2026-06-18 12:36</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>X:@realmadrid</t>
+        </is>
+      </c>
+      <c r="D334" s="2" t="inlineStr">
+        <is>
+          <t>Comunicado Oficial: Konaté.</t>
+        </is>
+      </c>
+      <c r="E334" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F334" t="inlineStr">
+        <is>
+          <t>https://nitter.net/realmadrid/status/2067533778319270351#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr"/>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>2026-06-18 12:36</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D335" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Konaté é o terceiro reforço do Real Madrid</t>
+        </is>
+      </c>
+      <c r="E335" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F335" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/real-madrid/internacional/oficial-konate-e-reforco-do-real-madrid</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr"/>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>2026-06-18 12:36</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D336" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Bruno Langa despede-se do Estrela da Amadora e ruma ao Qarabag</t>
+        </is>
+      </c>
+      <c r="E336" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, contratação, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F336" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/cronologia/6373897a0cf2254fb2824fe4#OFICIAL: Bruno Langa despede-se do Estre</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr"/>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>2026-06-18 12:36</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D337" s="2" t="inlineStr">
+        <is>
+          <t>Escócia: Rangers contrata treinador que liderou o sensacional Hearts</t>
+        </is>
+      </c>
+      <c r="E337" s="2" t="inlineStr">
+        <is>
+          <t>anunciou, chega</t>
+        </is>
+      </c>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/escocia/internacional/escocia-glasgow-rangers-contrata-treinador-que-liderou-o-sensacional-hearts</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr"/>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>2026-06-18 12:36</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D338" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Konaté é o terceiro reforço do Real Madrid</t>
+        </is>
+      </c>
+      <c r="E338" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, chega, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F338" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/real-madrid/internacional/oficial-konate-e-reforco-do-real-madrid</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr"/>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>2026-06-18 12:36</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D339" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Beñat San José é o novo treinador do Rayo Vallecano</t>
+        </is>
+      </c>
+      <c r="E339" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, chega, novo treinador, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F339" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/cronologia/6373897a0cf2254fb2824fe4#OFICIAL: Beñat San José é o novo treinad</t>
         </is>
       </c>
     </row>
@@ -9353,7 +9773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -10487,6 +10907,119 @@
       <c r="F40" t="inlineStr">
         <is>
           <t>https://nitter.net/FabrizioRomano/status/2067313857266172393#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2026-06-17 23:01</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>🚨💣 EXCLUSIVE: Liverpool are set to sign Víctor Muñoz with HIJACK done, HERE WE GO! 🔴🇪🇸
+Newcastle in advanced talks for days but #LFC enter the deal, verbally agree terms with Muñoz and activate €40m release clause.
+All set to be signed and another big surpise. 🧨</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>deal, signed, release, talks, set to sign, HERE WE GO</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067373788480622882#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2026-06-17 23:01</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Liverpool desvia Víctor Muñoz do Newcastle</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>transferência, negocia</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>https://x.com/hashtag/LFC?src=hash&amp;ref_src=twsrc%5Etfw</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2026-06-18 00:01</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Medical already done for Víctor Muñoz. ✅</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>deal, signed, release, talks, set to sign, HERE WE GO</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067385948296425545#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr"/>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2026-06-18 12:36</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>RT by @FabrizioRomano: 🚨💣 EXCLUSIVE: Liverpool are set to sign Víctor Muñoz with HIJACK done, HERE WE GO! 🔴🇪🇸
+Newcastle in advanced talks for days but #LFC enter the deal, verbally agree terms with Muñoz and activate €40m release clause.
+All set to be signed and another big surpise. 🧨</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>deal, signed, release, talks, set to sign, HERE WE GO</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067373788480622882#m</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker refresh Fri 20 Jun · TUR eliminated · Karl Hein → Bremen (already logged) · Bernardo Silva confirmation
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Transfer_Tracker.xlsx
+++ b/Transfer_Tracker.xlsx
@@ -500,7 +500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F339"/>
+  <dimension ref="A1:F436"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -9479,7 +9479,6 @@
       </c>
     </row>
     <row r="330">
-      <c r="A330" t="inlineStr"/>
       <c r="B330" t="inlineStr">
         <is>
           <t>2026-06-18 12:36</t>
@@ -9508,7 +9507,6 @@
       </c>
     </row>
     <row r="331">
-      <c r="A331" t="inlineStr"/>
       <c r="B331" t="inlineStr">
         <is>
           <t>2026-06-18 12:36</t>
@@ -9538,7 +9536,6 @@
       </c>
     </row>
     <row r="332">
-      <c r="A332" t="inlineStr"/>
       <c r="B332" t="inlineStr">
         <is>
           <t>2026-06-18 12:36</t>
@@ -9566,7 +9563,6 @@
       </c>
     </row>
     <row r="333">
-      <c r="A333" t="inlineStr"/>
       <c r="B333" t="inlineStr">
         <is>
           <t>2026-06-18 12:36</t>
@@ -9595,7 +9591,6 @@
       </c>
     </row>
     <row r="334">
-      <c r="A334" t="inlineStr"/>
       <c r="B334" t="inlineStr">
         <is>
           <t>2026-06-18 12:36</t>
@@ -9623,7 +9618,6 @@
       </c>
     </row>
     <row r="335">
-      <c r="A335" t="inlineStr"/>
       <c r="B335" t="inlineStr">
         <is>
           <t>2026-06-18 12:36</t>
@@ -9651,7 +9645,6 @@
       </c>
     </row>
     <row r="336">
-      <c r="A336" t="inlineStr"/>
       <c r="B336" t="inlineStr">
         <is>
           <t>2026-06-18 12:36</t>
@@ -9679,7 +9672,6 @@
       </c>
     </row>
     <row r="337">
-      <c r="A337" t="inlineStr"/>
       <c r="B337" t="inlineStr">
         <is>
           <t>2026-06-18 12:36</t>
@@ -9707,7 +9699,6 @@
       </c>
     </row>
     <row r="338">
-      <c r="A338" t="inlineStr"/>
       <c r="B338" t="inlineStr">
         <is>
           <t>2026-06-18 12:36</t>
@@ -9735,7 +9726,6 @@
       </c>
     </row>
     <row r="339">
-      <c r="A339" t="inlineStr"/>
       <c r="B339" t="inlineStr">
         <is>
           <t>2026-06-18 12:36</t>
@@ -9759,6 +9749,2646 @@
       <c r="F339" t="inlineStr">
         <is>
           <t>https://maisfutebol.iol.pt/cronologia/6373897a0cf2254fb2824fe4#OFICIAL: Beñat San José é o novo treinad</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>2026-06-18 13:01</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>X:@HullCity</t>
+        </is>
+      </c>
+      <c r="D340" s="2" t="inlineStr">
+        <is>
+          <t>Ahead of fixture release tomorrow, the club would like to provide an update on 26/27 memberships...
+Following promotion, we are working with the Premier League on required upgrades before Membership details and sales info can be confirmed.
+More info 🔗 https://www.wearehullcity.co.uk/news/2026/june</t>
+        </is>
+      </c>
+      <c r="E340" s="2" t="inlineStr">
+        <is>
+          <t>confirmed, release</t>
+        </is>
+      </c>
+      <c r="F340" t="inlineStr">
+        <is>
+          <t>https://nitter.net/HullCity/status/2067593196117373122#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>2026-06-18 14:01</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D341" s="2" t="inlineStr">
+        <is>
+          <t>🚨🔴⚪️ EXCLUSIVE: Arsenal sent official bid to Leicester City to get Jeremy Monga deal done.
+16 year old winger keen on joining #AFC and deal moving quickly now with optimism to sign #LCFC talent, seen as huge prospect for the future.
+⏳⌛️</t>
+        </is>
+      </c>
+      <c r="E341" s="2" t="inlineStr">
+        <is>
+          <t>deal, joining</t>
+        </is>
+      </c>
+      <c r="F341" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067591311130055043#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>2026-06-18 14:01</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>X:@BurnleyOfficial</t>
+        </is>
+      </c>
+      <c r="D342" s="2" t="inlineStr">
+        <is>
+          <t>R to @BurnleyOfficial: Read more: https://burnleyfootballclub.com/content/burnley-fc-launch-2026-27-memberships</t>
+        </is>
+      </c>
+      <c r="E342" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F342" t="inlineStr">
+        <is>
+          <t>https://nitter.net/BurnleyOfficial/status/2067602898213585201#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>2026-06-18 14:01</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D343" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Rui Mota assume comando técnico do SV Waldhof Mannheim</t>
+        </is>
+      </c>
+      <c r="E343" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F343" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/made-in/mercado-de-transferencias/oficial-rui-mota-assume-comando-tecnico-do-sv-waldhof-mannheim</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>2026-06-18 15:16</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D344" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Rui Mota assume comando técnico do SV Waldhof Mannheim</t>
+        </is>
+      </c>
+      <c r="E344" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F344" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/made-in/mercado-de-transferencias/oficial-rui-mota-assume-comando-tecnico-do-sv-waldhof-mannheim</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>2026-06-18 15:16</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D345" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Olivier Pantaloni sucede a Claude Puel no comando técnico do Nice</t>
+        </is>
+      </c>
+      <c r="E345" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, contrato, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F345" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/cronologia/6373897a0cf2254fb2824fe4#OFICIAL: Olivier Pantaloni sucede a Clau</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>2026-06-18 15:16</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D346" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: André Ricardo troca o PAOK pelo Lusitânia de Lourosa</t>
+        </is>
+      </c>
+      <c r="E346" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contratação, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F346" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/cronologia/6373897a0cf2254fb2824fe4#OFICIAL: André Ricardo troca o PAOK pelo</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>2026-06-18 16:01</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D347" s="2" t="inlineStr">
+        <is>
+          <t>🚨 OFFICIAL: Neymar Jr to miss Brazil game against Haiti, out of Ancelotti’s squad. 🇧🇷
+No risks taken as Ney Jr returned fo full team training only 24 hours ago, building his best condition.</t>
+        </is>
+      </c>
+      <c r="E347" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, 🚨 OFFICIAL, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F347" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067627190414405962#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:02</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>X:@SunderlandAFC</t>
+        </is>
+      </c>
+      <c r="D348" s="2" t="inlineStr">
+        <is>
+          <t>RT by @SunderlandAFC: Harrison Jones has joined Peterborough United on a permanent deal.
+All at Sunderland wish Harrison the best of luck with the next steps of his career ❤️</t>
+        </is>
+      </c>
+      <c r="E348" s="2" t="inlineStr">
+        <is>
+          <t>deal, joined</t>
+        </is>
+      </c>
+      <c r="F348" t="inlineStr">
+        <is>
+          <t>https://nitter.net/AcademyOfLight/status/2067639726287597971#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:02</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D349" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Milan garante primeiro «reforço» para Amorim</t>
+        </is>
+      </c>
+      <c r="E349" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F349" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/internacional/italia/oficial-milan-garante-primeiro-reforco-para-amorim</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:02</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D350" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Afonso Moreira troca Lyon pelo Bayer Leverkusen</t>
+        </is>
+      </c>
+      <c r="E350" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, transferência, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F350" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/made-in/bayer-leverkusen/oficial-afonso-moreira-troca-lyon-pelo-bayer-leverkusen</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:02</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D351" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Milan garante primeiro «reforço» para Amorim</t>
+        </is>
+      </c>
+      <c r="E351" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, contrato, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F351" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/internacional/italia/oficial-milan-garante-primeiro-reforco-para-amorim</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:02</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D352" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Afonso Moreira troca Lyon pelo Bayer Leverkusen</t>
+        </is>
+      </c>
+      <c r="E352" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, contrato, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F352" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/made-in/bayer-leverkusen/oficial-afonso-moreira-troca-lyon-pelo-bayer-leverkusen</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:02</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D353" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Liverpool · Carter Pinnington — Transfer Out · - West Brom</t>
+        </is>
+      </c>
+      <c r="E353" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F353" t="inlineStr">
+        <is>
+          <t>https://www.liverpoolfc.com/news/carter-pinnington-joins-west-bromwich-albion?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:02</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D354" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Sunderland · Milan Aleksic — loan-out · - Partizan Belgrade</t>
+        </is>
+      </c>
+      <c r="E354" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, loan, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F354" t="inlineStr">
+        <is>
+          <t>https://www.safc.com/news/2026/june/18/milan-aleksi--joins-partizan-belgrade-on-loan/?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>2026-06-18 18:01</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D355" s="2" t="inlineStr">
+        <is>
+          <t>🚨 OFFICIAL: Messi family statement. ❗️
+"The Messi family informs that Jorge Messi is currently going through a health situation.
+"At this time, he is under medical supervision, recovering and progressing favorably within the condition he is experiencing.
+"In light of the reports, rumors, and spec</t>
+        </is>
+      </c>
+      <c r="E355" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, thank you, rumor, rumor, 🚨 OFFICIAL, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F355" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067653899952042464#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>2026-06-18 18:01</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D356" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Moreno volta ao ativo e é o novo treinador do Felgueiras</t>
+        </is>
+      </c>
+      <c r="E356" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, contrato, novo treinador, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F356" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/ii-liga/felgueiras/oficial-moreno-volta-ao-ativo-e-e-o-novo-treinador-do-felgueiras</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>2026-06-18 18:01</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D357" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Chelsea · Jimmy-Jay Morgan — Transfer Out · - West Brom</t>
+        </is>
+      </c>
+      <c r="E357" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F357" t="inlineStr">
+        <is>
+          <t>https://www.chelseafc.com/en/news/article/jimmy-jay-morgan-joins-west-bromwich-albion?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>2026-06-18 18:01</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D358" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Sunderland · Harrison Jones — Transfer Out · - Peterborough</t>
+        </is>
+      </c>
+      <c r="E358" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F358" t="inlineStr">
+        <is>
+          <t>https://www.safc.com/news/2026/june/18/harrison-jones-joins-peterborough-united/?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>2026-06-18 19:01</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D359" s="2" t="inlineStr">
+        <is>
+          <t>🚨⚪️ OFFICIAL: Jan Paul van Hecke joins Tottenham on £52m deal plus 20% sell-on clause from Brighton.
+“Joining Spurs is a dream come true for me”, says van Hecke. 💭🇳🇱</t>
+        </is>
+      </c>
+      <c r="E359" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, deal, joins, joining, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F359" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067678186930860327#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>2026-06-18 19:01</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D360" s="2" t="inlineStr">
+        <is>
+          <t>RT by @FabrizioRomano: 🚨 OFFICIAL: Víctor Muñoz joins Liverpool, exclusive story confirmed. 🔴🇪🇸
+€40m release clause triggered from Osasuna, contract until June 2032 for Muñoz.
+Real Madrid receive around €20m.</t>
+        </is>
+      </c>
+      <c r="E360" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, confirmed, joins, release, 🚨 OFFICIAL, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F360" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067669183530188845#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>2026-06-18 19:01</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D361" s="2" t="inlineStr">
+        <is>
+          <t>🚨⚫️🔵 OFFICIAL: Cristian Chivu signs new deal at Inter valid until June 2028, as expected.</t>
+        </is>
+      </c>
+      <c r="E361" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, deal, signs, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F361" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067669277776150870#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>2026-06-18 19:01</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D362" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Jéssica Silva reforça o Galatasaray</t>
+        </is>
+      </c>
+      <c r="E362" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F362" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/transferencias/jessica-silva/oficial-jessica-silva-reforca-o-galatasaray</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>2026-06-18 19:01</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D363" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Moreno volta ao ativo e é o novo treinador do Felgueiras</t>
+        </is>
+      </c>
+      <c r="E363" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, novo treinador, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F363" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/ii-liga/felgueiras/oficial-moreno-volta-ao-ativo-e-e-o-novo-treinador-do-felgueiras</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>2026-06-18 19:01</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D364" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Jéssica Silva reforça o Galatasaray</t>
+        </is>
+      </c>
+      <c r="E364" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, contrato, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F364" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/transferencias/jessica-silva/oficial-jessica-silva-reforca-o-galatasaray</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>2026-06-18 19:01</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D365" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Brighton &amp; Hove Albion · Jan Paul van Hecke — Transfer Out · - Spurs</t>
+        </is>
+      </c>
+      <c r="E365" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F365" t="inlineStr">
+        <is>
+          <t>https://www.brightonandhovealbion.com/media-article/mft-transfer-news-jan-paul-van-hecke-tottenham-hotspur-june-2026?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=tra</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>2026-06-18 19:01</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D366" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Liverpool · Victor Munoz — Transfer In · - Osasuna</t>
+        </is>
+      </c>
+      <c r="E366" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F366" t="inlineStr">
+        <is>
+          <t>https://www.liverpoolfc.com/news/liverpool-agree-deal-sign-spain-forward-victor-munoz?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>2026-06-18 19:01</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D367" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Tottenham Hotspur · Jan Paul van Hecke — Transfer In · - Brighton</t>
+        </is>
+      </c>
+      <c r="E367" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F367" t="inlineStr">
+        <is>
+          <t>https://www.tottenhamhotspur.com/news/1073998/van-hecke-joins-from-brighton?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>2026-06-18 20:01</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D368" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Vedat Muriqi regressa ao Fenerbahçe para reforçar o ataque</t>
+        </is>
+      </c>
+      <c r="E368" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, regressa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F368" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/internacional/turquia/oficial-vedat-muriqi-regressa-ao-fenerbahce-para-reforcar-o-ataque</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>2026-06-18 20:01</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D369" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Ismail Kartal é o novo treinador do Fenerbahçe</t>
+        </is>
+      </c>
+      <c r="E369" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, novo treinador, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F369" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/internacional/turquia/oficial-ismail-kartal-e-o-novo-treinador-do-fenerbahce</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>2026-06-18 20:01</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D370" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Jan Paul van Hecke reforça a defesa do Tottenham</t>
+        </is>
+      </c>
+      <c r="E370" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F370" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/transferencias/jan-paul-van-hecke/oficial-jan-paul-van-hecke-reforca-a-defesa-do-tottenham</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>2026-06-18 20:01</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D371" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Cristian Chivu renova com o Inter até 2028</t>
+        </is>
+      </c>
+      <c r="E371" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F371" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/italia/christian-chivu/oficial-christian-chivu-renova-com-o-inter-ate-2028</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>2026-06-18 20:01</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D372" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Víctor Muñoz é reforço do Liverpool</t>
+        </is>
+      </c>
+      <c r="E372" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F372" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/transferencias/victor-munoz/oficial-victor-munoz-e-reforco-do-liverpool</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>2026-06-18 20:01</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D373" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Vedat Muriqi regressa ao Fenerbahçe para reforçar o ataque</t>
+        </is>
+      </c>
+      <c r="E373" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, contrato, regressa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F373" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/internacional/turquia/oficial-vedat-muriqi-regressa-ao-fenerbahce-para-reforcar-o-ataque</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>2026-06-18 20:01</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D374" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Ismail Kartal é o novo treinador do Fenerbahçe</t>
+        </is>
+      </c>
+      <c r="E374" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, contrato, novo treinador, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F374" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/internacional/turquia/oficial-ismail-kartal-e-o-novo-treinador-do-fenerbahce</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>2026-06-18 21:01</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D375" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Fahem Yahia Benaissa deixa o Casa Pia e assina pelo Mantova</t>
+        </is>
+      </c>
+      <c r="E375" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F375" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/liga/casa-pia/oficial-fahem-yahia-benaissa-deixa-o-casa-pia-e-assina-pelo-mantova</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>2026-06-18 21:01</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D376" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Artur Jorge recebe reforço para a defesa</t>
+        </is>
+      </c>
+      <c r="E376" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contratação, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F376" t="inlineStr">
+        <is>
+          <t>https://t.co/ESVX0dEOnj</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>2026-06-18 22:08</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D377" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Arruabarrena é o novo treinador do Boca Juniors</t>
+        </is>
+      </c>
+      <c r="E377" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, novo treinador, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F377" t="inlineStr">
+        <is>
+          <t>https://t.co/UeXQ5swAqa</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>2026-06-18 22:08</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D378" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Tim Payne, fenómeno das redes sociais, «muda-se» para o Paraguai</t>
+        </is>
+      </c>
+      <c r="E378" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, transferência, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F378" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/internacional/tim-payne/oficial-tim-payne-fenomeno-das-redes-sociais-muda-se-para-o-paraguai</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>2026-06-18 23:11</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D379" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Benfica renova contrato com avançado de 18 anos</t>
+        </is>
+      </c>
+      <c r="E379" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, contrato, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F379" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mundial-2026/mundial2026/oficial-benfica-renova-contrato-com-avancado-de-18-anos</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>2026-06-18 23:11</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D380" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Tim Payne, fenómeno das redes sociais, «muda-se» para o Paraguai</t>
+        </is>
+      </c>
+      <c r="E380" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/internacional/tim-payne/oficial-tim-payne-fenomeno-das-redes-sociais-muda-se-para-o-paraguai</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>2026-06-18 23:11</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D381" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Benfica renova contrato com avançado de 18 anos</t>
+        </is>
+      </c>
+      <c r="E381" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, contrato, novo treinador, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F381" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mundial-2026/mundial2026/oficial-benfica-renova-contrato-com-avancado-de-18-anos</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>2026-06-19 12:48</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D382" s="2" t="inlineStr">
+        <is>
+          <t>🚨🇸🇦 Bersant Celina joins Al Ettifaq in Saudi Pro League on a three year deal, agreed and sealed today.</t>
+        </is>
+      </c>
+      <c r="E382" s="2" t="inlineStr">
+        <is>
+          <t>agreed, deal, joins</t>
+        </is>
+      </c>
+      <c r="F382" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067853586218815690#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>2026-06-19 12:48</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D383" s="2" t="inlineStr">
+        <is>
+          <t>🌎🇲🇽 OFFICIAL: Luis Romo wins FIFA Man of the Match for Mexico-South Korea.</t>
+        </is>
+      </c>
+      <c r="E383" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F383" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067809279155835203#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>2026-06-19 12:48</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D384" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Mateo Flores é reforço do Arouca</t>
+        </is>
+      </c>
+      <c r="E384" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F384" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/liga/arouca/oficial-mateo-flores-e-reforco-do-arouca</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>2026-06-19 12:48</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D385" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Renato Gaúcho deixa o Vasco da Gama</t>
+        </is>
+      </c>
+      <c r="E385" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, deixa, chega, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F385" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/brasil/transferencias/oficial-renato-gaucho-deixa-o-vasco-da-gama</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>2026-06-19 12:48</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D386" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Mateo Flores é reforço do Arouca</t>
+        </is>
+      </c>
+      <c r="E386" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contratação, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F386" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/liga/arouca/oficial-mateo-flores-e-reforco-do-arouca</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>2026-06-19 12:48</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D387" s="2" t="inlineStr">
+        <is>
+          <t>Benfica tenta desviar jovem central brasileiro que estava a caminho do Nápoles</t>
+        </is>
+      </c>
+      <c r="E387" s="2" t="inlineStr">
+        <is>
+          <t>anunciou, contratação</t>
+        </is>
+      </c>
+      <c r="F387" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/benfica/transferencias/benfica-tenta-desviar-jovem-central-brasileiro-que-estava-a-caminho-do-napoles</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>2026-06-19 12:48</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D388" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Pablo Maffeo é reforço do Olympiacos</t>
+        </is>
+      </c>
+      <c r="E388" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contratação, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F388" t="inlineStr">
+        <is>
+          <t>https://t.co/1CwPKySH8Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>2026-06-19 12:48</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D389" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Tommaso Baldanzi regressa ao Génova</t>
+        </is>
+      </c>
+      <c r="E389" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, regressa, empréstimo, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F389" t="inlineStr">
+        <is>
+          <t>https://t.co/yC4ovyeaTt</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>2026-06-19 12:48</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D390" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Renato Gaúcho deixa o Vasco da Gama</t>
+        </is>
+      </c>
+      <c r="E390" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, deixa, interessado em, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F390" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/brasil/transferencias/oficial-renato-gaucho-deixa-o-vasco-da-gama</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>2026-06-19 13:00</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D391" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Benfica renova contrato com avançado de 18 anos</t>
+        </is>
+      </c>
+      <c r="E391" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, contrato, novo treinador, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F391" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mundial-2026/mundial2026/oficial-benfica-renova-contrato-com-avancado-de-18-anos</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>2026-06-19 13:00</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D392" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Vedat Muriqi regressa ao Fenerbahçe para reforçar o ataque</t>
+        </is>
+      </c>
+      <c r="E392" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, contrato, regressa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F392" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/internacional/turquia/oficial-vedat-muriqi-regressa-ao-fenerbahce-para-reforcar-o-ataque</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>2026-06-19 13:00</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D393" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Milan garante primeiro «reforço» para Amorim</t>
+        </is>
+      </c>
+      <c r="E393" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, contrato, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F393" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/internacional/italia/oficial-milan-garante-primeiro-reforco-para-amorim</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>2026-06-19 13:00</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D394" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Brentford · Jannik Schuster — Transfer In · - RB Salzburg</t>
+        </is>
+      </c>
+      <c r="E394" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F394" t="inlineStr">
+        <is>
+          <t>https://www.brentfordfc.com/en/news/article/first-team-brentford-jannik-schuster-red-bull-salzburg-transfer?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-wat</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>2026-06-19 13:00</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D395" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Fulham · Charlie Robinson — Released</t>
+        </is>
+      </c>
+      <c r="E395" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F395" t="inlineStr">
+        <is>
+          <t>https://www.fulhamfc.com/news/2026/june/08/player-contract-updates/?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>2026-06-19 13:00</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D396" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Liverpool · Kareem Ahmed — Released</t>
+        </is>
+      </c>
+      <c r="E396" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F396" t="inlineStr">
+        <is>
+          <t>https://www.liverpoolfc.com/news/liverpool-confirm-premier-league-retained-list?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>2026-06-19 13:00</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D397" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Newcastle · Max Thompson — Released</t>
+        </is>
+      </c>
+      <c r="E397" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F397" t="inlineStr">
+        <is>
+          <t>https://www.newcastleunited.com/en/news/newcastle-united-confirm-mens-first-team-retained-list?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>2026-06-19 13:00</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D398" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Tottenham Hotspur · Jan Paul van Hecke — Transfer In · - Brighton</t>
+        </is>
+      </c>
+      <c r="E398" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F398" t="inlineStr">
+        <is>
+          <t>https://www.tottenhamhotspur.com/news/1073998/van-hecke-joins-from-brighton?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:01</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D399" s="2" t="inlineStr">
+        <is>
+          <t>Benfica prestes a fechar jovem central brasileiro que estava a caminho do Nápoles</t>
+        </is>
+      </c>
+      <c r="E399" s="2" t="inlineStr">
+        <is>
+          <t>anunciou, contratação</t>
+        </is>
+      </c>
+      <c r="F399" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/benfica/transferencias/benfica-tenta-desviar-jovem-central-brasileiro-que-estava-a-caminho-do-napoles</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:01</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D400" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Milan garante primeiro «reforço» para Amorim</t>
+        </is>
+      </c>
+      <c r="E400" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, contrato, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F400" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/internacional/italia/oficial-milan-garante-primeiro-reforco-para-amorim</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:01</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D401" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Arsenal · Jakub Kiwior — Transfer Out · Porto</t>
+        </is>
+      </c>
+      <c r="E401" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F401" t="inlineStr">
+        <is>
+          <t>https://www.arsenal.com/news/loan-watch-sagoe-jr-flying-kafaji-reaches-final?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>2026-06-19 15:01</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D402" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Brighton &amp; Hove Albion · Joel Veltman — Released</t>
+        </is>
+      </c>
+      <c r="E402" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F402" t="inlineStr">
+        <is>
+          <t>https://www.premierleague.com/en/news/4672506</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>2026-06-19 15:01</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D403" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Sunderland · Bertrand Traore — Released</t>
+        </is>
+      </c>
+      <c r="E403" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F403" t="inlineStr">
+        <is>
+          <t>https://www.safc.com/news/2026/june/10/sunderland-afc-announce-retained-list-for-2026-27/?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>2026-06-19 16:01</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>X:@IpswichTown</t>
+        </is>
+      </c>
+      <c r="D404" s="2" t="inlineStr">
+        <is>
+          <t>RT by @IpswichTown: 🤝 Ipswich Town Women is pleased to announce that Leah Mitchell has signed a new two-year deal with the club.</t>
+        </is>
+      </c>
+      <c r="E404" s="2" t="inlineStr">
+        <is>
+          <t>deal, signed</t>
+        </is>
+      </c>
+      <c r="F404" t="inlineStr">
+        <is>
+          <t>https://nitter.net/ITFCWomen/status/2066521109642846651#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>2026-06-19 16:01</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D405" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Newcastle · Ewen Jaouen — Transfer In · - Reims</t>
+        </is>
+      </c>
+      <c r="E405" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F405" t="inlineStr">
+        <is>
+          <t>https://www.newcastleunited.com/en/news/ewen-jaouen-signs-for-newcastle-united?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>2026-06-19 16:01</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D406" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Tottenham Hotspur · Andy Robertson — Transfer In</t>
+        </is>
+      </c>
+      <c r="E406" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F406" t="inlineStr">
+        <is>
+          <t>https://www.tottenhamhotspur.com/news/1071931/robertson-signing-secured?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>2026-06-19 17:04</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>X:@miseleccionmx</t>
+        </is>
+      </c>
+      <c r="D407" s="2" t="inlineStr">
+        <is>
+          <t>#SomosMéxico y también somos oficialmente líderes de grupo. 😌🇲🇽
+A cerrar la Fase de Grupos de la mejor manera. ¡Y también nos vemos en la siguiente fase en nuestra casa! 💚🤍❤️
+¡Hagamos pesar el Estadio Ciudad de México todos juntos, Incondicionales! 🔥</t>
+        </is>
+      </c>
+      <c r="E407" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIALMENTE, OFICIALMENTE</t>
+        </is>
+      </c>
+      <c r="F407" t="inlineStr">
+        <is>
+          <t>https://nitter.net/miseleccionmx/status/2068008390312235325#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>2026-06-19 18:01</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D408" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Bruno Baltazar deixa o Radomiak da Polónia</t>
+        </is>
+      </c>
+      <c r="E408" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F408" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/made-in/radomiak-radom/oficial-bruno-baltazar-deixa-o-radomiak-da-polonia</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>2026-06-19 18:01</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D409" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Bruno Baltazar deixa o Radomiak da Polónia</t>
+        </is>
+      </c>
+      <c r="E409" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F409" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/made-in/radomiak-radom/oficial-bruno-baltazar-deixa-o-radomiak-da-polonia</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>2026-06-19 18:01</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D410" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Ismail Kartal é o novo treinador do Fenerbahçe</t>
+        </is>
+      </c>
+      <c r="E410" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, novo treinador, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F410" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/internacional/turquia/oficial-ismail-kartal-e-o-novo-treinador-do-fenerbahce</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>2026-06-19 19:02</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>X:@BurnleyOfficial</t>
+        </is>
+      </c>
+      <c r="D411" s="2" t="inlineStr">
+        <is>
+          <t>R to @BurnleyOfficial: Read more: https://burnleyfootballclub.com/content/burnley-fc-launch-2026-27-memberships</t>
+        </is>
+      </c>
+      <c r="E411" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F411" t="inlineStr">
+        <is>
+          <t>https://nitter.net/BurnleyOfficial/status/2067602898213585201#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>2026-06-19 19:02</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>X:@realmadrid</t>
+        </is>
+      </c>
+      <c r="D412" s="2" t="inlineStr">
+        <is>
+          <t>Comunicado Oficial: Sergio Rodríguez.</t>
+        </is>
+      </c>
+      <c r="E412" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F412" t="inlineStr">
+        <is>
+          <t>https://nitter.net/realmadrid/status/2068031059862909396#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>2026-06-19 19:02</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D413" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Ana Dias é reforço do Sporting</t>
+        </is>
+      </c>
+      <c r="E413" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, regressa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F413" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/futebol-feminino/transferencias/oficial-ana-dias-e-reforco-do-sporting</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>2026-06-19 19:02</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D414" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Bruno Pinheiro regressa à Liga para treinar o Académico Viseu</t>
+        </is>
+      </c>
+      <c r="E414" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, regressa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F414" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/liga/academico-viseu/oficial-bruno-pinheiro-regressa-a-liga-para-treinar-o-academico-viseu</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>2026-06-19 19:02</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D415" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Ana Dias é reforço do Sporting</t>
+        </is>
+      </c>
+      <c r="E415" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, chega, acordo verbal, deverá, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F415" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/futebol-feminino/transferencias/oficial-ana-dias-e-reforco-do-sporting</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>2026-06-19 19:02</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D416" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Bruno Pinheiro regressa à Liga para treinar o Académico Viseu</t>
+        </is>
+      </c>
+      <c r="E416" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, chega, regressa, acordo verbal, deverá, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F416" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/liga/academico-viseu/oficial-bruno-pinheiro-regressa-a-liga-para-treinar-o-academico-viseu</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>2026-06-19 19:02</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D417" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Newcastle · Ewen Jaouen — Transfer In · - Reims</t>
+        </is>
+      </c>
+      <c r="E417" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F417" t="inlineStr">
+        <is>
+          <t>https://www.newcastleunited.com/en/news/ewen-jaouen-signs-for-newcastle-united?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>2026-06-19 20:03</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D418" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Sp. Braga contrata Gabriel Silva ao Santa Clara</t>
+        </is>
+      </c>
+      <c r="E418" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F418" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/liga/sp-braga/oficial-sp-braga-contrata-gabriel-silva-ao-santa-clara</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>2026-06-19 20:03</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D419" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Sp. Braga contrata Gabriel Silva ao Santa Clara</t>
+        </is>
+      </c>
+      <c r="E419" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, contratação, contrato, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F419" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/liga/sp-braga/oficial-sp-braga-contrata-gabriel-silva-ao-santa-clara</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>2026-06-19 22:01</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D420" s="2" t="inlineStr">
+        <is>
+          <t>🚨🇺🇸 OFFICIAL: USA advance to FIFA World Cup Round of 32!</t>
+        </is>
+      </c>
+      <c r="E420" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F420" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2068075601169133915#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>2026-06-19 22:01</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>X:@David_Ornstein</t>
+        </is>
+      </c>
+      <c r="D421" s="2" t="inlineStr">
+        <is>
+          <t>🚨 Marcus Rashford deal at Man Utd includes £40m clause for all clubs bar #MCFC &amp; #LFC. €30m buy option in Barcelona loan expired yesterday. If returns to #MUFC 28yo’s preference is to honour contract (2028) rather than join another PL side @TheAthleticFC https://www.nytimes.com/athletic/7361885/2026</t>
+        </is>
+      </c>
+      <c r="E421" s="2" t="inlineStr">
+        <is>
+          <t>deal, loan</t>
+        </is>
+      </c>
+      <c r="F421" t="inlineStr">
+        <is>
+          <t>https://nitter.net/David_Ornstein/status/2066800458220359737#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>2026-06-19 22:01</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D422" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Tim Payne, fenómeno das redes sociais, «muda-se» para o Paraguai</t>
+        </is>
+      </c>
+      <c r="E422" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, transferência, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F422" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/internacional/tim-payne/oficial-tim-payne-fenomeno-das-redes-sociais-muda-se-para-o-paraguai</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>2026-06-19 23:01</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D423" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: João Resende reforça o Farense</t>
+        </is>
+      </c>
+      <c r="E423" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, chega, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F423" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DZx0LZtDNSC/?utm_source=ig_embed&amp;utm_campaign=loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>2026-06-19 23:01</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D424" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Jordan van der Gaag renova com UD Leiria</t>
+        </is>
+      </c>
+      <c r="E424" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F424" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://maisfutebol.iol.pt/cronologia/6373897a0cf2254fb2824fe4#OFICIAL: Jordan van der Gaag renova com </t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:01</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D425" s="2" t="inlineStr">
+        <is>
+          <t>🚨🇧🇷 OFFICIAL: Endrick has been benched again.
+Cunha, Vini Jr and Raphinha upfront for Brazil.</t>
+        </is>
+      </c>
+      <c r="E425" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F425" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2068110198321947044#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>2026-06-20 01:02</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D426" s="2" t="inlineStr">
+        <is>
+          <t>🌎🇲🇦 OFFICIAL: Ismael Saibari wins FIFA Man of the Match Award for Morocco-Scotland.</t>
+        </is>
+      </c>
+      <c r="E426" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F426" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2068129637771681947#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>2026-06-20 02:01</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D427" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Ipswich · Leon Ayinde — Transfer Out · - Doncaster</t>
+        </is>
+      </c>
+      <c r="E427" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F427" t="inlineStr">
+        <is>
+          <t>https://www.itfc.co.uk/news/2026/may/20/leon-ayinde-to-join-doncaster/?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>2026-06-20 03:01</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D428" s="2" t="inlineStr">
+        <is>
+          <t>🚨🇧🇷 OFFICIAL: Vini Jr wins FIFA Man of the Match for Brazil vs Haiti.
+Back to back. ⭐️⭐️</t>
+        </is>
+      </c>
+      <c r="E428" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F428" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2068164563581784161#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>2026-06-20 03:01</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D429" s="2" t="inlineStr">
+        <is>
+          <t>🚨🇭🇹 OFFICIAL: Haiti have been eliminated from the 2026 World Cup.</t>
+        </is>
+      </c>
+      <c r="E429" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F429" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2068162531781202101#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>2026-06-20 03:01</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D430" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Chelsea · Jimmy-Jay Morgan — Transfer Out · - West Brom</t>
+        </is>
+      </c>
+      <c r="E430" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F430" t="inlineStr">
+        <is>
+          <t>https://www.chelseafc.com/en/news/article/jimmy-jay-morgan-joins-west-bromwich-albion?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>2026-06-20 04:01</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D431" s="2" t="inlineStr">
+        <is>
+          <t>🚨💣 OFFICIAL: Neymar Jr will be called up for Brazil next game against Scotland. 🇧🇷
+“Neymar will train individually tomorrow, then Sunday back training with the team and then called up against Scotland”, announces Carlo Ancelotti after Brazil win against Haiti.</t>
+        </is>
+      </c>
+      <c r="E431" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F431" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2068176414910599435#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>2026-06-20 05:00</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D432" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Bruno Baltazar deixa o Radomiak da Polónia</t>
+        </is>
+      </c>
+      <c r="E432" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F432" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/made-in/radomiak-radom/oficial-bruno-baltazar-deixa-o-radomiak-da-polonia</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>2026-06-20 06:00</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D433" s="2" t="inlineStr">
+        <is>
+          <t>🚨⛔️ OFFICIAL: Turkiye have been ELIMINATED from the 2026 World Cup.
+Verdict after 2 games at group stages, 0 goals scored and 2 defeats. ❌</t>
+        </is>
+      </c>
+      <c r="E433" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F433" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2068198706113851671#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>2026-06-20 06:00</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D434" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Arsenal · Karl Hein — Transfer Out · Werder Bremen</t>
+        </is>
+      </c>
+      <c r="E434" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F434" t="inlineStr">
+        <is>
+          <t>https://www.arsenal.com/news/karl-hein-join-werder-bremen-permanent-deal?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr"/>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>2026-06-20 06:00</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D435" s="2" t="inlineStr">
+        <is>
+          <t>🚨⛔️ OFFICIAL: Turkiye have been ELIMINATED from the 2026 World Cup.
+Verdict after 2 games at group stages, 0 goals scored and 2 defeats. ❌</t>
+        </is>
+      </c>
+      <c r="E435" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F435" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2068198706113851671#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr"/>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>2026-06-20 06:00</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D436" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Arsenal · Karl Hein — Transfer Out · Werder Bremen</t>
+        </is>
+      </c>
+      <c r="E436" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F436" t="inlineStr">
+        <is>
+          <t>https://www.arsenal.com/news/karl-hein-join-werder-bremen-permanent-deal?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
         </is>
       </c>
     </row>
@@ -9773,7 +12403,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F44"/>
+  <dimension ref="A1:F59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -10994,7 +13624,6 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr"/>
       <c r="B44" t="inlineStr">
         <is>
           <t>2026-06-18 12:36</t>
@@ -11020,6 +13649,423 @@
       <c r="F44" t="inlineStr">
         <is>
           <t>https://nitter.net/FabrizioRomano/status/2067373788480622882#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2026-06-18 13:01</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>🚨🇵🇹 EXCL: Rennes have agreed deal to sign Gonçalo Oliveira from Benfica, here we go!
+€3.5m transfer fee for the captain of Benfica B and U21 international with Portugal. 🔴⚫️</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>agreed, deal, HERE WE GO, Here we go!, Here We Go, here we go</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067585549884346866#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:02</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Afonso Moreira has joined Bayer Leverkusen on €32m deal from OL, confirmed. 🔴⚫️✍🏻</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>confirmed, deal, joined, HERE WE GO, Here we go!, Here We Go</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067648855508664555#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:02</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>RT by @FabrizioRomano: 🚨 BREAKING: Ismael Saibari to FC Bayern, HERE WE GO! Deal sealed 🔴⚪️🇲🇦
+Exactly two weeks after exclusive story on Bayern in talks for surprise move, Saibari joins the German champions.
+€55m fee to PSV Eindhoven, medical in USA and then official. All done. ✅</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>deal, joins, talks, HERE WE GO, Here we go!, Here We Go</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2066448878837121047#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:02</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>🚨🔵⚪️ EXCL: Strasbourg agree deal to sign Swedish talent Benjamin Brantlind, here we go!
+Deal done with IFK Gothenburg as many clubs were in the race but the player has finally chosen Strasbourg and the BlueCo project as his next destination. 🇸🇪</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>deal, HERE WE GO, Here we go!, Here We Go, here we go</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067642930756489706#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>2026-06-18 18:01</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Here we go! Tonight Alphonso Davies plays his first FIFA World Cup™️ match on home soil. Will be a historic night in front of the Canadian fans. Update powered by @McDonalds</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>HERE WE GO, Here we go!, Here We Go, here we go</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067663930948755464#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>2026-06-18 19:01</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>✅🔥🔴 #LFC</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>deal, signed, release, talks, set to sign, HERE WE GO</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067668839374958739#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>2026-06-18 22:08</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>🚨🔴⚪️ Mika Marmol to Feyenoord, here we go! Agreement done on a contract until June 2030 with Dutch club. 🇳🇱
+Marmol will sign soon, as @FeyenoordTm reported.</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>HERE WE GO, Here we go!, Here We Go, here we go</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067715869828956338#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2026-06-18 23:11</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Allegri a caminho do Nápoles</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>contrato, deverá</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/cronologia/6373897a0cf2254fb2824fe4#Allegri a caminho do Nápoles</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2026-06-19 12:48</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>🚨🇪🇨 EXCL: Inter Miami agree deal to sign Fricio Caicedo as new centre back, here we go!
+Deal in place for 2008 born centre back who was close to joining Royal Antwerp… and now goes Inter Miami.
+Hijack done.</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>deal, joining, HERE WE GO, Here we go!, Here We Go, here we go</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067926113787994172#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2026-06-19 18:01</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>🚨🔵🔴 EXCLUSIVE: Barcelona reach verbal agreement to sign 2007 born winger Josué Caicedo from LDU Quito, here we go!
+Deal in place for Barcelona B team, loan with option to buy that could turn into obligation — fee around €2.5m.
+Another Ecuadorian talent to Europe. 🇪🇨</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>deal, loan, verbal agreement, HERE WE GO, Here we go!, Here We Go</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2068028220427976922#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>2026-06-19 18:01</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>🚨🔵⚪️ Como have sealed Kaiki deal with Cruzeiro as new left back, here we go! 🇧🇷
+All resolved on payment terms and details. Kaiki joins on €14m deal, loan with obligation to buy.</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>deal, joins, loan, HERE WE GO, Here we go!, Here We Go</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2068016681868304516#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>2026-06-19 18:01</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>X:@ManCity</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Bernardo Silva is set to join Real Madrid after leaving City this summer.
+🔗 http://mancity.co/BernardoRM</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>leaving, set to join</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>https://nitter.net/ManCity/status/2067182089208844337#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>2026-06-19 19:02</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>X:@ManCity</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Bernardo Silva is set to join Real Madrid after leaving City this summer.
+🔗 http://mancity.co/BernardoRM</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>leaving, set to join</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>https://nitter.net/ManCity/status/2067182089208844337#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>2026-06-19 19:02</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>X:@USMNT</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>Here we go!</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>HERE WE GO, Here we go!, Here We Go, here we go</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>https://nitter.net/USMNT/status/2068036383403597915#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>2026-06-19 19:02</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>Barcelona avança por jovem promessa equatoriana</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>chega, acordo verbal, deverá</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>https://t.co/dI7cju62u1</t>
         </is>
       </c>
     </row>
@@ -11034,7 +14080,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -11650,6 +14696,340 @@
       <c r="F22" t="inlineStr">
         <is>
           <t>https://maisfutebol.iol.pt/mundial-2026/uzbequistao/atencao-portugal-uzbequistao-troca-de-avancados-apos-lesao</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-06-19 00:11</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>X:@CanadaSoccerEN</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>RT by @CanadaSoccerEN: Nathan Saliba scores a free kick and honours Ismaël Koné following the injury.
+#FIFAWorldCup</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>injury, injury</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>https://nitter.net/TSN_Sports/status/2067751507156431287#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-06-19 01:05</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Canada makes it 6 against Qatar! 🌎🇨🇦
+Thoughts with Ismael Kone who suffered a bad injury.
+Who’s been your Man of the Match?</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>injury, injury</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067759694383374764#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-06-19 01:05</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>VÍDEO: jogador do Canadá sofre lesão arrepiante e diz adeus ao Mundial</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>lesão, lesão</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mundial-2026/canada/video-jogador-do-canada-sofre-lesao-arrepiante-e-diz-adeus-ao-mundial</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-06-19 03:01</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>🚨🇨🇦 Understand Canada midfielder Ismael Koné has suffered fractured fibula and tibia fracture as well.
+He’s now in the hospital with his mother Suzanne, supporting ahead of surgery.
+Koné could be out for 4-5 months, World Cup over.
+Madibo went to apologize in dressing room.</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>out for</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067786768838017031#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-06-19 12:48</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>X:@afcbournemouth</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Our 2026/27 fixtures will be announced this morning 🙌
+Which games are you looking out for? 👀</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>out for</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>https://nitter.net/afcbournemouth/status/2067885971652174209#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-06-19 12:48</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>De Los Angeles a Toronto: os imponentes estádios que ficaram de fora do Mundial 2026</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>fora do mundial, fora do mundial</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mundial-2026/mundial2026/de-los-angeles-a-toronto-os-imponentes-estadios-que-ficaram-fora-do-mundial-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-06-19 12:48</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Selecionador do Canadá reage à lesão de Koné: «Ouvimos o osso a partir»</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>lesão, lesão</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mundial-2026/mundial2026/selecionador-do-canada-reage-a-lesao-de-kone-ouvimos-o-osso-a-partir</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-06-19 16:01</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>X:@NUFC</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Tino Livramento has withdrawn from @England's #FIFAWorldCup 2026 squad. 
+The 23-year-old picked up a minor calf injury in training with the Three Lions on Sunday afternoon. A subsequent scan and medical assessment on Monday unfortunately confirmed he could play no further part in England's tourname</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>withdrawn from, injury, calf injury, confirmed, withdrawn from, injury</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>https://nitter.net/NUFC/status/2066875900944056421#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026-06-19 18:01</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>🚨⚠️ Christian Pulisic, out of USMNT squad to face Australia due to calf injury.</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>injury, calf injury, injury</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2068023670363017533#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026-06-19 18:01</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>X:@CanadaSoccerEN</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>RT by @CanadaSoccerEN: Last night, Ismaël Koné underwent successful surgery to repair a lower limb fracture. He is expected to make a full recovery but will miss the remainder of FIFA World Cup 2026™️.
+You will come back stronger, Isma! 🫶</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>will miss the</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>https://nitter.net/CANMNT_Official/status/2068020795037913377#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026-06-19 22:01</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>X:@David_Ornstein</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>🚨 Tino Livramento to miss World Cup with calf injury. Not serious but major blow for Newcastle United defender &amp; #England ahead of #2026FIFAWorldCup opener vs #Croatia  - 23yo returning to #NUFC + Trevoh Chalobah called up @TheAthleticFC post @Matt_Law_DT https://www.nytimes.com/athletic/7365471/202</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>miss world cup, injury, calf injury, injury, miss world cup</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>https://nitter.net/David_Ornstein/status/2066854654982463927#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-06-20 02:01</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>🚨⚠️ Raphinha leaves the pitch with an injury, subbed off.
+Rayan makes his World Cup debut. 🇧🇷</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>injury, leaves, injury</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2068141410876838114#m</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker refresh Sat 20 Jun · GER through R32 · Gakpo brace · Casemiro Inter Miami HWG · Malacia released
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Transfer_Tracker.xlsx
+++ b/Transfer_Tracker.xlsx
@@ -500,7 +500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F436"/>
+  <dimension ref="A1:F462"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -12336,7 +12336,6 @@
       </c>
     </row>
     <row r="435">
-      <c r="A435" t="inlineStr"/>
       <c r="B435" t="inlineStr">
         <is>
           <t>2026-06-20 06:00</t>
@@ -12365,7 +12364,6 @@
       </c>
     </row>
     <row r="436">
-      <c r="A436" t="inlineStr"/>
       <c r="B436" t="inlineStr">
         <is>
           <t>2026-06-20 06:00</t>
@@ -12389,6 +12387,713 @@
       <c r="F436" t="inlineStr">
         <is>
           <t>https://www.arsenal.com/news/karl-hein-join-werder-bremen-permanent-deal?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>2026-06-20 14:01</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D437" s="2" t="inlineStr">
+        <is>
+          <t>🚨🚜 Ipswich Town are set to seal the agreement with Gary O’Neill as new head coach.
+All done with formal steps to follow as O’Neill and RC Strasbourg are set to part ways soon.
+#ITFC agreed terms with O’Neill.</t>
+        </is>
+      </c>
+      <c r="E437" s="2" t="inlineStr">
+        <is>
+          <t>agreed, new head coach</t>
+        </is>
+      </c>
+      <c r="F437" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2068242453925355642#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>2026-06-20 14:01</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D438" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Grillitsch exerce opção e deixa o Sp. Braga</t>
+        </is>
+      </c>
+      <c r="E438" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, contrato, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F438" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mercado/sp-braga/oficial-grillitsch-exerce-opcao-e-deixa-o-sp-braga</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>2026-06-20 14:01</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D439" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Santa Clara confirma saída de Klismahn para o Neftchi Baku</t>
+        </is>
+      </c>
+      <c r="E439" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, confirma, transferência, saída, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F439" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/santa-clara/liga/oficial-santa-clara-confirma-saida-de-klismahn-para-o-neftchi-baku</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>2026-06-20 14:01</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D440" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Grillitsch exerce opção e deixa o Sp. Braga</t>
+        </is>
+      </c>
+      <c r="E440" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, transferência, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F440" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mercado/sp-braga/oficial-grillitsch-exerce-opcao-e-deixa-o-sp-braga</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>2026-06-20 14:01</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D441" s="2" t="inlineStr">
+        <is>
+          <t>Casemiro fecha acordo para jogar ao lado de Messi no Inter Miami</t>
+        </is>
+      </c>
+      <c r="E441" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, transferência</t>
+        </is>
+      </c>
+      <c r="F441" t="inlineStr">
+        <is>
+          <t>https://t.co/gHty3SWAIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>2026-06-20 14:01</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D442" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Keiber Lamadrid fica em definitivo no West Ham</t>
+        </is>
+      </c>
+      <c r="E442" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F442" t="inlineStr">
+        <is>
+          <t>https://x.com/WestHam/status/2068272898561966419?ref_src=twsrc%5Etfw</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>2026-06-20 15:01</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D443" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Santa Clara confirma saída de Klismahn para o Neftchi Baku</t>
+        </is>
+      </c>
+      <c r="E443" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, confirma, saída, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F443" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/santa-clara/liga/oficial-santa-clara-confirma-saida-de-klismahn-para-o-neftchi-baku</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>2026-06-20 15:01</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D444" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Grillitsch exerce opção e deixa o Sp. Braga</t>
+        </is>
+      </c>
+      <c r="E444" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, transferência, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F444" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mercado/sp-braga/oficial-grillitsch-exerce-opcao-e-deixa-o-sp-braga</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>2026-06-20 16:01</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D445" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Nuno Sequeira troca Pendikspor pelo Fafe</t>
+        </is>
+      </c>
+      <c r="E445" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contratação, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F445" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://maisfutebol.iol.pt/cronologia/6373897a0cf2254fb2824fe4#OFICIAL: Nuno Sequeira troca Pendikspor </t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>2026-06-20 16:01</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D446" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Ipswich · Chuba Akpom — Transfer In · - Ajax</t>
+        </is>
+      </c>
+      <c r="E446" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F446" t="inlineStr">
+        <is>
+          <t>https://www.itfc.co.uk/news/2026/may/05/permanent-deal-for-chuba/?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>2026-06-20 16:01</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D447" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Man Utd · Casemiro — Released</t>
+        </is>
+      </c>
+      <c r="E447" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F447" t="inlineStr">
+        <is>
+          <t>https://www.manutd.com/en/news/casemiro-to-leave-man-utd-at-the-end-of-the-2025-26-season?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>2026-06-20 16:01</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D448" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Newcastle · Ewen Jaouen — Transfer In · - Reims</t>
+        </is>
+      </c>
+      <c r="E448" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F448" t="inlineStr">
+        <is>
+          <t>https://www.newcastleunited.com/en/news/ewen-jaouen-signs-for-newcastle-united?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>2026-06-20 17:01</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D449" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Luís Pinto é o novo treinador do Gil Vicente</t>
+        </is>
+      </c>
+      <c r="E449" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, contrato, novo treinador, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F449" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/liga/gil-vicente/oficial-luis-pinto-e-o-novo-treinador-do-gil-vicente</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>2026-06-20 17:01</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D450" s="2" t="inlineStr">
+        <is>
+          <t>Real Madrid desmente interesse em Olise, pérola do Bayern Munique</t>
+        </is>
+      </c>
+      <c r="E450" s="2" t="inlineStr">
+        <is>
+          <t>anunciou, contratação</t>
+        </is>
+      </c>
+      <c r="F450" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/real-madrid/bayern/real-madrid-desmente-interesse-em-michael-olise-perola-do-bayern-munique</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>2026-06-20 17:01</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D451" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Gonçalo Oliveira deixa Benfica e ruma ao Rennes</t>
+        </is>
+      </c>
+      <c r="E451" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contratação, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F451" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/benfica/20-06-2026/oficial-goncalo-oliveira-deixa-benfica-e-ruma-ao-rennes</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>2026-06-20 17:01</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D452" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Luís Pinto é o novo treinador do Gil Vicente</t>
+        </is>
+      </c>
+      <c r="E452" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contratação, novo treinador, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F452" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/liga/gil-vicente/oficial-luis-pinto-e-o-novo-treinador-do-gil-vicente</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>2026-06-20 18:01</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D453" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Gonçalo Oliveira deixa Benfica e ruma ao Rennes</t>
+        </is>
+      </c>
+      <c r="E453" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F453" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/benfica/20-06-2026/oficial-goncalo-oliveira-deixa-benfica-e-ruma-ao-rennes</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>2026-06-20 19:15</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D454" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: FC Porto contrata jovem promessa Eirik Granaas</t>
+        </is>
+      </c>
+      <c r="E454" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F454" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/fc-porto/20-06-2026/oficial-fc-porto-contrata-jovem-promessa-eirik-granaas</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>2026-06-20 19:15</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D455" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Vizela contrata gigante sérvio para a baliza</t>
+        </is>
+      </c>
+      <c r="E455" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, chega, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F455" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DZ0Hta6MmDr/?utm_source=ig_embed&amp;utm_campaign=loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>2026-06-20 19:15</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D456" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: FC Porto contrata jovem promessa Eirik Granaas</t>
+        </is>
+      </c>
+      <c r="E456" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contratação, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F456" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/fc-porto/20-06-2026/oficial-fc-porto-contrata-jovem-promessa-eirik-granaas</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>2026-06-20 19:15</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D457" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Leeds United · Illan Meslier — Released</t>
+        </is>
+      </c>
+      <c r="E457" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F457" t="inlineStr">
+        <is>
+          <t>https://www.leedsunited.com/en/news/illan-meslier-to-leave-leeds-united?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>2026-06-20 20:14</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D458" s="2" t="inlineStr">
+        <is>
+          <t>🌎🇳🇱 OFFICIAL: Cody Gakpo wins FIFA Man of the Match Award after delivering a brace against Sweden.</t>
+        </is>
+      </c>
+      <c r="E458" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F458" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2068416185738129661#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>2026-06-20 22:01</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D459" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Man Utd · Tyrell Malacia — Released</t>
+        </is>
+      </c>
+      <c r="E459" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F459" t="inlineStr">
+        <is>
+          <t>https://www.manutd.com/en/news/tyrell-malacia-to-leave-united-in-the-summer-2026?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr"/>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>2026-06-20 22:19</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D460" s="2" t="inlineStr">
+        <is>
+          <t>🚨🇩🇪 OFFICIAL: Germany qualify to FIFA World Cup Round of 32.</t>
+        </is>
+      </c>
+      <c r="E460" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F460" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2068454051184849260#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr"/>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>2026-06-20 22:19</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D461" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Santa Clara confirma saída de Klismahn para o Neftchi Baku</t>
+        </is>
+      </c>
+      <c r="E461" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, confirma, transferência, saída, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F461" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/santa-clara/liga/oficial-santa-clara-confirma-saida-de-klismahn-para-o-neftchi-baku</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr"/>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>2026-06-20 22:19</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D462" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Fulham · Oliver Mayer — Released</t>
+        </is>
+      </c>
+      <c r="E462" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F462" t="inlineStr">
+        <is>
+          <t>https://www.fulhamfc.com/news/2026/june/08/player-contract-updates/?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
         </is>
       </c>
     </row>
@@ -12403,7 +13108,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F59"/>
+  <dimension ref="A1:F62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -14069,6 +14774,91 @@
         </is>
       </c>
     </row>
+    <row r="60">
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>2026-06-20 14:01</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>🚨 EXCLUSIVE: Inter Miami complete deal to sign Casemiro as new midfielder, here we go!
+Verbal agreement sealed with all parties involved and all formal steps resolved, now waiting to sign and announce the Brazilian.
+Casemiro wants to play with Messi. Future in MLS. 🇺🇸</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>deal, verbal agreement, HERE WE GO, Here we go!, Here We Go, here we go</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2068295942483198454#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>2026-06-20 18:01</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>RT by @FabrizioRomano: 🚨 EXCLUSIVE: Inter Miami complete deal to sign Casemiro as new midfielder, here we go!
+Verbal agreement sealed with all parties involved and all formal steps resolved, now waiting to sign and announce the Brazilian.
+Casemiro wants to play with Messi. Future in MLS. 🇺🇸</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>deal, verbal agreement, HERE WE GO, Here we go!, Here We Go, here we go</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2068295942483198454#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>2026-06-20 18:01</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>Barcelona avança por jovem promessa equatoriana</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>chega, acordo verbal, deverá</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>https://t.co/dI7cju62u1</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -14080,7 +14870,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -15030,6 +15820,170 @@
       <c r="F34" t="inlineStr">
         <is>
           <t>https://nitter.net/FabrizioRomano/status/2068141410876838114#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026-06-20 07:00</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>🚨 Carlo Ancelotti confirms Raphinha will undergo tests in the next 24h to assess his injury.</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>injury, injury</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2068213255256883467#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2026-06-20 14:01</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>X:@ChelseaFC</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Here's the games to look out for in #CFC's 26/27 #PL season! 👀</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>out for</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>https://nitter.net/ChelseaFC/status/2068320829482336368#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026-06-20 14:01</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Incrível: fora do Mundial 2026, Maguire distribui cromos nos EUA</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>fora do mundial, deixa, fora do mundial</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/incrivel/mundial2026/incrivel-fora-do-mundial-2026-maguire-distribui-cromos-nos-eua</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2026-06-20 15:01</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Incrível: fora do Mundial 2026, Maguire distribui cromos nos EUA</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>fora do mundial, deixa, fora do mundial</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/incrivel/mundial2026/incrivel-fora-do-mundial-2026-maguire-distribui-cromos-nos-eua</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2026-06-20 21:01</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>🚨 BREAKING: Raphinha has a muscle injury in his right thigh, Brazil tests have confirmed.
+Raphinha will now undergo intensive treatment, staying with Brazil squad at the World Cup and trying to recover for later stages.
+Rapha will miss the upcoming game vs Scotland.</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>will miss the, injury, muscle injury, confirmed, injury</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2068428781891543324#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2026-06-20 22:01</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>CBF confirma lesão de Raphinha, imprensa fala em paragem de duas semanas</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>lesão, confirma, lesão</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/internacional/raphinha/cbf-confirma-lesao-de-raphinha-imprensa-fala-em-paragem-de-duas-semanas</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker refresh Sun 21 Jun · Carter Pinnington loan LIV→WBA · Cedric Itten Bremen · ESP lineup
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Transfer_Tracker.xlsx
+++ b/Transfer_Tracker.xlsx
@@ -500,7 +500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F462"/>
+  <dimension ref="A1:F491"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -13014,7 +13014,6 @@
       </c>
     </row>
     <row r="460">
-      <c r="A460" t="inlineStr"/>
       <c r="B460" t="inlineStr">
         <is>
           <t>2026-06-20 22:19</t>
@@ -13042,7 +13041,6 @@
       </c>
     </row>
     <row r="461">
-      <c r="A461" t="inlineStr"/>
       <c r="B461" t="inlineStr">
         <is>
           <t>2026-06-20 22:19</t>
@@ -13070,7 +13068,6 @@
       </c>
     </row>
     <row r="462">
-      <c r="A462" t="inlineStr"/>
       <c r="B462" t="inlineStr">
         <is>
           <t>2026-06-20 22:19</t>
@@ -13094,6 +13091,791 @@
       <c r="F462" t="inlineStr">
         <is>
           <t>https://www.fulhamfc.com/news/2026/june/08/player-contract-updates/?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>2026-06-20 23:01</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D463" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Shakhtar Donetsk anuncia extremo brasileiro</t>
+        </is>
+      </c>
+      <c r="E463" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIALMENTE, anuncia, OFICIAL:, OFICIALMENTE</t>
+        </is>
+      </c>
+      <c r="F463" t="inlineStr">
+        <is>
+          <t>https://x.com/hashtag/Shakhtar?src=hash&amp;ref_src=twsrc%5Etfw</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>2026-06-21 02:01</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D464" s="2" t="inlineStr">
+        <is>
+          <t>Real Madrid desmente interesse em Olise, pérola do Bayern Munique</t>
+        </is>
+      </c>
+      <c r="E464" s="2" t="inlineStr">
+        <is>
+          <t>anunciou, contratação</t>
+        </is>
+      </c>
+      <c r="F464" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/real-madrid/bayern/real-madrid-desmente-interesse-em-michael-olise-perola-do-bayern-munique</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>2026-06-21 02:01</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D465" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Sunderland · Milan Aleksic — loan-out · - Partizan Belgrade</t>
+        </is>
+      </c>
+      <c r="E465" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, loan, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F465" t="inlineStr">
+        <is>
+          <t>https://www.safc.com/news/2026/june/18/milan-aleksi--joins-partizan-belgrade-on-loan/?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>2026-06-21 06:42</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D466" s="2" t="inlineStr">
+        <is>
+          <t>🚨🇹🇳 OFFICIAL: Tunisia have been ELIMINATED from the World Cup. ❌</t>
+        </is>
+      </c>
+      <c r="E466" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F466" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2068572332382212210#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>2026-06-21 06:42</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D467" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Gonçalo Oliveira deixa Benfica e ruma ao Rennes</t>
+        </is>
+      </c>
+      <c r="E467" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contratação, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F467" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/benfica/20-06-2026/oficial-goncalo-oliveira-deixa-benfica-e-ruma-ao-rennes</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>2026-06-21 08:40</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D468" s="2" t="inlineStr">
+        <is>
+          <t>🚨 Manchester City offered new deal to Rodri few months ago but there’s still no agreement at this stage. Deal on stand-by now, still long time to decide as current agreement set to expire in June 2027. Rodri could leave as free agent in one year. 🎥 http://youtu.be/K4Z8GebXIXo?is=i5CkRXpqwdgiwcMB</t>
+        </is>
+      </c>
+      <c r="E468" s="2" t="inlineStr">
+        <is>
+          <t>deal, free agent</t>
+        </is>
+      </c>
+      <c r="F468" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2068605087359119604#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>2026-06-21 08:40</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>X:@SpursOfficial</t>
+        </is>
+      </c>
+      <c r="D469" s="2" t="inlineStr">
+        <is>
+          <t>R to @SpursOfficial: Image</t>
+        </is>
+      </c>
+      <c r="E469" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F469" t="inlineStr">
+        <is>
+          <t>https://nitter.net/SpursOfficial/status/2068601195040559330#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>2026-06-21 08:40</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>X:@SpursOfficial</t>
+        </is>
+      </c>
+      <c r="D470" s="2" t="inlineStr">
+        <is>
+          <t>R to @SpursOfficial: Image</t>
+        </is>
+      </c>
+      <c r="E470" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F470" t="inlineStr">
+        <is>
+          <t>https://nitter.net/SpursOfficial/status/2068601189487276506#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>2026-06-21 08:40</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>X:@SpursOfficial</t>
+        </is>
+      </c>
+      <c r="D471" s="2" t="inlineStr">
+        <is>
+          <t>R to @SpursOfficial: Image</t>
+        </is>
+      </c>
+      <c r="E471" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F471" t="inlineStr">
+        <is>
+          <t>https://nitter.net/SpursOfficial/status/2068601185666281507#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>2026-06-21 08:40</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>X:@SpursOfficial</t>
+        </is>
+      </c>
+      <c r="D472" s="2" t="inlineStr">
+        <is>
+          <t>R to @SpursOfficial: Image</t>
+        </is>
+      </c>
+      <c r="E472" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F472" t="inlineStr">
+        <is>
+          <t>https://nitter.net/SpursOfficial/status/2068601181593616788#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>2026-06-21 08:40</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>X:@SpursOfficial</t>
+        </is>
+      </c>
+      <c r="D473" s="2" t="inlineStr">
+        <is>
+          <t>R to @SpursOfficial: Image</t>
+        </is>
+      </c>
+      <c r="E473" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F473" t="inlineStr">
+        <is>
+          <t>https://nitter.net/SpursOfficial/status/2068601178288541769#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>2026-06-21 08:40</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>X:@SpursOfficial</t>
+        </is>
+      </c>
+      <c r="D474" s="2" t="inlineStr">
+        <is>
+          <t>R to @SpursOfficial: Image</t>
+        </is>
+      </c>
+      <c r="E474" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F474" t="inlineStr">
+        <is>
+          <t>https://nitter.net/SpursOfficial/status/2068601174417137833#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>2026-06-21 08:40</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>X:@SpursOfficial</t>
+        </is>
+      </c>
+      <c r="D475" s="2" t="inlineStr">
+        <is>
+          <t>R to @SpursOfficial: Image</t>
+        </is>
+      </c>
+      <c r="E475" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F475" t="inlineStr">
+        <is>
+          <t>https://nitter.net/SpursOfficial/status/2068601170906472717#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>2026-06-21 08:40</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>X:@SpursOfficial</t>
+        </is>
+      </c>
+      <c r="D476" s="2" t="inlineStr">
+        <is>
+          <t>R to @SpursOfficial: Image</t>
+        </is>
+      </c>
+      <c r="E476" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F476" t="inlineStr">
+        <is>
+          <t>https://nitter.net/SpursOfficial/status/2068601167848808519#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>2026-06-21 08:40</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>X:@HullCity</t>
+        </is>
+      </c>
+      <c r="D477" s="2" t="inlineStr">
+        <is>
+          <t>Ahead of fixture release tomorrow, the club would like to provide an update on 26/27 memberships... Following promotion, we are working with the Premier League on required upgrades before Membership details and sales info can be confirmed. More info 🔗 https://www.wearehullcity.co.uk/news/2026/june/1</t>
+        </is>
+      </c>
+      <c r="E477" s="2" t="inlineStr">
+        <is>
+          <t>confirmed, release</t>
+        </is>
+      </c>
+      <c r="F477" t="inlineStr">
+        <is>
+          <t>https://nitter.net/HullCity/status/2067593196117373122#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>2026-06-21 08:40</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D478" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Ipswich · Leon Ayinde — Transfer Out · - Doncaster</t>
+        </is>
+      </c>
+      <c r="E478" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F478" t="inlineStr">
+        <is>
+          <t>https://www.itfc.co.uk/news/2026/may/20/leon-ayinde-to-join-doncaster/?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>2026-06-21 09:52</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D479" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Paulo Oliveira deixa o Sp. Braga</t>
+        </is>
+      </c>
+      <c r="E479" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F479" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mercado/paulo-oliveira/oficial-paulo-oliveira-deixa-o-sp-braga</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>2026-06-21 09:52</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D480" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Sp. Braga despede-se de Paulo Oliveira, um «exemplo»</t>
+        </is>
+      </c>
+      <c r="E480" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F480" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mercado/paulo-oliveira/oficial-paulo-oliveira-deixa-o-sp-braga</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>2026-06-21 10:24</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D481" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Brentford · Reiss Nelson — End of Loan · - Arsenal</t>
+        </is>
+      </c>
+      <c r="E481" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, loan, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F481" t="inlineStr">
+        <is>
+          <t>https://www.brentfordfc.com/en/news/article/first-team-ryan-trevitt-departs-brentford-reiss-nelson-returns-arsenal?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=trans</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>2026-06-21 11:54</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D482" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Sp. Braga despede-se de Paulo Oliveira, um «exemplo»</t>
+        </is>
+      </c>
+      <c r="E482" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F482" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mercado/paulo-oliveira/oficial-paulo-oliveira-deixa-o-sp-braga</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>2026-06-21 12:55</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D483" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Everton · Isaac Heath — Transfer Out · - Cambridge United</t>
+        </is>
+      </c>
+      <c r="E483" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F483" t="inlineStr">
+        <is>
+          <t>https://www.evertonfc.com/news/2026/june/15/heath-departs-for-cambridge?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch?utm_source=premier-league&amp;utm_med</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>2026-06-21 13:44</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D484" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Grillitsch exerce opção e deixa o Sp. Braga</t>
+        </is>
+      </c>
+      <c r="E484" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, transferência, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F484" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mercado/sp-braga/oficial-grillitsch-exerce-opcao-e-deixa-o-sp-braga</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>2026-06-21 14:02</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D485" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Brighton &amp; Hove Albion · Adam Webster — Released</t>
+        </is>
+      </c>
+      <c r="E485" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F485" t="inlineStr">
+        <is>
+          <t>https://www.brightonandhovealbion.com/media-article/webster-to-depart-albion-this-summer?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>2026-06-21 14:02</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D486" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Newcastle · Ewen Jaouen — Transfer In · - Reims</t>
+        </is>
+      </c>
+      <c r="E486" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F486" t="inlineStr">
+        <is>
+          <t>https://www.newcastleunited.com/en/news/ewen-jaouen-signs-for-newcastle-united?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>2026-06-21 15:02</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>X:@SpursOfficial</t>
+        </is>
+      </c>
+      <c r="D487" s="2" t="inlineStr">
+        <is>
+          <t>R to @SpursOfficial: Image</t>
+        </is>
+      </c>
+      <c r="E487" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F487" t="inlineStr">
+        <is>
+          <t>https://nitter.net/SpursOfficial/status/2068601178288541769#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>2026-06-21 15:02</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>X:@SEFutbol</t>
+        </is>
+      </c>
+      <c r="D488" s="2" t="inlineStr">
+        <is>
+          <t>🚨 OFICIAL | Ya tenemos nuestro 𝗢𝗡𝗖𝗘 ante Arabia Saudí. #VamosEspaña | #CopaMundialFIFA</t>
+        </is>
+      </c>
+      <c r="E488" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, 🚨 OFICIAL</t>
+        </is>
+      </c>
+      <c r="F488" t="inlineStr">
+        <is>
+          <t>https://nitter.net/SEFutbol/status/2068698958881227242#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>2026-06-21 15:02</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D489" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Cedric Itten troca Dusseldorf pelo Werder Bremen</t>
+        </is>
+      </c>
+      <c r="E489" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contratação, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F489" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/cronologia/6373897a0cf2254fb2824fe4#OFICIAL: Cedric Itten troca Dusseldorf p</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr"/>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>2026-06-21 15:05</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D490" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Gonçalo Oliveira deixa Benfica e ruma ao Rennes</t>
+        </is>
+      </c>
+      <c r="E490" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contratação, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F490" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/benfica/20-06-2026/oficial-goncalo-oliveira-deixa-benfica-e-ruma-ao-rennes</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr"/>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>2026-06-21 15:05</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D491" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Liverpool · Carter Pinnington — Transfer Out · - West Brom</t>
+        </is>
+      </c>
+      <c r="E491" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F491" t="inlineStr">
+        <is>
+          <t>https://www.liverpoolfc.com/news/carter-pinnington-joins-west-bromwich-albion?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
         </is>
       </c>
     </row>
@@ -13108,7 +13890,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F62"/>
+  <dimension ref="A1:F63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -14859,6 +15641,33 @@
         </is>
       </c>
     </row>
+    <row r="63">
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>2026-06-21 01:01</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>Gil Vicente: Luís Esteves perto de trocar Barcelos pelo México</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>saída, perto de</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/liga/gil-vicente/gil-vicente-luis-esteves-perto-de-trocar-barcelos-pelo-mexico</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -14870,7 +15679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -15984,6 +16793,196 @@
       <c r="F40" t="inlineStr">
         <is>
           <t>https://maisfutebol.iol.pt/internacional/raphinha/cbf-confirma-lesao-de-raphinha-imprensa-fala-em-paragem-de-duas-semanas</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2026-06-20 23:01</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>🚨🇩🇪 Nico Schlotterbeck World Cup could be over due to an injury.
+“Nico is suspected to have sustained a ligament injury. It's not looking good”, says Julian Nagelsmann.</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>injury, injury</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2068461893358846373#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2026-06-20 23:01</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>X:@David_Ornstein</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>🚨 Tino Livramento to miss World Cup with calf injury. Not serious but major blow for Newcastle United defender &amp; #England ahead of #2026FIFAWorldCup opener vs #Croatia  - 23yo returning to #NUFC + Trevoh Chalobah called up @TheAthleticFC post @Matt_Law_DT https://www.nytimes.com/athletic/7365471/202</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>miss world cup, injury, calf injury, injury, miss world cup</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>https://nitter.net/David_Ornstein/status/2066854654982463927#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2026-06-21 07:19</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>❌🇹🇳 Tunisia are out of the World Cup after two games, two different coaches, 9 goals conceded.</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>out of the world cup, out of the world, out of the world cup</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2068574304879472808#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2026-06-21 08:40</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>X:@David_Ornstein</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>R to @David_Ornstein: 🚨 Trevoh Chalobah called up last night &amp; travelling to join #England squad in USA. 26yo Chelsea defender not expected to be involved against #Croatia but will be available for subsequent group #2026FIFAWorldCup matches vs #Ghana &amp; #Panama @TheAthleticFC https://www.nytimes.com/</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>miss world cup, injury, calf injury, injury, miss world cup</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>https://nitter.net/David_Ornstein/status/2066860492295950545#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2026-06-21 08:40</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>X:@David_Ornstein</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>🚨 Tino Livramento to miss World Cup with calf injury. Not serious but major blow for Newcastle United defender &amp; #England ahead of #2026FIFAWorldCup opener vs #Croatia - 23yo returning to #NUFC + Trevoh Chalobah called up @TheAthleticFC post @Matt_Law_DT https://www.nytimes.com/athletic/7365471/2026</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>miss world cup, injury, calf injury, injury, miss world cup</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>https://nitter.net/David_Ornstein/status/2066854654982463927#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2026-06-21 08:40</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>X:@NUFC</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Tino Livramento has withdrawn from @England's #FIFAWorldCup 2026 squad. The 23-year-old picked up a minor calf injury in training with the Three Lions on Sunday afternoon. A subsequent scan and medical assessment on Monday unfortunately confirmed he could play no further part in England's tournament</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>withdrawn from, injury, calf injury, confirmed, withdrawn from, injury</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>https://nitter.net/NUFC/status/2066875900944056421#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2026-06-21 11:54</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Nico Schlotterbeck sofreu lesão ligamentar: «Não parece nada bom»</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>lesão, lesão</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mundial-2026/mundial2026/nico-schlotterbeck-sofreu-lesao-ligamentar-nao-parece-nada-bom</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Gueye released by EVE · tracker refresh Mon 22 Jun
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Transfer_Tracker.xlsx
+++ b/Transfer_Tracker.xlsx
@@ -500,7 +500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F491"/>
+  <dimension ref="A1:F521"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -13824,7 +13824,6 @@
       </c>
     </row>
     <row r="490">
-      <c r="A490" t="inlineStr"/>
       <c r="B490" t="inlineStr">
         <is>
           <t>2026-06-21 15:05</t>
@@ -13852,7 +13851,6 @@
       </c>
     </row>
     <row r="491">
-      <c r="A491" t="inlineStr"/>
       <c r="B491" t="inlineStr">
         <is>
           <t>2026-06-21 15:05</t>
@@ -13876,6 +13874,818 @@
       <c r="F491" t="inlineStr">
         <is>
           <t>https://www.liverpoolfc.com/news/carter-pinnington-joins-west-bromwich-albion?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>2026-06-21 17:46</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>X:@BurnleyOfficial</t>
+        </is>
+      </c>
+      <c r="D492" s="2" t="inlineStr">
+        <is>
+          <t>R to @BurnleyOfficial: Read more: https://burnleyfootballclub.com/content/burnley-fc-launch-2026-27-memberships</t>
+        </is>
+      </c>
+      <c r="E492" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F492" t="inlineStr">
+        <is>
+          <t>https://nitter.net/BurnleyOfficial/status/2067602898213585201#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>2026-06-21 17:46</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D493" s="2" t="inlineStr">
+        <is>
+          <t>Villas-Boas assume cobiça por Diogo Costa e fala de Mora: «Temos de pagar salários»</t>
+        </is>
+      </c>
+      <c r="E493" s="2" t="inlineStr">
+        <is>
+          <t>anunciou, contratação</t>
+        </is>
+      </c>
+      <c r="F493" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/fc-porto/villas-boas/villas-boas-assume-cobica-por-diogo-costa-e-fala-de-mora-temos-de-pagar-salarios</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>2026-06-21 17:46</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D494" s="2" t="inlineStr">
+        <is>
+          <t>«Pavlidis? Não temos propostas, ele quer e vai ficar no Benfica»</t>
+        </is>
+      </c>
+      <c r="E494" s="2" t="inlineStr">
+        <is>
+          <t>anunciou, contratação</t>
+        </is>
+      </c>
+      <c r="F494" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/benfica/mario-branco/pavlidis-nao-temos-propostas-ele-quer-e-vai-ficar-no-benfica</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>2026-06-21 18:30</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D495" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: União Leiria renova com avançado e blinda-o com cláusula de 50M</t>
+        </is>
+      </c>
+      <c r="E495" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F495" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/transferencias/uniao-leiria/oficial-uniao-leiria-renova-com-avancado-e-blinda-com-clausula-de-50m</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>2026-06-21 18:30</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D496" s="2" t="inlineStr">
+        <is>
+          <t>Sporting: Martim, irmão de Rodrigo Ribeiro, assina contrato profissional</t>
+        </is>
+      </c>
+      <c r="E496" s="2" t="inlineStr">
+        <is>
+          <t>anunciou, contratação, contrato</t>
+        </is>
+      </c>
+      <c r="F496" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/sporting/martim-ribeiro/sporting-martim-irmao-de-rodrigo-ribeiro-assina-contrato-profissional</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>2026-06-21 18:30</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D497" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: União Leiria renova com avançado e blinda-o com cláusula de 50M</t>
+        </is>
+      </c>
+      <c r="E497" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contratação, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F497" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/transferencias/uniao-leiria/oficial-uniao-leiria-renova-com-avancado-e-blinda-com-clausula-de-50m</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>2026-06-21 19:47</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D498" s="2" t="inlineStr">
+        <is>
+          <t>🌎🇪🇸 OFFICIAL: Mikel Oyarzabal, FIFA Man of the Match for Spain against Saudi. Two goals, one assist.</t>
+        </is>
+      </c>
+      <c r="E498" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F498" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2068763955602891213#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>2026-06-21 19:47</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D499" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: U. Leiria renova com avançado e blinda-o com cláusula de 50M</t>
+        </is>
+      </c>
+      <c r="E499" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F499" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/transferencias/uniao-leiria/oficial-uniao-leiria-renova-com-avancado-e-blinda-com-clausula-de-50m</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>2026-06-21 19:47</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D500" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: U. Leiria renova com avançado e blinda-o com cláusula de 50M</t>
+        </is>
+      </c>
+      <c r="E500" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contratação, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F500" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/transferencias/uniao-leiria/oficial-uniao-leiria-renova-com-avancado-e-blinda-com-clausula-de-50m</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>2026-06-21 19:47</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D501" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Liverpool · Andy Robertson — Released</t>
+        </is>
+      </c>
+      <c r="E501" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F501" t="inlineStr">
+        <is>
+          <t>https://www.liverpoolfc.com/news/andy-robertson-leave-liverpool-end-season?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>2026-06-21 20:21</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D502" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Liverpool · James Balagizi — Released</t>
+        </is>
+      </c>
+      <c r="E502" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F502" t="inlineStr">
+        <is>
+          <t>https://www.liverpoolfc.com/news/liverpool-confirm-premier-league-retained-list?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>2026-06-21 21:57</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D503" s="2" t="inlineStr">
+        <is>
+          <t>Ajax anuncia acordo para rescindir com Óscar García</t>
+        </is>
+      </c>
+      <c r="E503" s="2" t="inlineStr">
+        <is>
+          <t>anuncia, anunciou, contratação</t>
+        </is>
+      </c>
+      <c r="F503" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/ajax/mercado-de-transferencias/ajax-anuncia-acordo-para-rescindir-com-oscar-garcia</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>2026-06-22 00:01</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D504" s="2" t="inlineStr">
+        <is>
+          <t>🚨🇹🇷 Hrvoje Smolcic joins Arca Çorum FK on two year deal plus one year option, deal completed today. Green light from Eintracht Frankfurt.</t>
+        </is>
+      </c>
+      <c r="E504" s="2" t="inlineStr">
+        <is>
+          <t>deal, joins</t>
+        </is>
+      </c>
+      <c r="F504" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2068837664900399266#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>2026-06-22 00:01</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>X:@IpswichTown</t>
+        </is>
+      </c>
+      <c r="D505" s="2" t="inlineStr">
+        <is>
+          <t>RT by @IpswichTown: 🤝 The club is delighted to announce that captain Maria Boswell has signed a new deal.  Maria joined Town in the summer of 2019 and has now extended her stay in Suffolk for at least another year.</t>
+        </is>
+      </c>
+      <c r="E505" s="2" t="inlineStr">
+        <is>
+          <t>deal, signed, signs, joined</t>
+        </is>
+      </c>
+      <c r="F505" t="inlineStr">
+        <is>
+          <t>https://nitter.net/ITFCWomen/status/2067578083247292810#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>2026-06-22 01:01</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D506" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Liverpool · DJ Bernard — Released</t>
+        </is>
+      </c>
+      <c r="E506" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F506" t="inlineStr">
+        <is>
+          <t>https://www.liverpoolfc.com/news/liverpool-confirm-premier-league-retained-list?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>2026-06-22 02:01</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D507" s="2" t="inlineStr">
+        <is>
+          <t>🌎🍿 OFFICIAL: Kevin Pina, FIFA Man of the Match for Cape Verde vs Uruguay.</t>
+        </is>
+      </c>
+      <c r="E507" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F507" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2068869077909529043#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>2026-06-22 02:01</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D508" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Man Utd · Tyrell Malacia — Released</t>
+        </is>
+      </c>
+      <c r="E508" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F508" t="inlineStr">
+        <is>
+          <t>https://www.manutd.com/en/news/tyrell-malacia-to-leave-united-in-the-summer-2026?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>2026-06-22 03:01</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D509" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Everton · Isaac Heath — Transfer Out · - Cambridge United</t>
+        </is>
+      </c>
+      <c r="E509" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F509" t="inlineStr">
+        <is>
+          <t>https://www.evertonfc.com/news/2026/june/15/heath-departs-for-cambridge?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch?utm_source=premier-league&amp;utm_med</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>2026-06-22 04:37</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D510" s="2" t="inlineStr">
+        <is>
+          <t>🌎🇪🇬 OFFICIAL: Mo Salah wins Man of the Match Award for Egypt against New Zealand.</t>
+        </is>
+      </c>
+      <c r="E510" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F510" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2068898304566468849#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>2026-06-22 04:37</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>X:@SunderlandAFC</t>
+        </is>
+      </c>
+      <c r="D511" s="2" t="inlineStr">
+        <is>
+          <t>🛣️ Starting on the road 🎅 Boxing Day trip to Merseyside ⚔️ Derby days locked in The key takeaways from fixture release day 👇</t>
+        </is>
+      </c>
+      <c r="E511" s="2" t="inlineStr">
+        <is>
+          <t>confirmed, release</t>
+        </is>
+      </c>
+      <c r="F511" t="inlineStr">
+        <is>
+          <t>https://nitter.net/SunderlandAFC/status/2068272651160735762#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>2026-06-22 04:37</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D512" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Keiber Lamadrid fica em definitivo no West Ham</t>
+        </is>
+      </c>
+      <c r="E512" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F512" t="inlineStr">
+        <is>
+          <t>https://x.com/WestHam/status/2068272898561966419?ref_src=twsrc%5Etfw</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>2026-06-22 04:37</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D513" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Everton · Isaac Heath — Transfer Out · - Cambridge United</t>
+        </is>
+      </c>
+      <c r="E513" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F513" t="inlineStr">
+        <is>
+          <t>https://www.evertonfc.com/news/2026/june/15/heath-departs-for-cambridge?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch?utm_source=premier-league&amp;utm_med</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>2026-06-22 05:40</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>X:@SpursOfficial</t>
+        </is>
+      </c>
+      <c r="D514" s="2" t="inlineStr">
+        <is>
+          <t>R to @SpursOfficial: Image</t>
+        </is>
+      </c>
+      <c r="E514" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F514" t="inlineStr">
+        <is>
+          <t>https://nitter.net/SpursOfficial/status/2068601181593616788#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>2026-06-22 05:40</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D515" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Brighton &amp; Hove Albion · Jan Paul van Hecke — Transfer Out · - Spurs</t>
+        </is>
+      </c>
+      <c r="E515" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F515" t="inlineStr">
+        <is>
+          <t>https://www.brightonandhovealbion.com/media-article/mft-transfer-news-jan-paul-van-hecke-tottenham-hotspur-june-2026?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=tra</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>2026-06-22 06:42</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D516" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Arsenal · Sam Chapman — Released</t>
+        </is>
+      </c>
+      <c r="E516" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F516" t="inlineStr">
+        <is>
+          <t>https://www.arsenal.com/news/contract-updates-15-players-depart-summer?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>2026-06-22 06:42</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D517" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Fulham · Quinn Schutter — Released</t>
+        </is>
+      </c>
+      <c r="E517" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F517" t="inlineStr">
+        <is>
+          <t>https://www.fulhamfc.com/news/2026/june/08/player-contract-updates/?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>2026-06-22 12:01</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D518" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Everton · Idrissa Gana Gueye — Released</t>
+        </is>
+      </c>
+      <c r="E518" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F518" t="inlineStr">
+        <is>
+          <t>https://www.evertonfc.com/news/2026/june/10/everton-player-contracts-update/?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>2026-06-22 12:01</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D519" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Fulham · Callum Cliff — Released</t>
+        </is>
+      </c>
+      <c r="E519" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F519" t="inlineStr">
+        <is>
+          <t>https://www.fulhamfc.com/news/2026/june/08/player-contract-updates/?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr"/>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>2026-06-22 12:43</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>X:@realmadrid</t>
+        </is>
+      </c>
+      <c r="D520" s="2" t="inlineStr">
+        <is>
+          <t>Comunicado Oficial: Sergio Rodríguez.</t>
+        </is>
+      </c>
+      <c r="E520" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F520" t="inlineStr">
+        <is>
+          <t>https://nitter.net/realmadrid/status/2068031059862909396#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr"/>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>2026-06-22 12:43</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D521" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Rubén de la Barrera (ex-Vizela) é o novo treinador do Las Palmas</t>
+        </is>
+      </c>
+      <c r="E521" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, novo treinador, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F521" t="inlineStr">
+        <is>
+          <t>https://t.co/o72vfjOkga</t>
         </is>
       </c>
     </row>
@@ -13890,7 +14700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F63"/>
+  <dimension ref="A1:F64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -15665,6 +16475,33 @@
       <c r="F63" t="inlineStr">
         <is>
           <t>https://maisfutebol.iol.pt/liga/gil-vicente/gil-vicente-luis-esteves-perto-de-trocar-barcelos-pelo-mexico</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>2026-06-21 17:46</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>«Pavlidis? Não temos propostas, ele quer e vai ficar no Benfica»</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>contratação, chega, rumor, rumor, rumores</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/benfica/mario-branco/pavlidis-nao-temos-propostas-ele-quer-e-vai-ficar-no-benfica</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker refresh Tue 23 Jun · Maresca → MCI succeeds Pep (£17m to CHE) · TUR eliminated · Romero injury note
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Transfer_Tracker.xlsx
+++ b/Transfer_Tracker.xlsx
@@ -500,7 +500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F521"/>
+  <dimension ref="A1:F562"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -14634,7 +14634,6 @@
       </c>
     </row>
     <row r="520">
-      <c r="A520" t="inlineStr"/>
       <c r="B520" t="inlineStr">
         <is>
           <t>2026-06-22 12:43</t>
@@ -14662,7 +14661,6 @@
       </c>
     </row>
     <row r="521">
-      <c r="A521" t="inlineStr"/>
       <c r="B521" t="inlineStr">
         <is>
           <t>2026-06-22 12:43</t>
@@ -14686,6 +14684,1115 @@
       <c r="F521" t="inlineStr">
         <is>
           <t>https://t.co/o72vfjOkga</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>2026-06-22 13:01</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D522" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Newcastle · John Ruddy — Released</t>
+        </is>
+      </c>
+      <c r="E522" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F522" t="inlineStr">
+        <is>
+          <t>https://www.newcastleunited.com/en/news/newcastle-united-confirm-mens-first-team-retained-list?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>2026-06-22 16:01</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D523" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Gil Vicente segura capitão dos sub-23 com novo contrato</t>
+        </is>
+      </c>
+      <c r="E523" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, contrato, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F523" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/liga/gil-vicente/oficial-gil-vicente-segura-capitao-dos-sub-23-com-novo-contrato</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>2026-06-22 16:01</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D524" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Gil Vicente segura capitão dos sub-23 com novo contrato</t>
+        </is>
+      </c>
+      <c r="E524" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, contrato, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F524" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/liga/gil-vicente/oficial-gil-vicente-segura-capitao-dos-sub-23-com-novo-contrato</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>2026-06-22 16:01</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D525" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Rubén de la Barrera (ex-Vizela) é o novo treinador do Las Palmas</t>
+        </is>
+      </c>
+      <c r="E525" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, novo treinador, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F525" t="inlineStr">
+        <is>
+          <t>https://t.co/o72vfjOkga</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>2026-06-22 17:01</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D526" s="2" t="inlineStr">
+        <is>
+          <t>🔴⚪️ OFFICIAL: RB Leipzig confirms Martín Demichelis as their new head coach. The 45-year-old Argentine has signed a contract with the Red Bulls until June 30, 2028.</t>
+        </is>
+      </c>
+      <c r="E526" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, signed, new head coach, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F526" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069091740577910819#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>2026-06-22 17:01</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D527" s="2" t="inlineStr">
+        <is>
+          <t>🚨🇧🇬 Stefano Sensi has agreed to join CSKA Sofia for €200k release clause triggered from Anorthosis.</t>
+        </is>
+      </c>
+      <c r="E527" s="2" t="inlineStr">
+        <is>
+          <t>agreed, release</t>
+        </is>
+      </c>
+      <c r="F527" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069082369819111889#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>2026-06-22 17:01</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D528" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: após rescindir com Académico, Sérgio Fonseca assina pelo AVS</t>
+        </is>
+      </c>
+      <c r="E528" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F528" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/transferencias/liga/oficial-apos-rescindir-com-academico-sergio-fonseca-assina-pelo-avs</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>2026-06-22 17:01</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D529" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Manchester United compra terrenos para construir novo estádio</t>
+        </is>
+      </c>
+      <c r="E529" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F529" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/internacional/inglaterra/oficial-manchester-united-compra-terrenos-para-construir-novo-estadio</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>2026-06-22 17:01</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D530" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: após rescindir com Académico, Sérgio Fonseca assina pelo AVS</t>
+        </is>
+      </c>
+      <c r="E530" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F530" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/transferencias/liga/oficial-apos-rescindir-com-academico-sergio-fonseca-assina-pelo-avs</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>2026-06-22 17:01</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D531" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Gonçalo Oliveira deixa Benfica e ruma ao Rennes</t>
+        </is>
+      </c>
+      <c r="E531" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F531" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/benfica/20-06-2026/oficial-goncalo-oliveira-deixa-benfica-e-ruma-ao-rennes</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>2026-06-22 18:05</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D532" s="2" t="inlineStr">
+        <is>
+          <t>🚨🇦🇷 OFFICIAL: LEO MESSI IS WORLD CUP TOP SCORER EVER WITH 17 GOALS. 🌎🤩</t>
+        </is>
+      </c>
+      <c r="E532" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F532" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069113158078255401#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>2026-06-22 18:05</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D533" s="2" t="inlineStr">
+        <is>
+          <t>🚨🇺🇾 Francisco Calvo has agreed to sign as new Nacional de Uruguay player, deal done. Free transfer despite MLS and Saudi clubs keen, seen as ideal addition and ready for new chapter.</t>
+        </is>
+      </c>
+      <c r="E533" s="2" t="inlineStr">
+        <is>
+          <t>agreed, deal, free transfer, alvo</t>
+        </is>
+      </c>
+      <c r="F533" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069110599322095986#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>2026-06-22 18:05</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D534" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Leipzig paga a cláusula e Demichelis deixa o Maiorca</t>
+        </is>
+      </c>
+      <c r="E534" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F534" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mercado-de-transferencias/leipzig/oficial-leipizg-paga-a-clausula-e-demichelis-deixa-o-maiorca</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>2026-06-22 18:05</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D535" s="2" t="inlineStr">
+        <is>
+          <t>II Liga: Felgueiras anuncia cinco saídas</t>
+        </is>
+      </c>
+      <c r="E535" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anuncia, saída</t>
+        </is>
+      </c>
+      <c r="F535" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/cronologia/6373897a0cf2254fb2824fe4#II Liga: Felgueiras anuncia cinco saídas</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>2026-06-22 18:05</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D536" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Alessio Lisci é o novo treinador do PAOK</t>
+        </is>
+      </c>
+      <c r="E536" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, novo treinador, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F536" t="inlineStr">
+        <is>
+          <t>https://x.com/hashtag/Lisci?src=hash&amp;ref_src=twsrc%5Etfw</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>2026-06-22 18:05</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D537" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Sergio Canales regressa a Espanha, para o Racing Santander</t>
+        </is>
+      </c>
+      <c r="E537" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, regressa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F537" t="inlineStr">
+        <is>
+          <t>https://x.com/hashtag/LaLigaEASports?src=hash&amp;ref_src=twsrc%5Etfw</t>
+        </is>
+      </c>
+    </row>
+    <row r="538">
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>2026-06-22 18:05</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D538" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Leipzig paga a cláusula e Demichelis deixa o Maiorca</t>
+        </is>
+      </c>
+      <c r="E538" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, transferência, deixa, novo treinador, negocia, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F538" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mercado-de-transferencias/leipzig/oficial-leipizg-paga-a-clausula-e-demichelis-deixa-o-maiorca</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>2026-06-22 18:05</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D539" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Gil Vicente segura capitão dos sub-23 com novo contrato</t>
+        </is>
+      </c>
+      <c r="E539" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, contrato, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F539" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/liga/gil-vicente/oficial-gil-vicente-segura-capitao-dos-sub-23-com-novo-contrato</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>2026-06-22 18:05</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D540" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: U. Leiria renova com avançado e blinda-o com cláusula de 50M</t>
+        </is>
+      </c>
+      <c r="E540" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contratação, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F540" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/transferencias/uniao-leiria/oficial-uniao-leiria-renova-com-avancado-e-blinda-com-clausula-de-50m</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>2026-06-22 19:01</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D541" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Buntić é reforço do Farense</t>
+        </is>
+      </c>
+      <c r="E541" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contratação, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F541" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/cronologia/6373897a0cf2254fb2824fe4#OFICIAL: Buntić é reforço do Farense</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>2026-06-22 19:01</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D542" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Fulham · Ruban Khan — Released</t>
+        </is>
+      </c>
+      <c r="E542" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F542" t="inlineStr">
+        <is>
+          <t>https://www.fulhamfc.com/news/2026/june/08/player-contract-updates/?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>2026-06-22 19:01</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D543" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Liverpool · Ibrahima Konate — Released</t>
+        </is>
+      </c>
+      <c r="E543" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F543" t="inlineStr">
+        <is>
+          <t>https://www.liverpoolfc.com/news/ibrahima-konate-leave-liverpool-fc?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>2026-06-22 19:01</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D544" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Tottenham Hotspur · Andy Robertson — Transfer In</t>
+        </is>
+      </c>
+      <c r="E544" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F544" t="inlineStr">
+        <is>
+          <t>https://www.tottenhamhotspur.com/news/1071931/robertson-signing-secured?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>2026-06-22 20:01</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D545" s="2" t="inlineStr">
+        <is>
+          <t>🌎🇫🇷 OFFICIAL: Kylian Mbappé reaches 100 caps with French national team… with 58 goals, so far. Their best goalscorer ever. 🥇</t>
+        </is>
+      </c>
+      <c r="E545" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F545" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069143119270904073#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>2026-06-22 20:01</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D546" s="2" t="inlineStr">
+        <is>
+          <t>🌎🇦🇷 OFFICIAL: Lionel Messi, back to back FIFA Man of the Match in two 2026 World Cup games.</t>
+        </is>
+      </c>
+      <c r="E546" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F546" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069137477214843264#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>2026-06-22 20:01</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D547" s="2" t="inlineStr">
+        <is>
+          <t>🌎🇦🇷 OFFICIAL: Argentina qualify for World Cup round of 32!</t>
+        </is>
+      </c>
+      <c r="E547" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F547" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069133304784122002#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>2026-06-22 21:01</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D548" s="2" t="inlineStr">
+        <is>
+          <t>RT by @FabrizioRomano: 🚨🔴⚪️ EXCLUSIVE: Arsenal sent official bid to Leicester City to get Jeremy Monga deal done. 16 year old winger keen on joining #AFC and deal moving quickly now with optimism to sign #LCFC talent, seen as huge prospect for the future. ⏳⌛️</t>
+        </is>
+      </c>
+      <c r="E548" s="2" t="inlineStr">
+        <is>
+          <t>deal, joining</t>
+        </is>
+      </c>
+      <c r="F548" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2067591311130055043#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>2026-06-22 21:01</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D549" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Ricardo Costa substitui Gonçalo Feio como técnico do Tondela</t>
+        </is>
+      </c>
+      <c r="E549" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F549" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/transferencias/ii-liga/oficial-ricardo-costa-substitui-goncalo-feio-como-tecnico-do-tondela</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>2026-06-22 21:01</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D550" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Filipe Çelikkaya sucede a Nuno Campos no comando do Zalaegerszeg</t>
+        </is>
+      </c>
+      <c r="E550" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F550" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/made-in/internacional/oficial-filipe-celikkaya-sucede-a-nuno-campos-no-comando-do-zalaegerszeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>2026-06-22 21:01</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D551" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Ricardo Costa substitui Gonçalo Feio como técnico do Tondela</t>
+        </is>
+      </c>
+      <c r="E551" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, apontado, apontados, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F551" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/transferencias/ii-liga/oficial-ricardo-costa-substitui-goncalo-feio-como-tecnico-do-tondela</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>2026-06-22 21:01</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D552" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Filipe Çelikkaya sucede a Nuno Campos no comando do Zalaegerszeg</t>
+        </is>
+      </c>
+      <c r="E552" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, apontado, apontados, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F552" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/made-in/internacional/oficial-filipe-celikkaya-sucede-a-nuno-campos-no-comando-do-zalaegerszeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>2026-06-22 22:01</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D553" s="2" t="inlineStr">
+        <is>
+          <t>António Silva: «Renovação? Há uma proposta, mas ainda não sei»</t>
+        </is>
+      </c>
+      <c r="E553" s="2" t="inlineStr">
+        <is>
+          <t>deal, contrato, chega</t>
+        </is>
+      </c>
+      <c r="F553" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/benfica/antonio-silva/antonio-silva-renovacao-ha-uma-proposta-mas-ainda-nao-sei</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>2026-06-22 23:01</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D554" s="2" t="inlineStr">
+        <is>
+          <t>🚨 Atlético Madrid statement to @diarioas. “There is no amount of money for which Barça can buy Julián Álvarez. He will not be transferred to Barcelona”. “Either they pay the release clause for €500m or there is no deal”.</t>
+        </is>
+      </c>
+      <c r="E554" s="2" t="inlineStr">
+        <is>
+          <t>deal, release</t>
+        </is>
+      </c>
+      <c r="F554" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069190772105035994#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>2026-06-22 23:01</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D555" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Filipe Çelikkaya sucede a Nuno Campos no comando do Zalaegerszeg</t>
+        </is>
+      </c>
+      <c r="E555" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, apontado, apontados, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F555" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/made-in/internacional/oficial-filipe-celikkaya-sucede-a-nuno-campos-no-comando-do-zalaegerszeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>2026-06-22 23:01</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D556" s="2" t="inlineStr">
+        <is>
+          <t>Sporting: Martim, irmão de Rodrigo Ribeiro, assina contrato profissional</t>
+        </is>
+      </c>
+      <c r="E556" s="2" t="inlineStr">
+        <is>
+          <t>anunciou, contratação, contrato</t>
+        </is>
+      </c>
+      <c r="F556" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/sporting/martim-ribeiro/sporting-martim-irmao-de-rodrigo-ribeiro-assina-contrato-profissional</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>2026-06-23 01:28</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D557" s="2" t="inlineStr">
+        <is>
+          <t>🌎🇫🇷 OFFICIAL: Kylian Mbappé wins Man of the Match Award for France vs Iraq. ✨ 4 goals in 2 games. 16 World Cup goals in 16 career games in the competition. 💥</t>
+        </is>
+      </c>
+      <c r="E557" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F557" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069226673166315678#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>2026-06-23 01:28</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D558" s="2" t="inlineStr">
+        <is>
+          <t>🌎🇫🇷 OFFICIAL: France qualify to World Cup round of 32!</t>
+        </is>
+      </c>
+      <c r="E558" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F558" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069221027419136033#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>2026-06-23 01:28</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D559" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Newcastle · John Ruddy — Released</t>
+        </is>
+      </c>
+      <c r="E559" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F559" t="inlineStr">
+        <is>
+          <t>https://www.newcastleunited.com/en/news/newcastle-united-confirm-mens-first-team-retained-list?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>2026-06-23 02:01</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D560" s="2" t="inlineStr">
+        <is>
+          <t>Ajax anuncia acordo para rescindir com Óscar García</t>
+        </is>
+      </c>
+      <c r="E560" s="2" t="inlineStr">
+        <is>
+          <t>anuncia, anunciou, contratação</t>
+        </is>
+      </c>
+      <c r="F560" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/ajax/mercado-de-transferencias/ajax-anuncia-acordo-para-rescindir-com-oscar-garcia</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr"/>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>2026-06-23 02:19</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D561" s="2" t="inlineStr">
+        <is>
+          <t>🌎🇳🇴 OFFICIAL: Norway qualify to FIFA World Cup Round of 32!</t>
+        </is>
+      </c>
+      <c r="E561" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F561" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069238961826845161#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr"/>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>2026-06-23 02:19</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D562" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Fulham · Steven Benda — Released</t>
+        </is>
+      </c>
+      <c r="E562" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F562" t="inlineStr">
+        <is>
+          <t>https://www.fulhamfc.com/news/2026/june/08/player-contract-updates/?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
         </is>
       </c>
     </row>
@@ -14700,7 +15807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F64"/>
+  <dimension ref="A1:F68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -16505,6 +17612,114 @@
         </is>
       </c>
     </row>
+    <row r="65">
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>2026-06-22 15:01</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>Enzo Maresca and Manchester City, since May 19. Never in doubt and already 100% involved in transfer strategies. 🔵✅</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>deal, verbal agreement, HERE WE GO, Here we go!, Here We Go, here we go</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069061509276217793#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>2026-06-22 15:01</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>RT by @FabrizioRomano: 🚨🔵 BREAKING: Enzo Maresca has a total verbal agreement with Manchester City, HERE WE GO! The Italian manager has always been considered the ideal candidate to replace Pep Guardiola. Deal in place and Maresca will sign an initial three year deal at #MCFC. 🇮🇹 New era, soon.</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>deal, verbal agreement, HERE WE GO, Here we go!, Here We Go, here we go</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2056633452808847612#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>2026-06-22 17:01</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>Adjunto de Farioli associado ao cargo de treinador do Anderlecht</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>transferência, novo treinador, negocia</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/cronologia/6373897a0cf2254fb2824fe4#Adjunto de Farioli associado ao cargo de</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>2026-06-22 22:01</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>Álvarez quer sair do Atlético: «O melhor para todos é uma transferência»</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>transferência, apontado, apontados</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/espanha/mercado/julian-alvarez-admite-saida-do-atletico-o-melhor-para-todos-e-uma-transferencia</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -16516,7 +17731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:F50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -17820,6 +19035,87 @@
       <c r="F47" t="inlineStr">
         <is>
           <t>https://maisfutebol.iol.pt/mundial-2026/mundial2026/nico-schlotterbeck-sofreu-lesao-ligamentar-nao-parece-nada-bom</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2026-06-22 15:01</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>X:@David_Ornstein</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>🚨 Tino Livramento to miss World Cup with calf injury. Not serious but major blow for Newcastle United defender &amp; #England ahead of #2026FIFAWorldCup opener vs #Croatia - 23yo returning to #NUFC + Trevoh Chalobah called up @TheAthleticFC post @Matt_Law_DT https://www.nytimes.com/athletic/7365471/2026</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>miss world cup, injury, calf injury, injury, miss world cup</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>https://nitter.net/David_Ornstein/status/2066854654982463927#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>2026-06-22 17:01</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>X:@England</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Out for our final session before returning to action 🤩</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>out for</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>https://nitter.net/England/status/2069096807972454751#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>2026-06-22 21:01</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>🚨🇦🇷 Cuti Romero’s injury, not expected to be serious — reports @TyCSports. 🔋</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>injury, injury</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069157902082838534#m</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker refresh · BRA + MAR qualify R32 · Memo Ochoa farewell · Aston Villa interested Jardim LB
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Transfer_Tracker.xlsx
+++ b/Transfer_Tracker.xlsx
@@ -500,7 +500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F562"/>
+  <dimension ref="A1:F675"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -15741,7 +15741,6 @@
       </c>
     </row>
     <row r="561">
-      <c r="A561" t="inlineStr"/>
       <c r="B561" t="inlineStr">
         <is>
           <t>2026-06-23 02:19</t>
@@ -15769,7 +15768,6 @@
       </c>
     </row>
     <row r="562">
-      <c r="A562" t="inlineStr"/>
       <c r="B562" t="inlineStr">
         <is>
           <t>2026-06-23 02:19</t>
@@ -15793,6 +15791,3058 @@
       <c r="F562" t="inlineStr">
         <is>
           <t>https://www.fulhamfc.com/news/2026/june/08/player-contract-updates/?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>2026-06-23 03:01</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D563" s="2" t="inlineStr">
+        <is>
+          <t>🌎🇳🇴 OFFICIAL: Erling Haaland, back to back FIFA Man of the Match in his first two World Cup games.</t>
+        </is>
+      </c>
+      <c r="E563" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F563" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069253086653067324#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>2026-06-23 03:01</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D564" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Brentford · Ryan Trevitt — Released</t>
+        </is>
+      </c>
+      <c r="E564" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F564" t="inlineStr">
+        <is>
+          <t>https://www.brentfordfc.com/en/news/article/first-team-ryan-trevitt-departs-brentford-reiss-nelson-returns-arsenal?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=trans</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>2026-06-23 04:01</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D565" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Tottenham Hotspur · Andy Robertson — Transfer In</t>
+        </is>
+      </c>
+      <c r="E565" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F565" t="inlineStr">
+        <is>
+          <t>https://www.tottenhamhotspur.com/news/1071931/robertson-signing-secured?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>2026-06-23 07:17</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D566" s="2" t="inlineStr">
+        <is>
+          <t>🚨❌ OFFICIAL: Jordan have been ELIMINATED from the 2026 World Cup.</t>
+        </is>
+      </c>
+      <c r="E566" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F566" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069284837446357444#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>2026-06-23 09:29</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D567" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Kévin Boma deixa o Estoril e ruma ao Salzburgo</t>
+        </is>
+      </c>
+      <c r="E567" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, contrato, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F567" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/rb-salzburgo/kevin-boma/oficial-kevin-boma-deixa-o-estoril-e-ruma-ao-salzburgo</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>2026-06-23 09:29</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D568" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Marc Márquez renova com a Ducati até 2028</t>
+        </is>
+      </c>
+      <c r="E568" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F568" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/motogp/motociclismo/oficial-marc-marquez-renova-com-a-ducati-ate-2028</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>2026-06-23 09:29</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D569" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Kévin Boma deixa o Estoril e ruma ao Salzburgo</t>
+        </is>
+      </c>
+      <c r="E569" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F569" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/rb-salzburgo/kevin-boma/oficial-kevin-boma-deixa-o-estoril-e-ruma-ao-salzburgo</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>2026-06-23 09:29</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D570" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Marc Márquez renova com a Ducati até 2028</t>
+        </is>
+      </c>
+      <c r="E570" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F570" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/motogp/motociclismo/oficial-marc-marquez-renova-com-a-ducati-ate-2028</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>2026-06-23 10:30</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D571" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Norberto Alves deixa o comando técnico do Benfica</t>
+        </is>
+      </c>
+      <c r="E571" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F571" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/basquetebol/benfica/oficial-norberto-alves-deixa-o-comando-tecnico-do-benfica</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>2026-06-23 10:30</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D572" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Newcastle · Kieran Trippier — Released</t>
+        </is>
+      </c>
+      <c r="E572" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F572" t="inlineStr">
+        <is>
+          <t>https://www.newcastleunited.com/en/news/kieran-trippier-and-newcastle-united-to-part-ways?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>2026-06-23 11:36</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>X:@David_Ornstein</t>
+        </is>
+      </c>
+      <c r="D573" s="2" t="inlineStr">
+        <is>
+          <t>🚨 Fulham in process of closing deal to appoint Alvaro Arbeloa as new head coach - although #FFC insist 2 candidates remain in contention. Proposed 3yr contract for Spaniard &amp; staff, pending final decisions. W/ @GuillermoRai_ @MarioCortegana @TheAthleticFC https://www.nytimes.com/athletic/7349548/202</t>
+        </is>
+      </c>
+      <c r="E573" s="2" t="inlineStr">
+        <is>
+          <t>deal, new head coach</t>
+        </is>
+      </c>
+      <c r="F573" t="inlineStr">
+        <is>
+          <t>https://nitter.net/David_Ornstein/status/2069366412041220134#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>2026-06-23 11:36</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>X:@BurnleyOfficial</t>
+        </is>
+      </c>
+      <c r="D574" s="2" t="inlineStr">
+        <is>
+          <t>RT by @BurnleyOfficial: Burnley Football Club can announce that Head of Women’s Football Lola Ogunbote will leave her position at the end of June. We wish her every success in the next chapter of her career and thank her for everything she has done since taking on the role in 2021.</t>
+        </is>
+      </c>
+      <c r="E574" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F574" t="inlineStr">
+        <is>
+          <t>https://nitter.net/BurnleyFCWomen/status/2069359811557577056#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>2026-06-23 11:36</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>X:@realmadrid</t>
+        </is>
+      </c>
+      <c r="D575" s="2" t="inlineStr">
+        <is>
+          <t>Comunicado Oficial: operación CVC. https://www.realmadrid.com/es-ES/noticias/club/comunicados/comunicado-oficial-cvc-23-06-2026</t>
+        </is>
+      </c>
+      <c r="E575" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F575" t="inlineStr">
+        <is>
+          <t>https://nitter.net/realmadrid/status/2069378799918010734#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>2026-06-23 11:36</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D576" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Norberto Alves deixa o comando técnico do Benfica</t>
+        </is>
+      </c>
+      <c r="E576" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F576" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/basquetebol/benfica/oficial-norberto-alves-deixa-o-comando-tecnico-do-benfica</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>2026-06-23 13:01</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D577" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Hamza Abdelkarim assina em definitivo pelo Barcelona</t>
+        </is>
+      </c>
+      <c r="E577" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F577" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mundial-2026/mundial2026/oficial-hamza-abdelkarim-assina-em-definitivo-pelo-barcelona</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>2026-06-23 14:01</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D578" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Hamza Abdelkarim assina em definitivo pelo Barcelona</t>
+        </is>
+      </c>
+      <c r="E578" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, contrato, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F578" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mundial-2026/mundial2026/oficial-hamza-abdelkarim-assina-em-definitivo-pelo-barcelona</t>
+        </is>
+      </c>
+    </row>
+    <row r="579">
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>2026-06-23 14:01</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D579" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Gattuso é o novo treinador da Lazio</t>
+        </is>
+      </c>
+      <c r="E579" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, novo treinador, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F579" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/italia/gennaro-gattuso/oficial-gattuso-e-o-novo-treinador-da-lazio</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>2026-06-23 14:01</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D580" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Liverpool · Mohamed Salah — Released</t>
+        </is>
+      </c>
+      <c r="E580" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F580" t="inlineStr">
+        <is>
+          <t>https://www.liverpoolfc.com/news/mohamed-salah-leave-liverpool-end-season?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>2026-06-23 15:01</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D581" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: acionistas do Deportivo Corunha aprovam mudança de nome</t>
+        </is>
+      </c>
+      <c r="E581" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F581" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/espanha/deportivo-corunha/oficial-acionistas-do-deportivo-corunha-aprovam-mudanca-de-nome</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>2026-06-23 15:01</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D582" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Gattuso é o novo treinador da Lazio</t>
+        </is>
+      </c>
+      <c r="E582" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, novo treinador, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F582" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/italia/gennaro-gattuso/oficial-gattuso-e-o-novo-treinador-da-lazio</t>
+        </is>
+      </c>
+    </row>
+    <row r="583">
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>2026-06-23 16:01</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D583" s="2" t="inlineStr">
+        <is>
+          <t>🚨🇵🇹 OFFICIAL: Pedro Neto, João Félix and Cristiano Ronaldo start upfront for Portugal. Nuno Mendes also starts at left back, now fully recovered.</t>
+        </is>
+      </c>
+      <c r="E583" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F583" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069445454664745175#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>2026-06-23 16:01</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>X:@IpswichTown</t>
+        </is>
+      </c>
+      <c r="D584" s="2" t="inlineStr">
+        <is>
+          <t>We are delighted to announce Gary O'Neil as our new Manager. The 43-year-old, who is the 20th manager in the Blues’ 90-year professional history, arrives at Portman Road from French side Strasbourg, signing a three-year deal to the summer of 2029.</t>
+        </is>
+      </c>
+      <c r="E584" s="2" t="inlineStr">
+        <is>
+          <t>we are delighted to announce, are delighted to announce, deal, appointed, new manager</t>
+        </is>
+      </c>
+      <c r="F584" t="inlineStr">
+        <is>
+          <t>https://nitter.net/IpswichTown/status/2069436314597081134#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="585">
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>2026-06-23 16:01</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D585" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Iñaki Peña deixa o Barcelona e ruma ao Panathinaikos</t>
+        </is>
+      </c>
+      <c r="E585" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contratação, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F585" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/grecia/mercado/oficial-inaki-pena-deixa-o-barcelona-e-ruma-ao-panathinaikos</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>2026-06-23 16:01</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D586" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Bernardo Fontes reforça a baliza do Sp. Braga</t>
+        </is>
+      </c>
+      <c r="E586" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contratação, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F586" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/sp-braga/liga/oficial-bernardo-fontes-reforca-a-baliza-do-sp-braga</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>2026-06-23 16:01</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D587" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: melhor jogador da Liga Revelação renova com o Famalicão</t>
+        </is>
+      </c>
+      <c r="E587" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contratação, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F587" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/famalicao/liga/oficial-melhor-jogador-da-liga-revelacao-renova-com-o-famalicao</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>2026-06-23 16:01</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D588" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Gary O´Neil é o novo treinador do Ipswich</t>
+        </is>
+      </c>
+      <c r="E588" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contratação, novo treinador, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F588" t="inlineStr">
+        <is>
+          <t>https://t.co/ZD6cxicPtO</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>2026-06-23 16:01</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D589" s="2" t="inlineStr">
+        <is>
+          <t>Domen Gril anuncia saída do Ac. Viseu: «Cada história tem o seu fim...»</t>
+        </is>
+      </c>
+      <c r="E589" s="2" t="inlineStr">
+        <is>
+          <t>anuncia, saída</t>
+        </is>
+      </c>
+      <c r="F589" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/ii-liga/academico-viseu/domen-gril-anuncia-saida-do-ac-viseu-cada-historia-tem-o-seu-fim</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>2026-06-23 17:01</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D590" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Arsenal · Harrison Dudziak — Released</t>
+        </is>
+      </c>
+      <c r="E590" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F590" t="inlineStr">
+        <is>
+          <t>https://www.arsenal.com/news/contract-updates-15-players-depart-summer?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>2026-06-23 17:01</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D591" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Everton · Isaac Heath — Transfer Out · - Cambridge United</t>
+        </is>
+      </c>
+      <c r="E591" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F591" t="inlineStr">
+        <is>
+          <t>https://www.evertonfc.com/news/2026/june/15/heath-departs-for-cambridge?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch?utm_source=premier-league&amp;utm_med</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>2026-06-23 17:01</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D592" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Fulham · Devan Tanton — Released</t>
+        </is>
+      </c>
+      <c r="E592" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F592" t="inlineStr">
+        <is>
+          <t>https://www.fulhamfc.com/news/2026/june/08/player-contract-updates/?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>2026-06-23 17:01</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D593" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Fulham · Quinn Schutter — Released</t>
+        </is>
+      </c>
+      <c r="E593" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F593" t="inlineStr">
+        <is>
+          <t>https://www.fulhamfc.com/news/2026/june/08/player-contract-updates/?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>2026-06-23 17:01</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D594" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Newcastle · Ewen Jaouen — Transfer In · - Reims</t>
+        </is>
+      </c>
+      <c r="E594" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F594" t="inlineStr">
+        <is>
+          <t>https://www.newcastleunited.com/en/news/ewen-jaouen-signs-for-newcastle-united?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>2026-06-23 17:01</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D595" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Newcastle · Anthony Gordon — Transfer Out · - Barcelona</t>
+        </is>
+      </c>
+      <c r="E595" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F595" t="inlineStr">
+        <is>
+          <t>https://www.newcastleunited.com/en/news/anthony-gordon-signs-for-barcelona?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>2026-06-23 18:07</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D596" s="2" t="inlineStr">
+        <is>
+          <t>🌎🇵🇹 OFFICIAL: Cristiano Ronaldo, the second World Cup oldest goalscorer EVER. Milla, Cristiano Ronaldo and Pepe in the top three.</t>
+        </is>
+      </c>
+      <c r="E596" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F596" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069474465679827371#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>2026-06-23 18:07</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D597" s="2" t="inlineStr">
+        <is>
+          <t>🚨🇵🇹 OFFICIAL: Cristiano Ronaldo equals Eusebio’s record as top goalscorer ever for Portugal at World Cups. 9 goals. 9️⃣⭐️</t>
+        </is>
+      </c>
+      <c r="E597" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F597" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069468002932719731#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>2026-06-23 18:07</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D598" s="2" t="inlineStr">
+        <is>
+          <t>🚨🇵🇹 OFFICIAL: CRISTIANO RONALDO IS THE FIRST PLAYER EVER TO SCORE AT 6 WORLD CUPS.</t>
+        </is>
+      </c>
+      <c r="E598" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F598" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069467261815926797#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>2026-06-23 18:07</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D599" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Iñaki Peña deixa o Barcelona e ruma ao Panathinaikos</t>
+        </is>
+      </c>
+      <c r="E599" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F599" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/grecia/mercado/oficial-inaki-pena-deixa-o-barcelona-e-ruma-ao-panathinaikos</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>2026-06-23 18:07</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D600" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Bernardo Fontes reforça a baliza do Sp. Braga</t>
+        </is>
+      </c>
+      <c r="E600" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, regressa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F600" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/sp-braga/liga/oficial-bernardo-fontes-reforca-a-baliza-do-sp-braga</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>2026-06-23 18:07</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D601" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: melhor jogador da Liga Revelação renova com o Famalicão</t>
+        </is>
+      </c>
+      <c r="E601" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F601" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/famalicao/liga/oficial-melhor-jogador-da-liga-revelacao-renova-com-o-famalicao</t>
+        </is>
+      </c>
+    </row>
+    <row r="602">
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>2026-06-23 18:07</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D602" s="2" t="inlineStr">
+        <is>
+          <t>Domen Gril anuncia saída do Ac. Viseu: «Cada história tem o seu fim...»</t>
+        </is>
+      </c>
+      <c r="E602" s="2" t="inlineStr">
+        <is>
+          <t>anuncia, saída</t>
+        </is>
+      </c>
+      <c r="F602" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/ii-liga/academico-viseu/domen-gril-anuncia-saida-do-ac-viseu-cada-historia-tem-o-seu-fim</t>
+        </is>
+      </c>
+    </row>
+    <row r="603">
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>2026-06-23 18:07</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D603" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Brighton &amp; Hove Albion · Solly March — Released</t>
+        </is>
+      </c>
+      <c r="E603" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F603" t="inlineStr">
+        <is>
+          <t>https://www.brightonandhovealbion.com/media-article/a-letter-to-albion-fans-from-solly-march?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>2026-06-23 19:01</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D604" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: AFC Bournemouth · Marcos Senesi — Released</t>
+        </is>
+      </c>
+      <c r="E604" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F604" t="inlineStr">
+        <is>
+          <t>https://www.afcb.co.uk/news/2026/may/15/senesi-to-depart-in-the-summer/?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>2026-06-23 19:01</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D605" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Brighton &amp; Hove Albion · Zadok Yohanna — Transfer In · - AIK Stockholm</t>
+        </is>
+      </c>
+      <c r="E605" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F605" t="inlineStr">
+        <is>
+          <t>https://www.brightonandhovealbion.com/media-article/mft-signing-albion-agree-deal-to-sign-zadok-yohanna?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>2026-06-23 19:01</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D606" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Fulham · Charlie Robinson — Released</t>
+        </is>
+      </c>
+      <c r="E606" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F606" t="inlineStr">
+        <is>
+          <t>https://www.fulhamfc.com/news/2026/june/08/player-contract-updates/?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>2026-06-23 19:01</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D607" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Tottenham Hotspur · Marcos Senesi — Transfer In</t>
+        </is>
+      </c>
+      <c r="E607" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F607" t="inlineStr">
+        <is>
+          <t>https://www.tottenhamhotspur.com/news/1072863/senesi-switch-sealed?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>2026-06-23 20:01</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D608" s="2" t="inlineStr">
+        <is>
+          <t>🚨🏅 OFFICIAL: Cristiano Ronaldo with FIFA Man of the Match Award today. 💥🇵🇹</t>
+        </is>
+      </c>
+      <c r="E608" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F608" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069503343307657622#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>2026-06-23 20:01</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D609" s="2" t="inlineStr">
+        <is>
+          <t>🌎🇵🇹 OFFICIAL: Cristiano Ronaldo wins Man of the Match Award for Portugal vs Uzbekistan.</t>
+        </is>
+      </c>
+      <c r="E609" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F609" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069498154534240573#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="610">
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>2026-06-24 01:01</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>X:@SEFutbol</t>
+        </is>
+      </c>
+      <c r="D610" s="2" t="inlineStr">
+        <is>
+          <t>RT by @SEFutbol: 🏠🇪🇸 𝗖𝗮𝘀𝗮 𝗘𝘀𝗽𝗮𝗻̃𝗮 abre este miércoles sus puertas en Guadalajara (México) a partir de las 10:00, hora local. ➡️ El presidente de la @rfef inaugurará oficialmente el jueves este punto de encuentro para todos los seguidores de la @SEFutbol. 🔗 https://rfef.es/es/noticias/casa-espana-abr</t>
+        </is>
+      </c>
+      <c r="E610" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIALMENTE, OFICIALMENTE</t>
+        </is>
+      </c>
+      <c r="F610" t="inlineStr">
+        <is>
+          <t>https://nitter.net/rfef/status/2069536071008829618#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="611">
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>2026-06-24 01:01</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D611" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Vítor Bruno é o novo treinador do Anderlecht</t>
+        </is>
+      </c>
+      <c r="E611" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, novo treinador, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F611" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/belgica/treinador/oficial-vitor-bruno-e-o-novo-treinador-do-anderlecht</t>
+        </is>
+      </c>
+    </row>
+    <row r="612">
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>2026-06-24 01:01</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D612" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Vítor Bruno é o novo treinador do Anderlecht</t>
+        </is>
+      </c>
+      <c r="E612" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, contratação, novo treinador, interessado em, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F612" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/belgica/treinador/oficial-vitor-bruno-e-o-novo-treinador-do-anderlecht</t>
+        </is>
+      </c>
+    </row>
+    <row r="613">
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>2026-06-24 01:01</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D613" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Brighton &amp; Hove Albion · Adam Webster — Released</t>
+        </is>
+      </c>
+      <c r="E613" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F613" t="inlineStr">
+        <is>
+          <t>https://www.brightonandhovealbion.com/media-article/webster-to-depart-albion-this-summer?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>2026-06-24 02:01</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D614" s="2" t="inlineStr">
+        <is>
+          <t>🚨❌ OFFICIAL: Panama are OUT the 2026 World Cup.</t>
+        </is>
+      </c>
+      <c r="E614" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F614" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069585067328901330#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>2026-06-24 02:01</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D615" s="2" t="inlineStr">
+        <is>
+          <t>🚨🏴󠁧󠁢󠁥󠁮󠁧󠁿 OFFICIAL: Jude Bellingham, FIFA Man of the Match for England against Ghana.</t>
+        </is>
+      </c>
+      <c r="E615" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F615" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069548038872244269#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="616">
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>2026-06-24 02:01</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D616" s="2" t="inlineStr">
+        <is>
+          <t>🚨🔴⚪️ OFFICIAL: Atlético Madrid to file complaint against Barcelona to FIFA for Julián Álvarez deal. Club CEO Gil Marin: “Our responsibility is to defend the interests of Atlético and that is why we are going to file a complaint with FIFA against Barcelona for negotiating with a player under an activ</t>
+        </is>
+      </c>
+      <c r="E616" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, deal, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F616" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069532449256997090#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="617">
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>2026-06-24 02:01</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D617" s="2" t="inlineStr">
+        <is>
+          <t>🚨🏴󠁧󠁢󠁥󠁮󠁧󠁿 OFFICIAL: Jude Bellingham is the youngest player ever to reach 50 caps with England.</t>
+        </is>
+      </c>
+      <c r="E617" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F617" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069518016685998583#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>2026-06-24 02:01</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D618" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Arsenal · Karl Hein — Transfer Out · Werder Bremen</t>
+        </is>
+      </c>
+      <c r="E618" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F618" t="inlineStr">
+        <is>
+          <t>https://www.arsenal.com/news/karl-hein-join-werder-bremen-permanent-deal?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="619">
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>2026-06-24 02:01</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D619" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Liverpool · Ibrahima Konate — Released</t>
+        </is>
+      </c>
+      <c r="E619" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F619" t="inlineStr">
+        <is>
+          <t>https://www.liverpoolfc.com/news/ibrahima-konate-leave-liverpool-fc?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>2026-06-24 02:01</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D620" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Newcastle · Aaron Ramsdale — End of Loan · - Southampton</t>
+        </is>
+      </c>
+      <c r="E620" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, loan, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F620" t="inlineStr">
+        <is>
+          <t>https://www.newcastleunited.com/en/news/newcastle-united-confirm-mens-first-team-retained-list?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>2026-06-24 02:01</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D621" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Sunderland · Milan Aleksic — loan-out · - Partizan Belgrade</t>
+        </is>
+      </c>
+      <c r="E621" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, loan, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F621" t="inlineStr">
+        <is>
+          <t>https://www.safc.com/news/2026/june/18/milan-aleksi--joins-partizan-belgrade-on-loan/?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>2026-06-24 03:06</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D622" s="2" t="inlineStr">
+        <is>
+          <t>🚨🇧🇷 OFFICIAL: Neymar Jr day at the World Cup, he can play and 100% available. 🔙 “Neymar can play, he’s training very well and he’s ready. I am very happy with him”, says Carlo Ancelotti. ✅</t>
+        </is>
+      </c>
+      <c r="E622" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F622" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069609580397473839#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>2026-06-24 03:06</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D623" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Fulham · Harley Platel — Released</t>
+        </is>
+      </c>
+      <c r="E623" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F623" t="inlineStr">
+        <is>
+          <t>https://www.fulhamfc.com/news/2026/june/08/player-contract-updates/?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>2026-06-24 03:06</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D624" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Liverpool · Carter Pinnington — Transfer Out · - West Brom</t>
+        </is>
+      </c>
+      <c r="E624" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F624" t="inlineStr">
+        <is>
+          <t>https://www.liverpoolfc.com/news/carter-pinnington-joins-west-bromwich-albion?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>2026-06-24 04:08</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D625" s="2" t="inlineStr">
+        <is>
+          <t>🌎🇨🇴 OFFICIAL: Colombia qualify to World Cup Round of 32! 🤩👏🏿</t>
+        </is>
+      </c>
+      <c r="E625" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F625" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069631049764585676#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>2026-06-24 07:27</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D626" s="2" t="inlineStr">
+        <is>
+          <t>🌎🇨🇴 OFFICIAL: Daniel Munoz, Man of the Match for Colombia vs DR Congo.</t>
+        </is>
+      </c>
+      <c r="E626" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F626" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069638739689673065#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>2026-06-24 09:09</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D627" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: ex-V. Guimarães assina por clube da Tunísia</t>
+        </is>
+      </c>
+      <c r="E627" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, contratação, contrato, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F627" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/cronologia/6373897a0cf2254fb2824fe4#OFICIAL: ex-V. Guimarães assina por club</t>
+        </is>
+      </c>
+    </row>
+    <row r="628">
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:02</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D628" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Ipswich · Cedric Kipre — Transfer In · - Reims</t>
+        </is>
+      </c>
+      <c r="E628" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F628" t="inlineStr">
+        <is>
+          <t>https://www.itfc.co.uk/news/2026/may/05/c-dric-makes-move-permanent/?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>2026-06-24 12:08</t>
+        </is>
+      </c>
+      <c r="C629" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D629" s="2" t="inlineStr">
+        <is>
+          <t>🚨🏆 OFFICIAL: Donald Trump and Gianni Infantino to handle World Cup trophy to the winners in New York on final day. “We will be together with the president enjoying the final and handing the trophy to the winner, of course, together”, says Gianni Infantino.</t>
+        </is>
+      </c>
+      <c r="E629" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F629" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069750131889471934#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="630">
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>2026-06-24 12:08</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>X:@David_Ornstein</t>
+        </is>
+      </c>
+      <c r="D630" s="2" t="inlineStr">
+        <is>
+          <t>🚨 EXCL: Leeds United reach agreement to sign Harry Wilson as free agent. 29yo winger targeted by many clubs amid expiring #FFC contract but #LUFC win race - Wales int’l to do medical in due course &amp; join on long-term deal with higher salary @TheAthleticFC https://www.nytimes.com/athletic/7263255/202</t>
+        </is>
+      </c>
+      <c r="E630" s="2" t="inlineStr">
+        <is>
+          <t>deal, free agent</t>
+        </is>
+      </c>
+      <c r="F630" t="inlineStr">
+        <is>
+          <t>https://nitter.net/David_Ornstein/status/2069730252654284944#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>2026-06-24 12:08</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D631" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Eugénio Rodrigues deixa o basquetebol feminino do Benfica</t>
+        </is>
+      </c>
+      <c r="E631" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F631" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/basquetebol/eugenio-rodrigues/oficial-eugenio-rodrigues-deixa-o-basquetebol-feminino-do-benfica</t>
+        </is>
+      </c>
+    </row>
+    <row r="632">
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>2026-06-24 13:01</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D632" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Amara Diouf é reforço do Fenerbahçe</t>
+        </is>
+      </c>
+      <c r="E632" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contratação, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F632" t="inlineStr">
+        <is>
+          <t>https://t.co/nA8c689hqd</t>
+        </is>
+      </c>
+    </row>
+    <row r="633">
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>2026-06-24 13:01</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D633" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Tiago Margarido é o novo treinador do V. Guimarães</t>
+        </is>
+      </c>
+      <c r="E633" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, transferência, novo treinador, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F633" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mercado/24-06-2026/oficial-tiago-margarido-e-o-novo-treinador-do-v-guimaraes</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>2026-06-24 14:00</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D634" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Joaquim Nazaré reforça andebol do Benfica</t>
+        </is>
+      </c>
+      <c r="E634" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, regressa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F634" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/benfica/andebol/oficial-joaquim-nazare-reforca-andebol-do-benfica</t>
+        </is>
+      </c>
+    </row>
+    <row r="635">
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>2026-06-24 14:00</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D635" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Tiago Margarido é o novo treinador do V. Guimarães</t>
+        </is>
+      </c>
+      <c r="E635" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, regressa, novo treinador, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F635" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mercado/24-06-2026/oficial-tiago-margarido-e-o-novo-treinador-do-v-guimaraes</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>2026-06-24 14:00</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D636" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Benfica renova com jovem avançado nigeriano</t>
+        </is>
+      </c>
+      <c r="E636" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contratação, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F636" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/benfica/peter-edokpolor/oficial-benfica-renova-com-jovem-avancado-nigeriano</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>2026-06-24 15:01</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D637" s="2" t="inlineStr">
+        <is>
+          <t>Futsal feminino: Benfica confirma saída de Paulinho Roxo</t>
+        </is>
+      </c>
+      <c r="E637" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, confirma, saída</t>
+        </is>
+      </c>
+      <c r="F637" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/benfica/futsal-feminino/futsal-feminino-benfica-confirma-saida-de-paulinho-roxo</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>2026-06-24 15:01</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D638" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Benfica renova com jovem avançado nigeriano</t>
+        </is>
+      </c>
+      <c r="E638" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F638" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/benfica/peter-edokpolor/oficial-benfica-renova-com-jovem-avancado-nigeriano</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>2026-06-24 15:01</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D639" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Leeds United · Illan Meslier — Released</t>
+        </is>
+      </c>
+      <c r="E639" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F639" t="inlineStr">
+        <is>
+          <t>https://www.leedsunited.com/en/news/illan-meslier-to-leave-leeds-united?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>2026-06-24 15:01</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D640" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Tottenham Hotspur · Martin Dubravka — Transfer In</t>
+        </is>
+      </c>
+      <c r="E640" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F640" t="inlineStr">
+        <is>
+          <t>https://www.tottenhamhotspur.com/news/1074879/dubravka-deal-completed?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>2026-06-24 16:01</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D641" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: melhor jogador da Liga Revelação renova com o Famalicão</t>
+        </is>
+      </c>
+      <c r="E641" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contratação, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F641" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/famalicao/liga/oficial-melhor-jogador-da-liga-revelacao-renova-com-o-famalicao</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>2026-06-24 16:01</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D642" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Liverpool · James Balagizi — Released</t>
+        </is>
+      </c>
+      <c r="E642" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F642" t="inlineStr">
+        <is>
+          <t>https://www.liverpoolfc.com/news/liverpool-confirm-premier-league-retained-list?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>2026-06-24 16:01</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D643" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Man Utd · Casemiro — Released</t>
+        </is>
+      </c>
+      <c r="E643" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F643" t="inlineStr">
+        <is>
+          <t>https://www.manutd.com/en/news/casemiro-to-leave-man-utd-at-the-end-of-the-2025-26-season?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>2026-06-24 17:02</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>X:@Wolves</t>
+        </is>
+      </c>
+      <c r="D644" s="2" t="inlineStr">
+        <is>
+          <t>RT by @Wolves: Welcome to Wolves, Jas Matthews! The former Liverpool defender joins on a two-year deal as our first signing of the summer ✍️ 🔗 http://wolves.short.gy/JasMatthewsSigns</t>
+        </is>
+      </c>
+      <c r="E644" s="2" t="inlineStr">
+        <is>
+          <t>deal, signs, joins</t>
+        </is>
+      </c>
+      <c r="F644" t="inlineStr">
+        <is>
+          <t>https://nitter.net/WolvesWomen/status/2069813787486470374#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>2026-06-24 17:02</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D645" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Diogo Sousa deixa o V. Guimarães e reforça o Estrasburgo</t>
+        </is>
+      </c>
+      <c r="E645" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F645" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/v-guimaraes/liga/oficial-diogo-sousa-deixa-o-v-guimaraes-e-reforca-o-estrasburgo</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>2026-06-24 17:02</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D646" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Dirk Kuyt integra equipa técnica do Fenerbahçe</t>
+        </is>
+      </c>
+      <c r="E646" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F646" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/turquia/fenerbahce/oficial-dirk-kuyt-e-o-novo-treinador-do-fenerbahce</t>
+        </is>
+      </c>
+    </row>
+    <row r="647">
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>2026-06-24 17:02</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D647" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: campeão da Liga 3, Fernando Almeida assina com o AVS</t>
+        </is>
+      </c>
+      <c r="E647" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contratação, chega, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F647" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/cronologia/6373897a0cf2254fb2824fe4#OFICIAL: campeão da Liga 3, Fernando Alm</t>
+        </is>
+      </c>
+    </row>
+    <row r="648">
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>2026-06-24 17:02</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D648" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Diogo Sousa deixa o V. Guimarães e reforça o Estrasburgo</t>
+        </is>
+      </c>
+      <c r="E648" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, contrato, deixa, deverá, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F648" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/v-guimaraes/liga/oficial-diogo-sousa-deixa-o-v-guimaraes-e-reforca-o-estrasburgo</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>2026-06-24 17:02</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D649" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Martin Dubravka a caminho do Tottenham</t>
+        </is>
+      </c>
+      <c r="E649" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F649" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/cronologia/6373897a0cf2254fb2824fe4#OFICIAL: Martin Dubravka a caminho do To</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>2026-06-24 17:02</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D650" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Ipswich · Cedric Kipre — Transfer In · - Reims</t>
+        </is>
+      </c>
+      <c r="E650" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F650" t="inlineStr">
+        <is>
+          <t>https://www.itfc.co.uk/news/2026/may/05/c-dric-makes-move-permanent/?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>2026-06-24 17:02</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D651" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Liverpool · Jacob Poytress — Released</t>
+        </is>
+      </c>
+      <c r="E651" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F651" t="inlineStr">
+        <is>
+          <t>https://www.liverpoolfc.com/news/liverpool-confirm-premier-league-retained-list?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>2026-06-24 17:02</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D652" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Man Utd · Jadon Sancho — Released</t>
+        </is>
+      </c>
+      <c r="E652" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F652" t="inlineStr">
+        <is>
+          <t>https://www.manutd.com/en/news/uniteds-retained-list-and-released-players?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>2026-06-24 23:01</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D653" s="2" t="inlineStr">
+        <is>
+          <t>🚨🌎 OFFICIAL: Switzerland win Group B, Canada also fly to World Cup round of 32!</t>
+        </is>
+      </c>
+      <c r="E653" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F653" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069889000718918032#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>2026-06-24 23:01</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D654" s="2" t="inlineStr">
+        <is>
+          <t>🌎🇨🇦 OFFICIAL: Canada qualify to World Cup round of 32!</t>
+        </is>
+      </c>
+      <c r="E654" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F654" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069888732266643901#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>2026-06-24 23:01</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D655" s="2" t="inlineStr">
+        <is>
+          <t>🚨🇨🇭 OFFICIAL: Switzerland qualify to World Cup Round of 32! 🌎</t>
+        </is>
+      </c>
+      <c r="E655" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F655" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069888665279414617#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>2026-06-24 23:01</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D656" s="2" t="inlineStr">
+        <is>
+          <t>🚨❌ OFFICIAL: Qatar are OUT of the 2026 World Cup.</t>
+        </is>
+      </c>
+      <c r="E656" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F656" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069888540989612373#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>2026-06-24 23:01</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D657" s="2" t="inlineStr">
+        <is>
+          <t>🚨🇧🇷 OFFICIAL: Endrick and Neymar Jr are both on the bench for Brazil against Scotland.</t>
+        </is>
+      </c>
+      <c r="E657" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F657" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069881599051620462#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>2026-06-24 23:01</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D658" s="2" t="inlineStr">
+        <is>
+          <t>Paulinho Bóia despede-se do Nacional após época e meia na Madeira</t>
+        </is>
+      </c>
+      <c r="E658" s="2" t="inlineStr">
+        <is>
+          <t>anunciou, contratação, chega</t>
+        </is>
+      </c>
+      <c r="F658" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/liga/nacional/paulinho-boia-despede-se-do-nacional-apos-epoca-e-meia-na-madeira</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>2026-06-24 23:01</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D659" s="2" t="inlineStr">
+        <is>
+          <t>Tiago Fernandes regressa ao Sporting para comandar a equipa B</t>
+        </is>
+      </c>
+      <c r="E659" s="2" t="inlineStr">
+        <is>
+          <t>anunciou, contratação, chega, regressa</t>
+        </is>
+      </c>
+      <c r="F659" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/sporting/tiago-fernandes/tiago-fernandes-regressa-ao-sporting-para-comandar-a-equipa-b</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>2026-06-24 23:01</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D660" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Ipswich · Leon Ayinde — Transfer Out · - Doncaster</t>
+        </is>
+      </c>
+      <c r="E660" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F660" t="inlineStr">
+        <is>
+          <t>https://www.itfc.co.uk/news/2026/may/20/leon-ayinde-to-join-doncaster/?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>2026-06-24 23:01</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D661" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Tottenham Hotspur · Martin Dubravka — Transfer In</t>
+        </is>
+      </c>
+      <c r="E661" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F661" t="inlineStr">
+        <is>
+          <t>https://www.tottenhamhotspur.com/news/1074879/dubravka-deal-completed?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>2026-06-25 00:01</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D662" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Benfica anuncia saída de Cristina Martín-Prieto</t>
+        </is>
+      </c>
+      <c r="E662" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anuncia, saída, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F662" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/benfica/futebol-feminino/oficial-benfica-anuncia-saida-de-cristina-martin-prieto</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>2026-06-25 00:01</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D663" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Benfica anuncia saída de Cristina Martín-Prieto</t>
+        </is>
+      </c>
+      <c r="E663" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anuncia, anunciou, contratação, saída, chega</t>
+        </is>
+      </c>
+      <c r="F663" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/benfica/futebol-feminino/oficial-benfica-anuncia-saida-de-cristina-martin-prieto</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>2026-06-25 00:01</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D664" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Gattuso é o novo treinador da Lazio</t>
+        </is>
+      </c>
+      <c r="E664" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, novo treinador, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F664" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/italia/gennaro-gattuso/oficial-gattuso-e-o-novo-treinador-da-lazio</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>2026-06-25 00:01</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D665" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Brighton &amp; Hove Albion · James Milner — Released</t>
+        </is>
+      </c>
+      <c r="E665" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F665" t="inlineStr">
+        <is>
+          <t>https://www.brightonandhovealbion.com/media-article/albion-pay-tribute-to-james-milner-after-retirement-announcement?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=tra</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>2026-06-25 00:01</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D666" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Fulham · Olly Sanderson — Transfer Out · - Stevenage</t>
+        </is>
+      </c>
+      <c r="E666" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F666" t="inlineStr">
+        <is>
+          <t>https://www.fulhamfc.com/news/2026/june/13/olly-sanderson-departs/</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>2026-06-25 00:01</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D667" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Newcastle · Emil Krafth — Released</t>
+        </is>
+      </c>
+      <c r="E667" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F667" t="inlineStr">
+        <is>
+          <t>https://www.newcastleunited.com/en/news/emil-krafth-to-depart-newcastle-united-this-summer?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>2026-06-25 00:01</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D668" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Sunderland · Milan Aleksic — loan-out · - Partizan Belgrade</t>
+        </is>
+      </c>
+      <c r="E668" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, loan, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F668" t="inlineStr">
+        <is>
+          <t>https://www.safc.com/news/2026/june/18/milan-aleksi--joins-partizan-belgrade-on-loan/?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>2026-06-25 01:00</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D669" s="2" t="inlineStr">
+        <is>
+          <t>🌎🇧🇷 OFFICIAL: Vini Jr, back to back to back FIFA Man of the Match for Brazil. Three in a row. 🥇🇲🇦 Brazil vs Morocco: 𝐅𝐈𝐅𝐀 𝐌𝐎𝐓𝐌 🥇🇭🇹 Brazil vs Haiti: 𝐅𝐈𝐅𝐀 𝐌𝐎𝐓𝐌 🥇🏴󠁧󠁢󠁳󠁣󠁴󠁿 Brazil vs Scotland: 𝐅𝐈𝐅𝐀 𝐌𝐎𝐓𝐌</t>
+        </is>
+      </c>
+      <c r="E669" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F669" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069941133757571418#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>2026-06-25 01:00</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D670" s="2" t="inlineStr">
+        <is>
+          <t>🌎🇲🇦 OFFICIAL: Achraf Hakimi, FIFA Man of the Match for Morocco.</t>
+        </is>
+      </c>
+      <c r="E670" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F670" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069940962151809122#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>2026-06-25 01:00</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D671" s="2" t="inlineStr">
+        <is>
+          <t>🌎🇧🇷🇲🇦 OFFICIAL: Brazil win their group as they qualify with Morocco to Round of 32!</t>
+        </is>
+      </c>
+      <c r="E671" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F671" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069934361412067651#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>2026-06-25 01:00</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D672" s="2" t="inlineStr">
+        <is>
+          <t>🌎🇧🇷 OFFICIAL: Brazil qualify to FIFA World Cup Round of 32. ✈️</t>
+        </is>
+      </c>
+      <c r="E672" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F672" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069933991822504248#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>2026-06-25 01:00</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D673" s="2" t="inlineStr">
+        <is>
+          <t>🌎🇲🇦 OFFICIAL: Morocco qualify to World Cup round of 32!</t>
+        </is>
+      </c>
+      <c r="E673" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F673" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069933569670103313#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>2026-06-25 02:01</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D674" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Fulham · Harley Platel — Released</t>
+        </is>
+      </c>
+      <c r="E674" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F674" t="inlineStr">
+        <is>
+          <t>https://www.fulhamfc.com/news/2026/june/08/player-contract-updates/?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr"/>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>2026-06-25 02:58</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D675" s="2" t="inlineStr">
+        <is>
+          <t>👏🏼🇲🇽 OFFICIAL: Memo Ochoa plays his likely-to-be last career game now featuring at 6th World Cup with Mexico. The 40-year old goalkeeper plans to retire after this achievement. Magic moment at the legendary Azteca.</t>
+        </is>
+      </c>
+      <c r="E675" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F675" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069974955937108461#m</t>
         </is>
       </c>
     </row>
@@ -15807,7 +18857,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F68"/>
+  <dimension ref="A1:F81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -17720,6 +20770,357 @@
         </is>
       </c>
     </row>
+    <row r="69">
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>2026-06-23 15:01</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>Vítor Bruno a caminho do Anderlecht</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>deixa, perto de</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mercado/vitor-bruno/vitor-bruno-a-caminho-do-anderlecht</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>2026-06-23 18:07</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>Aston Villa interessado em lateral de Leonardo Jardim</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>contratação, interessado em</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/cronologia/6373897a0cf2254fb2824fe4#Aston Villa interessado em lateral de Le</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>2026-06-23 20:01</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>X:@David_Ornstein</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>🚨 Ipswich Town working to finalise appointment of Gary O’Neil as head coach. #ITFC in positive talks with 43yo + BlueCo; possible announcement early next. Well regarded for work at #AFCB #WWFC #RCSA. Would bring Tim Jenkins + Neil Critchley @TheAthleticFC https://www.nytimes.com/athletic/7352726/202</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>new head coach, talks, talks with</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>https://nitter.net/David_Ornstein/status/2068054550523617302#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>2026-06-24 01:01</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>X:@FCBayern</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>Here we go again, wird ne lange Nacht für den Admin. 😄</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>HERE WE GO, Here We Go, here we go</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FCBayern/status/2069512552740966510#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>2026-06-24 09:09</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>🚨🔵 BREAKING: Marco Palestra to Chelsea, here we go! Verbal agreement in place between all parties. Atalanta to receive package over €55m fee plus sell-on clause, long term deal to Italian talented RWB. Chelsea hijack Inter move and get new talent for Xabi Alonso.</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>deal, verbal agreement, HERE WE GO, Here we go!, Here We Go, here we go</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069669349489828237#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>2026-06-24 12:08</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>RT by @FabrizioRomano: 🚨 Martin Dubravka to Tottenham, here we go! Deal agreed for former Burnley and Man United goalkeeper to join #THFC. Move completed today with Dubravka set to be backup GK at Spurs behind Kinski. 🔃🇸🇰 Guglielmo Vicario to leave this summer.</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>agreed, deal, HERE WE GO, Here we go!, Here We Go, here we go</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069729744170475729#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>2026-06-24 12:08</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>RT by @FabrizioRomano: 🚨🔵 BREAKING: Marco Palestra to Chelsea, here we go! Verbal agreement in place between all parties. Atalanta to receive package over €55m fee plus sell-on clause, long term deal to Italian talented RWB. Chelsea hijack Inter move and get new talent for Xabi Alonso.</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>deal, verbal agreement, HERE WE GO, Here we go!, Here We Go, here we go</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069669349489828237#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>2026-06-24 17:02</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>RT by @FabrizioRomano: 🚨❤️🤍 Alejandro Grimaldo to Atlético Madrid, here we go! Verbal agreement in place between all parties. Bayer Leverkusen accept final proposal worth over €20m as total package with add-ons. Grimaldo only wanted Atléti, personal terms agreed last week — and deal now in place.</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>agreed, deal, verbal agreement, HERE WE GO, Here we go!, Here We Go</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069814044031078708#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>2026-06-24 17:02</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>Sporting: Altimira praticamente fechado, valores podem chegar aos 20 milhões</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>chega, deverá</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/sporting/transferencias/sporting-altimira-fechado-valores-podem-chegar-aos-20-milhoes</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>2026-06-24 17:02</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>Sporting: Altimira praticamente fechado, valores podem chegar aos 20 milhões</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>contrato, chega, deverá</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/sporting/transferencias/sporting-altimira-fechado-valores-podem-chegar-aos-20-milhoes</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>2026-06-24 17:02</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>Chelsea desvia Palestra do Inter</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>contrato, deverá</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>https://x.com/hashtag/CFC?src=hash&amp;ref_src=twsrc%5Etfw</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>2026-06-24 23:01</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>Here we go @McDonalds! Big Mac sauce is 🔥</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>HERE WE GO, Here We Go, here we go</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069888166178299942#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>2026-06-25 00:01</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>Aston Villa interessado em lateral de Leonardo Jardim</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>contratação, interessado em</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/cronologia/6373897a0cf2254fb2824fe4#Aston Villa interessado em lateral de Le</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -17731,7 +21132,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F50"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -19116,6 +22517,195 @@
       <c r="F50" t="inlineStr">
         <is>
           <t>https://nitter.net/FabrizioRomano/status/2069157902082838534#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>2026-06-23 07:17</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>🚨 Kylian Mbappé: “I tried to have the best season possible at Real Madrid. The injury in January didn’t help me, but then I returned in the best shape”. “The World Cup is important for every player, of course”, told @AbrahamPRomero.</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>injury, injury</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069305451804836327#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2026-06-23 11:36</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>🚨 Kylian Mbappé: “I tried to have the best season possible at Real Madrid. The injury in January didn’t help me, but then I returned in the best shape”. “The World Cup is important for every player, of course”, told @AbrahamPRomero.</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>injury, injury</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069305451804836327#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:02</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Jogadores envolvidos na lesão mais grave do Mundial reencontram-se fora de campo</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>lesão, lesão</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mundial-2026/mundial2026/jogadores-envolvidos-na-lesao-mais-grave-do-mundial-reencontram-se-fora-de-campo</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2026-06-24 12:08</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>X:@NUFC</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Tino Livramento has withdrawn from @England's #FIFAWorldCup 2026 squad. The 23-year-old picked up a minor calf injury in training with the Three Lions on Sunday afternoon. A subsequent scan and medical assessment on Monday unfortunately confirmed he could play no further part in England's tournament</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>withdrawn from, injury, calf injury, confirmed, withdrawn from, injury</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>https://nitter.net/NUFC/status/2066875900944056421#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>2026-06-24 12:08</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Mundial 2026: Senegal com baixa de peso na baliza</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>lesionou-se</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mundial-2026/mundial2026/mundial2026-senegal-com-baixa-de-peso-na-baliza</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>2026-06-24 14:00</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>X:@NUFC</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Tino Livramento has withdrawn from @England's #FIFAWorldCup 2026 squad. The 23-year-old picked up a minor calf injury in training with the Three Lions on Sunday afternoon. A subsequent scan and medical assessment on Monday unfortunately confirmed he could play no further part in England's tournament</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>withdrawn from, injury, calf injury, confirmed, withdrawn from, injury</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>https://nitter.net/NUFC/status/2066875900944056421#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>2026-06-24 23:01</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Mundial 2026: FIFA castiga Madibo com cinco jogos após lesão grave de Koné</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>lesão, lesão</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mundial-2026/qatar/fifa-castiga-madibo-com-cinco-jogos-apos-lesao-grave-de-kone</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker refresh Thu 25 Jun · PL retained lists incoming: Salah · Senesi · Coleman · Targett · Thompson all released
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Transfer_Tracker.xlsx
+++ b/Transfer_Tracker.xlsx
@@ -500,7 +500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F675"/>
+  <dimension ref="A1:F738"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -18819,7 +18819,6 @@
       </c>
     </row>
     <row r="675">
-      <c r="A675" t="inlineStr"/>
       <c r="B675" t="inlineStr">
         <is>
           <t>2026-06-25 02:58</t>
@@ -18843,6 +18842,1709 @@
       <c r="F675" t="inlineStr">
         <is>
           <t>https://nitter.net/FabrizioRomano/status/2069974955937108461#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>2026-06-25 04:02</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D676" s="2" t="inlineStr">
+        <is>
+          <t>🚨🇨🇦🇿🇦 OFFICIAL: Canada 🆚 South Africa in World Cup Round of 32.</t>
+        </is>
+      </c>
+      <c r="E676" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F676" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069981514171859376#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>2026-06-25 04:02</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D677" s="2" t="inlineStr">
+        <is>
+          <t>🌎🇲🇽 OFFICIAL: Mexico qualify for World Cup round of 32 after 3/3 wins! ✈️</t>
+        </is>
+      </c>
+      <c r="E677" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F677" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069979128925691958#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="678">
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>2026-06-25 04:02</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D678" s="2" t="inlineStr">
+        <is>
+          <t>🌎🇿🇦 OFFICIAL: South Africa make history and qualify to World Cup round of 32! 💥</t>
+        </is>
+      </c>
+      <c r="E678" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F678" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069978993147678723#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>2026-06-25 04:02</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D679" s="2" t="inlineStr">
+        <is>
+          <t>🚨❌ OFFICIAL: Czech Republic are OUT of the 2026 World Cup.</t>
+        </is>
+      </c>
+      <c r="E679" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F679" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2069978927838204223#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>2026-06-25 04:02</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D680" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Ipswich · Cedric Kipre — Transfer In · - Reims</t>
+        </is>
+      </c>
+      <c r="E680" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F680" t="inlineStr">
+        <is>
+          <t>https://www.itfc.co.uk/news/2026/may/05/c-dric-makes-move-permanent/?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>2026-06-25 06:25</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D681" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Liverpool · Jeremy Jacquet — Transfer In · - Rennes</t>
+        </is>
+      </c>
+      <c r="E681" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F681" t="inlineStr">
+        <is>
+          <t>https://www.liverpoolfc.com/news/liverpool-agree-deal-sign-jeremy-jacquet?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>2026-06-25 10:46</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D682" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Djibril Soumaré deixa Sp. Braga em definitivo e ruma ao Stoke</t>
+        </is>
+      </c>
+      <c r="E682" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F682" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/sp-braga/djibril-soumare/oficial-djibril-soumare-deixa-sp-braga-em-definitivo-e-ruma-ao-stoke</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>2026-06-25 10:46</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D683" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Djibril Soumaré deixa Sp. Braga e rende quatro milhões</t>
+        </is>
+      </c>
+      <c r="E683" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contratação, contrato, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F683" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/sp-braga/djibril-soumare/oficial-djibril-soumare-deixa-sp-braga-em-definitivo-e-ruma-ao-stoke</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>2026-06-25 10:46</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D684" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Youssef El Kachati é reforço do Stade de Reims</t>
+        </is>
+      </c>
+      <c r="E684" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contratação, contrato, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F684" t="inlineStr">
+        <is>
+          <t>https://x.com/StadeDeReims/status/2070074519478260216?ref_src=twsrc%5Etfw</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>2026-06-25 10:46</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D685" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: AFC Bournemouth · Michael Dacosta Gonzalez — Transfer Out · - Moreirense</t>
+        </is>
+      </c>
+      <c r="E685" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F685" t="inlineStr">
+        <is>
+          <t>https://www.afcb.co.uk/news/2026/june/15/dacosta-gonzalez-completes-moreirense-switch/?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="686">
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>2026-06-25 11:45</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>X:@LCFC</t>
+        </is>
+      </c>
+      <c r="D686" s="2" t="inlineStr">
+        <is>
+          <t>Our full fixture list confirmed for 26/27 🦊</t>
+        </is>
+      </c>
+      <c r="E686" s="2" t="inlineStr">
+        <is>
+          <t>⚠️ FOLLOW-UP CLICK LINK, confirmed, release, released</t>
+        </is>
+      </c>
+      <c r="F686" t="inlineStr">
+        <is>
+          <t>https://nitter.net/LCFC/status/2070099690394362295#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>2026-06-25 11:45</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>X:@BurnleyOfficial</t>
+        </is>
+      </c>
+      <c r="D687" s="2" t="inlineStr">
+        <is>
+          <t>All of our @EFL Championship fixtures for 2026/27</t>
+        </is>
+      </c>
+      <c r="E687" s="2" t="inlineStr">
+        <is>
+          <t>confirmed, release</t>
+        </is>
+      </c>
+      <c r="F687" t="inlineStr">
+        <is>
+          <t>https://nitter.net/BurnleyOfficial/status/2070099879288799405#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="688">
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>2026-06-25 11:45</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D688" s="2" t="inlineStr">
+        <is>
+          <t>Grimaldo confirma conversas para reforçar o Atlético de Madrid</t>
+        </is>
+      </c>
+      <c r="E688" s="2" t="inlineStr">
+        <is>
+          <t>confirma, deixa, deverá</t>
+        </is>
+      </c>
+      <c r="F688" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/internacional/espanha/grimaldo-confirma-conversas-para-reforcar-o-atletico-de-madrid</t>
+        </is>
+      </c>
+    </row>
+    <row r="689">
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>2026-06-25 11:45</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D689" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Djibril Soumaré deixa Sp. Braga e rende quatro milhões</t>
+        </is>
+      </c>
+      <c r="E689" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F689" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/sp-braga/djibril-soumare/oficial-djibril-soumare-deixa-sp-braga-em-definitivo-e-ruma-ao-stoke</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>2026-06-25 11:45</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D690" s="2" t="inlineStr">
+        <is>
+          <t>Grimaldo confirma conversas para reforçar o Atlético de Madrid</t>
+        </is>
+      </c>
+      <c r="E690" s="2" t="inlineStr">
+        <is>
+          <t>confirma, anunciou, contratação, contrato</t>
+        </is>
+      </c>
+      <c r="F690" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/internacional/espanha/grimaldo-confirma-conversas-para-reforcar-o-atletico-de-madrid</t>
+        </is>
+      </c>
+    </row>
+    <row r="691">
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>2026-06-25 11:45</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D691" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Everton · Idrissa Gana Gueye — Released</t>
+        </is>
+      </c>
+      <c r="E691" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F691" t="inlineStr">
+        <is>
+          <t>https://www.evertonfc.com/news/2026/june/10/everton-player-contracts-update/?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="692">
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>2026-06-25 11:45</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D692" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Fulham · Marcell Hall — Released</t>
+        </is>
+      </c>
+      <c r="E692" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F692" t="inlineStr">
+        <is>
+          <t>https://www.fulhamfc.com/news/2026/june/08/player-contract-updates/?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="693">
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>2026-06-25 11:45</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D693" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Sunderland · Bertrand Traore — Released</t>
+        </is>
+      </c>
+      <c r="E693" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F693" t="inlineStr">
+        <is>
+          <t>https://www.safc.com/news/2026/june/10/sunderland-afc-announce-retained-list-for-2026-27/?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="694">
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>2026-06-25 12:15</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D694" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: ex-Sporting Jesé renova com Las Palmas até 2028</t>
+        </is>
+      </c>
+      <c r="E694" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contrato, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F694" t="inlineStr">
+        <is>
+          <t>https://t.co/AZ8lLzeRHB</t>
+        </is>
+      </c>
+    </row>
+    <row r="695">
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>2026-06-25 12:15</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D695" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Dani Figueira deixa Gil Vicente e ruma à Arménia</t>
+        </is>
+      </c>
+      <c r="E695" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contratação, contrato, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F695" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/liga/gil-vicente/oficial-dani-figueira-deixa-gil-vicente-e-ruma-a-armenia</t>
+        </is>
+      </c>
+    </row>
+    <row r="696">
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>2026-06-25 12:15</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D696" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: ex-V. Guimarães assina por clube da Tunísia</t>
+        </is>
+      </c>
+      <c r="E696" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, contratação, contrato, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F696" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/cronologia/6373897a0cf2254fb2824fe4#OFICIAL: ex-V. Guimarães assina por club</t>
+        </is>
+      </c>
+    </row>
+    <row r="697">
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>2026-06-25 12:15</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D697" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Leeds United · Sam Byram — Released</t>
+        </is>
+      </c>
+      <c r="E697" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F697" t="inlineStr">
+        <is>
+          <t>https://www.leedsunited.com/en/news/leeds-united-2026-27-retained-list?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="698">
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>2026-06-25 13:01</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>X:@LCFC</t>
+        </is>
+      </c>
+      <c r="D698" s="2" t="inlineStr">
+        <is>
+          <t>Pinned: Our full fixture list confirmed for 26/27 🦊</t>
+        </is>
+      </c>
+      <c r="E698" s="2" t="inlineStr">
+        <is>
+          <t>⚠️ FOLLOW-UP CLICK LINK, confirmed, release, released</t>
+        </is>
+      </c>
+      <c r="F698" t="inlineStr">
+        <is>
+          <t>https://nitter.net/LCFC/status/2070099690394362295#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="699">
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>2026-06-25 13:01</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D699" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Dani Figueira deixa Gil Vicente e ruma à Arménia</t>
+        </is>
+      </c>
+      <c r="E699" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F699" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/liga/gil-vicente/oficial-dani-figueira-deixa-gil-vicente-e-ruma-a-armenia</t>
+        </is>
+      </c>
+    </row>
+    <row r="700">
+      <c r="B700" t="inlineStr">
+        <is>
+          <t>2026-06-25 13:01</t>
+        </is>
+      </c>
+      <c r="C700" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D700" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Benfica renova com jovem avançado nigeriano</t>
+        </is>
+      </c>
+      <c r="E700" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contratação, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F700" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/benfica/peter-edokpolor/oficial-benfica-renova-com-jovem-avancado-nigeriano</t>
+        </is>
+      </c>
+    </row>
+    <row r="701">
+      <c r="B701" t="inlineStr">
+        <is>
+          <t>2026-06-25 13:01</t>
+        </is>
+      </c>
+      <c r="C701" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D701" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Tottenham Hotspur · Andy Robertson — Transfer In</t>
+        </is>
+      </c>
+      <c r="E701" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F701" t="inlineStr">
+        <is>
+          <t>https://www.tottenhamhotspur.com/news/1071931/robertson-signing-secured?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="702">
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>2026-06-25 14:01</t>
+        </is>
+      </c>
+      <c r="C702" t="inlineStr">
+        <is>
+          <t>X:@premierleague</t>
+        </is>
+      </c>
+      <c r="D702" s="2" t="inlineStr">
+        <is>
+          <t>RT by @premierleague: Hincapie's here to stay 🇪🇨 The club is delighted to announce that Piero has signed a permanent deal at The Arsenal 👊</t>
+        </is>
+      </c>
+      <c r="E702" s="2" t="inlineStr">
+        <is>
+          <t>deal, signed, joins</t>
+        </is>
+      </c>
+      <c r="F702" t="inlineStr">
+        <is>
+          <t>https://nitter.net/Arsenal/status/2070130082677662002#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="703">
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>2026-06-25 14:01</t>
+        </is>
+      </c>
+      <c r="C703" t="inlineStr">
+        <is>
+          <t>X:@Arsenal</t>
+        </is>
+      </c>
+      <c r="D703" s="2" t="inlineStr">
+        <is>
+          <t>Hincapie's here to stay 🇪🇨 The club is delighted to announce that Piero has signed a permanent deal at The Arsenal 👊</t>
+        </is>
+      </c>
+      <c r="E703" s="2" t="inlineStr">
+        <is>
+          <t>deal, signed, joins</t>
+        </is>
+      </c>
+      <c r="F703" t="inlineStr">
+        <is>
+          <t>https://nitter.net/Arsenal/status/2070130082677662002#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="704">
+      <c r="B704" t="inlineStr">
+        <is>
+          <t>2026-06-25 14:01</t>
+        </is>
+      </c>
+      <c r="C704" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D704" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Arsenal contrata Piero Hincapié em definitivo</t>
+        </is>
+      </c>
+      <c r="E704" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F704" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/inglaterra/arsenal/oficial-arsenal-segura-contratacao-de-hincapie-em-definitivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="705">
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>2026-06-25 14:01</t>
+        </is>
+      </c>
+      <c r="C705" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D705" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: ex-Benfica Gilberto troca de clube no Brasileirão</t>
+        </is>
+      </c>
+      <c r="E705" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F705" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/internacional/brasil/oficial-ex-benfica-gilberto-troca-de-clube-no-brasileirao</t>
+        </is>
+      </c>
+    </row>
+    <row r="706">
+      <c r="B706" t="inlineStr">
+        <is>
+          <t>2026-06-25 14:01</t>
+        </is>
+      </c>
+      <c r="C706" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D706" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Gabriel Souza troca Tondela pelo Lusitânia de Lourosa</t>
+        </is>
+      </c>
+      <c r="E706" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contratação, contrato, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F706" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DaAaOLgDLhN/?utm_source=ig_embed&amp;utm_campaign=loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="707">
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>2026-06-25 14:01</t>
+        </is>
+      </c>
+      <c r="C707" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D707" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Benfica confirma saída de Christy Ucheibe</t>
+        </is>
+      </c>
+      <c r="E707" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, confirma, anunciou, contrato, saída, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F707" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/futebol-feminino/feminino/oficial-benfica-confirma-saida-de-christy-ucheibe</t>
+        </is>
+      </c>
+    </row>
+    <row r="708">
+      <c r="B708" t="inlineStr">
+        <is>
+          <t>2026-06-25 14:01</t>
+        </is>
+      </c>
+      <c r="C708" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D708" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Fraser Forster renova com o Bournemouth por mais uma época</t>
+        </is>
+      </c>
+      <c r="E708" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contrato, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F708" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/cronologia/6373897a0cf2254fb2824fe4#OFICIAL: Fraser Forster renova com o Bou</t>
+        </is>
+      </c>
+    </row>
+    <row r="709">
+      <c r="B709" t="inlineStr">
+        <is>
+          <t>2026-06-25 14:01</t>
+        </is>
+      </c>
+      <c r="C709" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D709" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Arsenal contrata Piero Hincapié em definitivo</t>
+        </is>
+      </c>
+      <c r="E709" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contrato, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F709" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/inglaterra/arsenal/oficial-arsenal-segura-contratacao-de-hincapie-em-definitivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="710">
+      <c r="B710" t="inlineStr">
+        <is>
+          <t>2026-06-25 14:01</t>
+        </is>
+      </c>
+      <c r="C710" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D710" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: ex-Benfica Gilberto troca de clube no Brasileirão</t>
+        </is>
+      </c>
+      <c r="E710" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contrato, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F710" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/internacional/brasil/oficial-ex-benfica-gilberto-troca-de-clube-no-brasileirao</t>
+        </is>
+      </c>
+    </row>
+    <row r="711">
+      <c r="B711" t="inlineStr">
+        <is>
+          <t>2026-06-25 14:01</t>
+        </is>
+      </c>
+      <c r="C711" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D711" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Arsenal · Piero Hincapie — Transfer In · Bayer Leverkusen</t>
+        </is>
+      </c>
+      <c r="E711" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F711" t="inlineStr">
+        <is>
+          <t>https://www.arsenal.com/news/piero-hincapie-joins-arsenal-permanent-deal?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="712">
+      <c r="B712" t="inlineStr">
+        <is>
+          <t>2026-06-25 14:01</t>
+        </is>
+      </c>
+      <c r="C712" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D712" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Brentford · Reiss Nelson — End of Loan · - Arsenal</t>
+        </is>
+      </c>
+      <c r="E712" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, loan, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F712" t="inlineStr">
+        <is>
+          <t>https://www.brentfordfc.com/en/news/article/first-team-ryan-trevitt-departs-brentford-reiss-nelson-returns-arsenal?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=trans</t>
+        </is>
+      </c>
+    </row>
+    <row r="713">
+      <c r="B713" t="inlineStr">
+        <is>
+          <t>2026-06-25 15:01</t>
+        </is>
+      </c>
+      <c r="C713" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D713" s="2" t="inlineStr">
+        <is>
+          <t>🚨 Pedri: “I love Julián Álvarez. I hope he joins Barcelona, I hope the deal happens”. “He’s among the best players and we want the best at Barça”, told RTVE. 🔵🔴</t>
+        </is>
+      </c>
+      <c r="E713" s="2" t="inlineStr">
+        <is>
+          <t>deal, joins</t>
+        </is>
+      </c>
+      <c r="F713" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2070156156023013806#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="714">
+      <c r="B714" t="inlineStr">
+        <is>
+          <t>2026-06-25 15:01</t>
+        </is>
+      </c>
+      <c r="C714" t="inlineStr">
+        <is>
+          <t>X:@SouthamptonFC</t>
+        </is>
+      </c>
+      <c r="D714" s="2" t="inlineStr">
+        <is>
+          <t>Fixtures: confirmed ✅ Have you added them to your calendar? 📲</t>
+        </is>
+      </c>
+      <c r="E714" s="2" t="inlineStr">
+        <is>
+          <t>confirmed, release</t>
+        </is>
+      </c>
+      <c r="F714" t="inlineStr">
+        <is>
+          <t>https://nitter.net/SouthamptonFC/status/2070153414810501549#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="715">
+      <c r="B715" t="inlineStr">
+        <is>
+          <t>2026-06-25 15:01</t>
+        </is>
+      </c>
+      <c r="C715" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D715" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: aos 59 anos, Kazu Miura vai jogar a 42.ª época da carreira</t>
+        </is>
+      </c>
+      <c r="E715" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F715" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mercado/transferencias/oficial-aos-59-anos-kazu-miura-vai-jogar-a-42-epoca-da-carreira</t>
+        </is>
+      </c>
+    </row>
+    <row r="716">
+      <c r="B716" t="inlineStr">
+        <is>
+          <t>2026-06-25 15:01</t>
+        </is>
+      </c>
+      <c r="C716" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D716" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Benfica confirma saída de Christy Ucheibe</t>
+        </is>
+      </c>
+      <c r="E716" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, confirma, contrato, saída, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F716" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/futebol-feminino/feminino/oficial-benfica-confirma-saida-de-christy-ucheibe</t>
+        </is>
+      </c>
+    </row>
+    <row r="717">
+      <c r="B717" t="inlineStr">
+        <is>
+          <t>2026-06-25 15:01</t>
+        </is>
+      </c>
+      <c r="C717" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D717" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: aos 59 anos, Kazu Miura vai jogar a 42.ª época da carreira</t>
+        </is>
+      </c>
+      <c r="E717" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F717" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/mercado/transferencias/oficial-aos-59-anos-kazu-miura-vai-jogar-a-42-epoca-da-carreira</t>
+        </is>
+      </c>
+    </row>
+    <row r="718">
+      <c r="B718" t="inlineStr">
+        <is>
+          <t>2026-06-25 15:01</t>
+        </is>
+      </c>
+      <c r="C718" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D718" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Sandro Mendes vai treinar em Angola</t>
+        </is>
+      </c>
+      <c r="E718" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F718" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DaAeENSKfqL/?utm_source=ig_embed&amp;utm_campaign=loading</t>
+        </is>
+      </c>
+    </row>
+    <row r="719">
+      <c r="B719" t="inlineStr">
+        <is>
+          <t>2026-06-25 15:01</t>
+        </is>
+      </c>
+      <c r="C719" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D719" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Liverpool · Carter Pinnington — Transfer Out · - West Brom</t>
+        </is>
+      </c>
+      <c r="E719" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F719" t="inlineStr">
+        <is>
+          <t>https://www.liverpoolfc.com/news/carter-pinnington-joins-west-bromwich-albion?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="720">
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>2026-06-25 16:01</t>
+        </is>
+      </c>
+      <c r="C720" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D720" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: ex-Benfica Gilberto troca de clube no Brasileirão</t>
+        </is>
+      </c>
+      <c r="E720" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contrato, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F720" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/internacional/brasil/oficial-ex-benfica-gilberto-troca-de-clube-no-brasileirao</t>
+        </is>
+      </c>
+    </row>
+    <row r="721">
+      <c r="B721" t="inlineStr">
+        <is>
+          <t>2026-06-25 16:01</t>
+        </is>
+      </c>
+      <c r="C721" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D721" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Diogo Sousa deixa o V. Guimarães e reforça o Estrasburgo</t>
+        </is>
+      </c>
+      <c r="E721" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, contrato, deixa, deverá, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F721" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/v-guimaraes/liga/oficial-diogo-sousa-deixa-o-v-guimaraes-e-reforca-o-estrasburgo</t>
+        </is>
+      </c>
+    </row>
+    <row r="722">
+      <c r="B722" t="inlineStr">
+        <is>
+          <t>2026-06-25 16:01</t>
+        </is>
+      </c>
+      <c r="C722" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D722" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Aston Villa · Modou Keba Cisse — Transfer In · - LASK</t>
+        </is>
+      </c>
+      <c r="E722" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F722" t="inlineStr">
+        <is>
+          <t>https://www.avfc.co.uk/news/2025/july/19/villa-announce-cisse-signing/?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="723">
+      <c r="B723" t="inlineStr">
+        <is>
+          <t>2026-06-25 16:01</t>
+        </is>
+      </c>
+      <c r="C723" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D723" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: AFC Bournemouth · Hamed Traore — Transfer Out · - Marseille</t>
+        </is>
+      </c>
+      <c r="E723" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F723" t="inlineStr">
+        <is>
+          <t>https://www.afcb.co.uk/news/2025/august/29/traore-completes-move-to-marseille/?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="724">
+      <c r="B724" t="inlineStr">
+        <is>
+          <t>2026-06-25 16:01</t>
+        </is>
+      </c>
+      <c r="C724" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D724" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Liverpool · Emmanuel Airoboma — Released</t>
+        </is>
+      </c>
+      <c r="E724" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F724" t="inlineStr">
+        <is>
+          <t>https://www.liverpoolfc.com/news/liverpool-confirm-premier-league-retained-list?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="725">
+      <c r="B725" t="inlineStr">
+        <is>
+          <t>2026-06-25 17:01</t>
+        </is>
+      </c>
+      <c r="C725" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D725" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Arsenal contrata Piero Hincapié em definitivo</t>
+        </is>
+      </c>
+      <c r="E725" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F725" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/inglaterra/arsenal/oficial-arsenal-segura-contratacao-de-hincapie-em-definitivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="726">
+      <c r="B726" t="inlineStr">
+        <is>
+          <t>2026-06-25 18:01</t>
+        </is>
+      </c>
+      <c r="C726" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D726" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Ágata Filipa reforça futebol feminino do Sporting</t>
+        </is>
+      </c>
+      <c r="E726" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F726" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/sporting/agata-filipa/oficial-agata-filipa-reforca-futebol-feminino-do-sporting</t>
+        </is>
+      </c>
+    </row>
+    <row r="727">
+      <c r="B727" t="inlineStr">
+        <is>
+          <t>2026-06-25 18:01</t>
+        </is>
+      </c>
+      <c r="C727" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D727" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Arsenal contrata Piero Hincapié em definitivo</t>
+        </is>
+      </c>
+      <c r="E727" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, anunciou, contrato, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F727" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/inglaterra/arsenal/oficial-arsenal-segura-contratacao-de-hincapie-em-definitivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="728">
+      <c r="B728" t="inlineStr">
+        <is>
+          <t>2026-06-25 19:01</t>
+        </is>
+      </c>
+      <c r="C728" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D728" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Sporting reforça equipa B com Catarino Pascoal</t>
+        </is>
+      </c>
+      <c r="E728" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F728" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/sporting/ii-liga/oficial-sporting-reforca-equipa-b-com-catarino-pascoal</t>
+        </is>
+      </c>
+    </row>
+    <row r="729">
+      <c r="B729" t="inlineStr">
+        <is>
+          <t>2026-06-25 19:01</t>
+        </is>
+      </c>
+      <c r="C729" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D729" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Nuno Braga deixa comando técnico do Paços de Ferreira</t>
+        </is>
+      </c>
+      <c r="E729" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F729" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/liga-3/pacos-de-ferreira/oficial-nuno-braga-deixa-comando-tecnico-do-pacos-de-ferreira</t>
+        </is>
+      </c>
+    </row>
+    <row r="730">
+      <c r="B730" t="inlineStr">
+        <is>
+          <t>2026-06-25 19:01</t>
+        </is>
+      </c>
+      <c r="C730" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D730" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Fulham · Quinn Schutter — Released</t>
+        </is>
+      </c>
+      <c r="E730" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F730" t="inlineStr">
+        <is>
+          <t>https://www.fulhamfc.com/news/2026/june/08/player-contract-updates/?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="731">
+      <c r="B731" t="inlineStr">
+        <is>
+          <t>2026-06-25 20:02</t>
+        </is>
+      </c>
+      <c r="C731" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D731" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Sporting reforça equipa B com Catarino Pascoal</t>
+        </is>
+      </c>
+      <c r="E731" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F731" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/sporting/ii-liga/oficial-sporting-reforca-equipa-b-com-catarino-pascoal</t>
+        </is>
+      </c>
+    </row>
+    <row r="732">
+      <c r="B732" t="inlineStr">
+        <is>
+          <t>2026-06-25 20:02</t>
+        </is>
+      </c>
+      <c r="C732" t="inlineStr">
+        <is>
+          <t>maisfutebol RSS</t>
+        </is>
+      </c>
+      <c r="D732" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL: Nuno Braga deixa comando técnico do Paços de Ferreira</t>
+        </is>
+      </c>
+      <c r="E732" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, deixa, OFICIAL:</t>
+        </is>
+      </c>
+      <c r="F732" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/liga-3/pacos-de-ferreira/oficial-nuno-braga-deixa-comando-tecnico-do-pacos-de-ferreira</t>
+        </is>
+      </c>
+    </row>
+    <row r="733">
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>2026-06-25 20:02</t>
+        </is>
+      </c>
+      <c r="C733" t="inlineStr">
+        <is>
+          <t>maisfutebol cronologia</t>
+        </is>
+      </c>
+      <c r="D733" s="2" t="inlineStr">
+        <is>
+          <t>Milan envia proposta oficial por Gonçalo Ramos, dizem em Itália</t>
+        </is>
+      </c>
+      <c r="E733" s="2" t="inlineStr">
+        <is>
+          <t>OFICIAL, transferência</t>
+        </is>
+      </c>
+      <c r="F733" t="inlineStr">
+        <is>
+          <t>https://maisfutebol.iol.pt/cronologia/6373897a0cf2254fb2824fe4#Milan envia proposta oficial por Gonçalo</t>
+        </is>
+      </c>
+    </row>
+    <row r="734">
+      <c r="B734" t="inlineStr">
+        <is>
+          <t>2026-06-25 20:02</t>
+        </is>
+      </c>
+      <c r="C734" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D734" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: AFC Bournemouth · Marcos Senesi — Released</t>
+        </is>
+      </c>
+      <c r="E734" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F734" t="inlineStr">
+        <is>
+          <t>https://www.afcb.co.uk/news/2026/may/15/senesi-to-depart-in-the-summer/?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="735">
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>2026-06-25 20:02</t>
+        </is>
+      </c>
+      <c r="C735" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D735" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Liverpool · Mohamed Salah — Released</t>
+        </is>
+      </c>
+      <c r="E735" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F735" t="inlineStr">
+        <is>
+          <t>https://www.liverpoolfc.com/news/mohamed-salah-leave-liverpool-end-season?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="736">
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>2026-06-25 20:02</t>
+        </is>
+      </c>
+      <c r="C736" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D736" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Newcastle · Max Thompson — Released</t>
+        </is>
+      </c>
+      <c r="E736" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F736" t="inlineStr">
+        <is>
+          <t>https://www.newcastleunited.com/en/news/newcastle-united-confirm-mens-first-team-retained-list?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" t="inlineStr"/>
+      <c r="B737" t="inlineStr">
+        <is>
+          <t>2026-06-25 20:33</t>
+        </is>
+      </c>
+      <c r="C737" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D737" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Everton · Seamus Coleman — Released</t>
+        </is>
+      </c>
+      <c r="E737" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F737" t="inlineStr">
+        <is>
+          <t>https://www.evertonfc.com/news/2026/may/15/Coleman-Calls-Time-On-Everton-Playing-Career/?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" t="inlineStr"/>
+      <c r="B738" t="inlineStr">
+        <is>
+          <t>2026-06-25 20:33</t>
+        </is>
+      </c>
+      <c r="C738" t="inlineStr">
+        <is>
+          <t>PL Official</t>
+        </is>
+      </c>
+      <c r="D738" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL: Newcastle · Matt Targett — Released</t>
+        </is>
+      </c>
+      <c r="E738" s="2" t="inlineStr">
+        <is>
+          <t>OFFICIAL:, release, released, OFFICIAL:</t>
+        </is>
+      </c>
+      <c r="F738" t="inlineStr">
+        <is>
+          <t>https://www.newcastleunited.com/en/news/newcastle-united-confirm-mens-first-team-retained-list?utm_source=premier-league&amp;utm_medium=referral&amp;utm_campaign=pl-referral&amp;utm_term=transfer-watch</t>
         </is>
       </c>
     </row>
@@ -18857,7 +20559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F81"/>
+  <dimension ref="A1:F83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -21118,6 +22820,60 @@
       <c r="F81" t="inlineStr">
         <is>
           <t>https://maisfutebol.iol.pt/cronologia/6373897a0cf2254fb2824fe4#Aston Villa interessado em lateral de Le</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>2026-06-25 16:01</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>🚨🇹🇷 BREAKING: André Onana to Trabzonspor, here we go! 🫱🏻‍🫲🏿 New loan deal verbally agreed as Onana is not part of #MUFC plan for next season and Trabzon are ready to re-sign him. Trabzonspor to pay loan fee to United as details being sorted then done, as @yagosabuncuoglu reports.</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>agreed, deal, loan, HERE WE GO, Here we go!, Here We Go</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2070173917302419525#m</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>2026-06-25 18:01</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>X:@FabrizioRomano</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>🚨 Nathaniel Brown to FC Bayern, here we go! Deal in place with Eintracht Frankfurt for the left back. 🔴⚪️ Never in doubt as Brown agreed terms weeks ago and only wanted Bayern move. Fee will be €55m agreed with Markus Krösche. Five year deal ready for Brown at Bayern, as @Plettigoal reports.</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>agreed, deal, HERE WE GO, Here we go!, Here We Go, here we go</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>https://nitter.net/FabrizioRomano/status/2070200602328461359#m</t>
         </is>
       </c>
     </row>

</xml_diff>